<commit_message>
BOM with Price added.
</commit_message>
<xml_diff>
--- a/Design-Files/WIFI_BoardV4.0/BOM/BOM-With Price-WIFI_BoardV4.00.xlsx
+++ b/Design-Files/WIFI_BoardV4.0/BOM/BOM-With Price-WIFI_BoardV4.00.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="286">
   <si>
     <t>#</t>
   </si>
@@ -315,9 +315,6 @@
     <t>SMD,18x25.5mm WiFi Modules ROHS</t>
   </si>
   <si>
-    <t>SOT-223 Linear Voltage Regulators (LDO) ROHS</t>
-  </si>
-  <si>
     <t>Footprint</t>
   </si>
   <si>
@@ -375,9 +372,6 @@
     <t>41-SMD Module</t>
   </si>
   <si>
-    <t>SOT- 223</t>
-  </si>
-  <si>
     <t>Manufacturer Part Number</t>
   </si>
   <si>
@@ -477,9 +471,6 @@
     <t>ESP32-S3-WROOM-1-N8R2</t>
   </si>
   <si>
-    <t>AMS1117-3.3</t>
-  </si>
-  <si>
     <t>Manufacturer</t>
   </si>
   <si>
@@ -546,9 +537,6 @@
     <t>Espressif Systems</t>
   </si>
   <si>
-    <t>GUOXIN JIAPIN SEMICONDUCTOR</t>
-  </si>
-  <si>
     <t>LCSC Part Number</t>
   </si>
   <si>
@@ -660,9 +648,6 @@
     <t>C2913204</t>
   </si>
   <si>
-    <t>C2992570</t>
-  </si>
-  <si>
     <t>0.01uF</t>
   </si>
   <si>
@@ -870,9 +855,6 @@
     <t>5.4071</t>
   </si>
   <si>
-    <t>0.0348</t>
-  </si>
-  <si>
     <t>Digikey</t>
   </si>
   <si>
@@ -880,6 +862,21 @@
   </si>
   <si>
     <t>C143791</t>
+  </si>
+  <si>
+    <t>55dB@(120Hz) 1A Fixed 3.3V Positive 10V SOT-223-5 Voltage Regulators - Linear, Low Drop Out (LDO) Regulators ROHS</t>
+  </si>
+  <si>
+    <t>SOT-223-5</t>
+  </si>
+  <si>
+    <t>LP38692MPX-3.3/NOPB</t>
+  </si>
+  <si>
+    <t>TI</t>
+  </si>
+  <si>
+    <t>C2866079</t>
   </si>
 </sst>
 </file>
@@ -1233,17 +1230,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1256,18 +1242,29 @@
     <xf numFmtId="164" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1591,14 +1588,14 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17"/>
-      <c r="M1" s="17"/>
-      <c r="N1" s="17"/>
-      <c r="O1" s="17"/>
-      <c r="P1" s="17"/>
-      <c r="Q1" s="17"/>
-      <c r="R1" s="17"/>
+      <c r="K1" s="23"/>
+      <c r="L1" s="23"/>
+      <c r="M1" s="23"/>
+      <c r="N1" s="23"/>
+      <c r="O1" s="23"/>
+      <c r="P1" s="23"/>
+      <c r="Q1" s="23"/>
+      <c r="R1" s="23"/>
     </row>
     <row r="2" spans="1:18" ht="15.75" thickBot="1">
       <c r="A2" s="1"/>
@@ -1615,43 +1612,43 @@
         <v>60</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="I2" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="P2" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="J2" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="K2" s="5" t="s">
+      <c r="Q2" s="5" t="s">
         <v>234</v>
       </c>
-      <c r="L2" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="M2" s="5" t="s">
+      <c r="R2" s="5" t="s">
         <v>235</v>
-      </c>
-      <c r="N2" s="5" t="s">
-        <v>236</v>
-      </c>
-      <c r="O2" s="5" t="s">
-        <v>237</v>
-      </c>
-      <c r="P2" s="5" t="s">
-        <v>238</v>
-      </c>
-      <c r="Q2" s="5" t="s">
-        <v>239</v>
-      </c>
-      <c r="R2" s="5" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -1670,20 +1667,20 @@
         <v>61</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="I3" s="6"/>
       <c r="J3" s="6" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="L3" s="6">
         <v>2</v>
@@ -1692,13 +1689,13 @@
         <f>L3*5</f>
         <v>10</v>
       </c>
-      <c r="N3" s="21">
+      <c r="N3" s="18">
         <v>100</v>
       </c>
-      <c r="O3" s="27" t="s">
-        <v>285</v>
-      </c>
-      <c r="P3" s="23">
+      <c r="O3" s="22" t="s">
+        <v>279</v>
+      </c>
+      <c r="P3" s="20">
         <v>1.1999999999999999E-3</v>
       </c>
       <c r="Q3" s="7">
@@ -1723,20 +1720,20 @@
         <v>62</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="I4" s="12"/>
       <c r="J4" s="12" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="K4" s="12" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="L4" s="12">
         <v>1</v>
@@ -1745,15 +1742,15 @@
         <f t="shared" ref="M4" si="1">L4*5</f>
         <v>5</v>
       </c>
-      <c r="N4" s="20" t="s">
-        <v>245</v>
-      </c>
-      <c r="O4" s="25" t="str">
+      <c r="N4" s="17" t="s">
+        <v>240</v>
+      </c>
+      <c r="O4" s="21" t="str">
         <f>HYPERLINK(M4, "LCSC")</f>
         <v>LCSC</v>
       </c>
-      <c r="P4" s="22" t="s">
-        <v>252</v>
+      <c r="P4" s="19" t="s">
+        <v>247</v>
       </c>
       <c r="Q4" s="13">
         <f t="shared" ref="Q4" si="2">P4*N4</f>
@@ -1777,20 +1774,20 @@
         <v>63</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="I5" s="6"/>
       <c r="J5" s="6" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="L5" s="6">
         <v>1</v>
@@ -1799,15 +1796,15 @@
         <f>L5*5</f>
         <v>5</v>
       </c>
-      <c r="N5" s="21" t="s">
-        <v>246</v>
-      </c>
-      <c r="O5" s="25" t="str">
+      <c r="N5" s="18" t="s">
+        <v>241</v>
+      </c>
+      <c r="O5" s="21" t="str">
         <f t="shared" ref="O5:O41" si="3">HYPERLINK(M5, "LCSC")</f>
         <v>LCSC</v>
       </c>
-      <c r="P5" s="23" t="s">
-        <v>253</v>
+      <c r="P5" s="20" t="s">
+        <v>248</v>
       </c>
       <c r="Q5" s="7">
         <f>P5*N5</f>
@@ -1831,20 +1828,20 @@
         <v>64</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="I6" s="12"/>
       <c r="J6" s="12" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="K6" s="12" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="L6" s="12">
         <v>1</v>
@@ -1853,15 +1850,15 @@
         <f t="shared" ref="M6" si="4">L6*5</f>
         <v>5</v>
       </c>
-      <c r="N6" s="20" t="s">
-        <v>247</v>
-      </c>
-      <c r="O6" s="25" t="str">
+      <c r="N6" s="17" t="s">
+        <v>242</v>
+      </c>
+      <c r="O6" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P6" s="22" t="s">
-        <v>254</v>
+      <c r="P6" s="19" t="s">
+        <v>249</v>
       </c>
       <c r="Q6" s="13">
         <f t="shared" ref="Q6" si="5">P6*N6</f>
@@ -1885,20 +1882,20 @@
         <v>65</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="I7" s="6"/>
       <c r="J7" s="6" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="L7" s="6">
         <v>4</v>
@@ -1907,15 +1904,15 @@
         <f>L7*5</f>
         <v>20</v>
       </c>
-      <c r="N7" s="21" t="s">
-        <v>245</v>
-      </c>
-      <c r="O7" s="25" t="str">
+      <c r="N7" s="18" t="s">
+        <v>240</v>
+      </c>
+      <c r="O7" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P7" s="23" t="s">
-        <v>255</v>
+      <c r="P7" s="20" t="s">
+        <v>250</v>
       </c>
       <c r="Q7" s="7">
         <f>P7*N7</f>
@@ -1939,20 +1936,20 @@
         <v>66</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="I8" s="12"/>
       <c r="J8" s="12" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="K8" s="12" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="L8" s="12">
         <v>1</v>
@@ -1961,14 +1958,14 @@
         <f t="shared" ref="M8" si="6">L8*5</f>
         <v>5</v>
       </c>
-      <c r="N8" s="20">
+      <c r="N8" s="17">
         <v>6</v>
       </c>
-      <c r="O8" s="25" t="s">
-        <v>284</v>
-      </c>
-      <c r="P8" s="22" t="s">
-        <v>256</v>
+      <c r="O8" s="21" t="s">
+        <v>278</v>
+      </c>
+      <c r="P8" s="19" t="s">
+        <v>251</v>
       </c>
       <c r="Q8" s="13">
         <f t="shared" ref="Q8" si="7">P8*N8</f>
@@ -1992,20 +1989,20 @@
         <v>67</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="I9" s="6"/>
       <c r="J9" s="6" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="L9" s="6">
         <v>2</v>
@@ -2014,15 +2011,15 @@
         <f>L9*5</f>
         <v>10</v>
       </c>
-      <c r="N9" s="21" t="s">
-        <v>246</v>
-      </c>
-      <c r="O9" s="25" t="str">
+      <c r="N9" s="18" t="s">
+        <v>241</v>
+      </c>
+      <c r="O9" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P9" s="23" t="s">
-        <v>257</v>
+      <c r="P9" s="20" t="s">
+        <v>252</v>
       </c>
       <c r="Q9" s="7">
         <f>P9*N9</f>
@@ -2046,20 +2043,20 @@
         <v>68</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="I10" s="12"/>
       <c r="J10" s="12" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="K10" s="12" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="L10" s="12">
         <v>1</v>
@@ -2068,15 +2065,15 @@
         <f t="shared" ref="M10" si="8">L10*5</f>
         <v>5</v>
       </c>
-      <c r="N10" s="20" t="s">
-        <v>248</v>
-      </c>
-      <c r="O10" s="25" t="str">
+      <c r="N10" s="17" t="s">
+        <v>243</v>
+      </c>
+      <c r="O10" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P10" s="22" t="s">
-        <v>258</v>
+      <c r="P10" s="19" t="s">
+        <v>253</v>
       </c>
       <c r="Q10" s="13">
         <f t="shared" ref="Q10" si="9">P10*N10</f>
@@ -2100,20 +2097,20 @@
         <v>69</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="I11" s="6"/>
       <c r="J11" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="L11" s="6">
         <v>1</v>
@@ -2122,15 +2119,15 @@
         <f>L11*5</f>
         <v>5</v>
       </c>
-      <c r="N11" s="21" t="s">
-        <v>246</v>
-      </c>
-      <c r="O11" s="25" t="str">
+      <c r="N11" s="18" t="s">
+        <v>241</v>
+      </c>
+      <c r="O11" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P11" s="23" t="s">
-        <v>259</v>
+      <c r="P11" s="20" t="s">
+        <v>254</v>
       </c>
       <c r="Q11" s="7">
         <f>P11*N11</f>
@@ -2154,20 +2151,20 @@
         <v>70</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G12" s="12" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="H12" s="12" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="I12" s="12"/>
       <c r="J12" s="12" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="K12" s="12" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="L12" s="12">
         <v>1</v>
@@ -2176,15 +2173,15 @@
         <f t="shared" ref="M12" si="10">L12*5</f>
         <v>5</v>
       </c>
-      <c r="N12" s="20" t="s">
-        <v>248</v>
-      </c>
-      <c r="O12" s="25" t="str">
+      <c r="N12" s="17" t="s">
+        <v>243</v>
+      </c>
+      <c r="O12" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P12" s="22" t="s">
-        <v>260</v>
+      <c r="P12" s="19" t="s">
+        <v>255</v>
       </c>
       <c r="Q12" s="13">
         <f t="shared" ref="Q12" si="11">P12*N12</f>
@@ -2208,20 +2205,20 @@
         <v>71</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="I13" s="6"/>
       <c r="J13" s="6" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="L13" s="6">
         <v>3</v>
@@ -2230,15 +2227,15 @@
         <f>L13*5</f>
         <v>15</v>
       </c>
-      <c r="N13" s="21" t="s">
-        <v>245</v>
-      </c>
-      <c r="O13" s="25" t="str">
+      <c r="N13" s="18" t="s">
+        <v>240</v>
+      </c>
+      <c r="O13" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P13" s="23" t="s">
-        <v>261</v>
+      <c r="P13" s="20" t="s">
+        <v>256</v>
       </c>
       <c r="Q13" s="7">
         <f>P13*N13</f>
@@ -2262,20 +2259,20 @@
         <v>72</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G14" s="12" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H14" s="12" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="I14" s="12"/>
       <c r="J14" s="12" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="L14" s="12">
         <v>6</v>
@@ -2284,15 +2281,15 @@
         <f t="shared" ref="M14" si="12">L14*5</f>
         <v>30</v>
       </c>
-      <c r="N14" s="20" t="s">
-        <v>249</v>
-      </c>
-      <c r="O14" s="25" t="str">
+      <c r="N14" s="17" t="s">
+        <v>244</v>
+      </c>
+      <c r="O14" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P14" s="22" t="s">
-        <v>262</v>
+      <c r="P14" s="19" t="s">
+        <v>257</v>
       </c>
       <c r="Q14" s="13">
         <f t="shared" ref="Q14" si="13">P14*N14</f>
@@ -2316,20 +2313,20 @@
         <v>73</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I15" s="6"/>
       <c r="J15" s="6" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="L15" s="6">
         <v>1</v>
@@ -2338,15 +2335,15 @@
         <f>L15*5</f>
         <v>5</v>
       </c>
-      <c r="N15" s="21" t="s">
-        <v>247</v>
-      </c>
-      <c r="O15" s="25" t="str">
+      <c r="N15" s="18" t="s">
+        <v>242</v>
+      </c>
+      <c r="O15" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P15" s="23" t="s">
-        <v>263</v>
+      <c r="P15" s="20" t="s">
+        <v>258</v>
       </c>
       <c r="Q15" s="7">
         <f>P15*N15</f>
@@ -2370,20 +2367,20 @@
         <v>74</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="G16" s="12" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="H16" s="12" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="I16" s="12"/>
       <c r="J16" s="12" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="L16" s="12">
         <v>1</v>
@@ -2392,15 +2389,15 @@
         <f t="shared" ref="M16" si="14">L16*5</f>
         <v>5</v>
       </c>
-      <c r="N16" s="20" t="s">
-        <v>250</v>
-      </c>
-      <c r="O16" s="25" t="str">
+      <c r="N16" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="O16" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P16" s="22" t="s">
-        <v>264</v>
+      <c r="P16" s="19" t="s">
+        <v>259</v>
       </c>
       <c r="Q16" s="13">
         <f t="shared" ref="Q16" si="15">P16*N16</f>
@@ -2424,20 +2421,20 @@
         <v>75</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="I17" s="6"/>
       <c r="J17" s="6" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="L17" s="6">
         <v>1</v>
@@ -2446,15 +2443,15 @@
         <f>L17*5</f>
         <v>5</v>
       </c>
-      <c r="N17" s="21" t="s">
-        <v>248</v>
-      </c>
-      <c r="O17" s="25" t="str">
+      <c r="N17" s="18" t="s">
+        <v>243</v>
+      </c>
+      <c r="O17" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P17" s="23" t="s">
-        <v>265</v>
+      <c r="P17" s="20" t="s">
+        <v>260</v>
       </c>
       <c r="Q17" s="7">
         <f>P17*N17</f>
@@ -2478,20 +2475,20 @@
         <v>76</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="G18" s="12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H18" s="12" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="I18" s="12"/>
       <c r="J18" s="12" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="K18" s="6" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="L18" s="12">
         <v>1</v>
@@ -2500,15 +2497,15 @@
         <f t="shared" ref="M18" si="16">L18*5</f>
         <v>5</v>
       </c>
-      <c r="N18" s="20" t="s">
-        <v>248</v>
-      </c>
-      <c r="O18" s="25" t="str">
+      <c r="N18" s="17" t="s">
+        <v>243</v>
+      </c>
+      <c r="O18" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P18" s="22" t="s">
-        <v>266</v>
+      <c r="P18" s="19" t="s">
+        <v>261</v>
       </c>
       <c r="Q18" s="13">
         <f t="shared" ref="Q18" si="17">P18*N18</f>
@@ -2532,20 +2529,20 @@
         <v>77</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="I19" s="6"/>
       <c r="J19" s="6" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="L19" s="6">
         <v>1</v>
@@ -2554,15 +2551,15 @@
         <f>L19*5</f>
         <v>5</v>
       </c>
-      <c r="N19" s="21" t="s">
-        <v>248</v>
-      </c>
-      <c r="O19" s="25" t="str">
+      <c r="N19" s="18" t="s">
+        <v>243</v>
+      </c>
+      <c r="O19" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P19" s="23" t="s">
-        <v>267</v>
+      <c r="P19" s="20" t="s">
+        <v>262</v>
       </c>
       <c r="Q19" s="7">
         <f>P19*N19</f>
@@ -2586,20 +2583,20 @@
         <v>78</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="H20" s="12" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="I20" s="12"/>
       <c r="J20" s="12" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="L20" s="12">
         <v>1</v>
@@ -2608,15 +2605,15 @@
         <f t="shared" ref="M20" si="18">L20*5</f>
         <v>5</v>
       </c>
-      <c r="N20" s="20" t="s">
-        <v>247</v>
-      </c>
-      <c r="O20" s="25" t="str">
+      <c r="N20" s="17" t="s">
+        <v>242</v>
+      </c>
+      <c r="O20" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P20" s="22" t="s">
-        <v>268</v>
+      <c r="P20" s="19" t="s">
+        <v>263</v>
       </c>
       <c r="Q20" s="13">
         <f t="shared" ref="Q20" si="19">P20*N20</f>
@@ -2640,20 +2637,20 @@
         <v>79</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="I21" s="6"/>
       <c r="J21" s="6" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="K21" s="6" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="L21" s="6">
         <v>1</v>
@@ -2662,15 +2659,15 @@
         <f>L21*5</f>
         <v>5</v>
       </c>
-      <c r="N21" s="21" t="s">
-        <v>245</v>
-      </c>
-      <c r="O21" s="25" t="str">
+      <c r="N21" s="18" t="s">
+        <v>240</v>
+      </c>
+      <c r="O21" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P21" s="23" t="s">
-        <v>269</v>
+      <c r="P21" s="20" t="s">
+        <v>264</v>
       </c>
       <c r="Q21" s="7">
         <f>P21*N21</f>
@@ -2694,20 +2691,20 @@
         <v>80</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G22" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="H22" s="12" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="I22" s="12"/>
       <c r="J22" s="12" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="K22" s="6" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="L22" s="12">
         <v>1</v>
@@ -2716,15 +2713,15 @@
         <f t="shared" ref="M22" si="20">L22*5</f>
         <v>5</v>
       </c>
-      <c r="N22" s="20" t="s">
-        <v>249</v>
-      </c>
-      <c r="O22" s="25" t="str">
+      <c r="N22" s="17" t="s">
+        <v>244</v>
+      </c>
+      <c r="O22" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P22" s="22" t="s">
-        <v>270</v>
+      <c r="P22" s="19" t="s">
+        <v>265</v>
       </c>
       <c r="Q22" s="13">
         <f t="shared" ref="Q22" si="21">P22*N22</f>
@@ -2748,20 +2745,20 @@
         <v>81</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="I23" s="6"/>
       <c r="J23" s="6" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="K23" s="6" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="L23" s="6">
         <v>1</v>
@@ -2770,15 +2767,15 @@
         <f>L23*5</f>
         <v>5</v>
       </c>
-      <c r="N23" s="21" t="s">
-        <v>245</v>
-      </c>
-      <c r="O23" s="25" t="str">
+      <c r="N23" s="18" t="s">
+        <v>240</v>
+      </c>
+      <c r="O23" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P23" s="23" t="s">
-        <v>271</v>
+      <c r="P23" s="20" t="s">
+        <v>266</v>
       </c>
       <c r="Q23" s="7">
         <f>P23*N23</f>
@@ -2802,20 +2799,20 @@
         <v>82</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G24" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="H24" s="12" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="I24" s="12"/>
       <c r="J24" s="12" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="K24" s="12" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="L24" s="12">
         <v>5</v>
@@ -2824,15 +2821,15 @@
         <f t="shared" ref="M24" si="22">L24*5</f>
         <v>25</v>
       </c>
-      <c r="N24" s="20" t="s">
-        <v>246</v>
-      </c>
-      <c r="O24" s="25" t="str">
+      <c r="N24" s="17" t="s">
+        <v>241</v>
+      </c>
+      <c r="O24" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P24" s="22" t="s">
-        <v>272</v>
+      <c r="P24" s="19" t="s">
+        <v>267</v>
       </c>
       <c r="Q24" s="13">
         <f t="shared" ref="Q24" si="23">P24*N24</f>
@@ -2856,20 +2853,20 @@
         <v>83</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="H25" s="12" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="I25" s="6"/>
       <c r="J25" s="6" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="K25" s="6" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="L25" s="6">
         <v>3</v>
@@ -2878,15 +2875,15 @@
         <f>L25*5</f>
         <v>15</v>
       </c>
-      <c r="N25" s="21" t="s">
-        <v>245</v>
-      </c>
-      <c r="O25" s="25" t="str">
+      <c r="N25" s="18" t="s">
+        <v>240</v>
+      </c>
+      <c r="O25" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P25" s="23" t="s">
-        <v>273</v>
+      <c r="P25" s="20" t="s">
+        <v>268</v>
       </c>
       <c r="Q25" s="7">
         <f>P25*N25</f>
@@ -2910,20 +2907,20 @@
         <v>84</v>
       </c>
       <c r="F26" s="12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G26" s="12" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="H26" s="12" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="I26" s="12"/>
       <c r="J26" s="12" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="K26" s="12" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="L26" s="12">
         <v>2</v>
@@ -2932,15 +2929,15 @@
         <f t="shared" ref="M26" si="24">L26*5</f>
         <v>10</v>
       </c>
-      <c r="N26" s="20" t="s">
-        <v>246</v>
-      </c>
-      <c r="O26" s="25" t="str">
+      <c r="N26" s="17" t="s">
+        <v>241</v>
+      </c>
+      <c r="O26" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P26" s="22" t="s">
-        <v>274</v>
+      <c r="P26" s="19" t="s">
+        <v>269</v>
       </c>
       <c r="Q26" s="13">
         <f t="shared" ref="Q26" si="25">P26*N26</f>
@@ -2964,20 +2961,20 @@
         <v>85</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="I27" s="6"/>
       <c r="J27" s="6" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="K27" s="6" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="L27" s="6">
         <v>2</v>
@@ -2986,15 +2983,15 @@
         <f>L27*5</f>
         <v>10</v>
       </c>
-      <c r="N27" s="21" t="s">
-        <v>246</v>
-      </c>
-      <c r="O27" s="25" t="str">
+      <c r="N27" s="18" t="s">
+        <v>241</v>
+      </c>
+      <c r="O27" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P27" s="23" t="s">
-        <v>275</v>
+      <c r="P27" s="20" t="s">
+        <v>270</v>
       </c>
       <c r="Q27" s="7">
         <f>P27*N27</f>
@@ -3018,20 +3015,20 @@
         <v>86</v>
       </c>
       <c r="F28" s="12" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G28" s="12" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="H28" s="12" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="I28" s="12"/>
       <c r="J28" s="12" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="K28" s="12" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="L28" s="12">
         <v>4</v>
@@ -3040,15 +3037,15 @@
         <f t="shared" ref="M28" si="26">L28*5</f>
         <v>20</v>
       </c>
-      <c r="N28" s="20" t="s">
-        <v>245</v>
-      </c>
-      <c r="O28" s="25" t="str">
+      <c r="N28" s="17" t="s">
+        <v>240</v>
+      </c>
+      <c r="O28" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P28" s="22" t="s">
-        <v>276</v>
+      <c r="P28" s="19" t="s">
+        <v>271</v>
       </c>
       <c r="Q28" s="13">
         <f t="shared" ref="Q28" si="27">P28*N28</f>
@@ -3072,20 +3069,20 @@
         <v>87</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="I29" s="6"/>
       <c r="J29" s="6" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="K29" s="6" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="L29" s="6">
         <v>1</v>
@@ -3094,15 +3091,15 @@
         <f>L29*5</f>
         <v>5</v>
       </c>
-      <c r="N29" s="21" t="s">
-        <v>246</v>
-      </c>
-      <c r="O29" s="25" t="str">
+      <c r="N29" s="18" t="s">
+        <v>241</v>
+      </c>
+      <c r="O29" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P29" s="23" t="s">
-        <v>275</v>
+      <c r="P29" s="20" t="s">
+        <v>270</v>
       </c>
       <c r="Q29" s="7">
         <f>P29*N29</f>
@@ -3126,20 +3123,20 @@
         <v>88</v>
       </c>
       <c r="F30" s="12" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G30" s="12" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="H30" s="12" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="I30" s="12"/>
       <c r="J30" s="12" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="K30" s="12" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="L30" s="12">
         <v>1</v>
@@ -3148,15 +3145,15 @@
         <f t="shared" ref="M30" si="28">L30*5</f>
         <v>5</v>
       </c>
-      <c r="N30" s="20" t="s">
-        <v>246</v>
-      </c>
-      <c r="O30" s="25" t="str">
+      <c r="N30" s="17" t="s">
+        <v>241</v>
+      </c>
+      <c r="O30" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P30" s="22" t="s">
-        <v>277</v>
+      <c r="P30" s="19" t="s">
+        <v>272</v>
       </c>
       <c r="Q30" s="13">
         <f t="shared" ref="Q30" si="29">P30*N30</f>
@@ -3180,20 +3177,20 @@
         <v>89</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="I31" s="6"/>
       <c r="J31" s="6" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="K31" s="6" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="L31" s="6">
         <v>1</v>
@@ -3202,15 +3199,15 @@
         <f>L31*5</f>
         <v>5</v>
       </c>
-      <c r="N31" s="21" t="s">
-        <v>246</v>
-      </c>
-      <c r="O31" s="25" t="str">
+      <c r="N31" s="18" t="s">
+        <v>241</v>
+      </c>
+      <c r="O31" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P31" s="23" t="s">
-        <v>272</v>
+      <c r="P31" s="20" t="s">
+        <v>267</v>
       </c>
       <c r="Q31" s="7">
         <f>P31*N31</f>
@@ -3234,20 +3231,20 @@
         <v>90</v>
       </c>
       <c r="F32" s="12" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G32" s="12" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="H32" s="12" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="I32" s="12"/>
       <c r="J32" s="12" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="K32" s="12" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="L32" s="12">
         <v>1</v>
@@ -3256,15 +3253,15 @@
         <f t="shared" ref="M32" si="30">L32*5</f>
         <v>5</v>
       </c>
-      <c r="N32" s="20" t="s">
-        <v>246</v>
-      </c>
-      <c r="O32" s="25" t="str">
+      <c r="N32" s="17" t="s">
+        <v>241</v>
+      </c>
+      <c r="O32" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P32" s="22" t="s">
-        <v>272</v>
+      <c r="P32" s="19" t="s">
+        <v>267</v>
       </c>
       <c r="Q32" s="13">
         <f t="shared" ref="Q32" si="31">P32*N32</f>
@@ -3288,20 +3285,20 @@
         <v>91</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="I33" s="6"/>
       <c r="J33" s="6" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="K33" s="6" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="L33" s="6">
         <v>1</v>
@@ -3310,15 +3307,15 @@
         <f>L33*5</f>
         <v>5</v>
       </c>
-      <c r="N33" s="21" t="s">
-        <v>246</v>
-      </c>
-      <c r="O33" s="25" t="str">
+      <c r="N33" s="18" t="s">
+        <v>241</v>
+      </c>
+      <c r="O33" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P33" s="23" t="s">
-        <v>277</v>
+      <c r="P33" s="20" t="s">
+        <v>272</v>
       </c>
       <c r="Q33" s="7">
         <f>P33*N33</f>
@@ -3342,20 +3339,20 @@
         <v>92</v>
       </c>
       <c r="F34" s="12" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G34" s="12" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H34" s="12" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="I34" s="12"/>
       <c r="J34" s="12" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="K34" s="12" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="L34" s="12">
         <v>2</v>
@@ -3364,15 +3361,15 @@
         <f t="shared" ref="M34" si="32">L34*5</f>
         <v>10</v>
       </c>
-      <c r="N34" s="20" t="s">
-        <v>246</v>
-      </c>
-      <c r="O34" s="25" t="str">
+      <c r="N34" s="17" t="s">
+        <v>241</v>
+      </c>
+      <c r="O34" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P34" s="22" t="s">
-        <v>277</v>
+      <c r="P34" s="19" t="s">
+        <v>272</v>
       </c>
       <c r="Q34" s="13">
         <f t="shared" ref="Q34" si="33">P34*N34</f>
@@ -3396,20 +3393,20 @@
         <v>93</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="I35" s="6"/>
       <c r="J35" s="6" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="K35" s="6" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="L35" s="6">
         <v>1</v>
@@ -3418,15 +3415,15 @@
         <f>L35*5</f>
         <v>5</v>
       </c>
-      <c r="N35" s="21" t="s">
-        <v>246</v>
-      </c>
-      <c r="O35" s="25" t="str">
+      <c r="N35" s="18" t="s">
+        <v>241</v>
+      </c>
+      <c r="O35" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P35" s="23" t="s">
-        <v>275</v>
+      <c r="P35" s="20" t="s">
+        <v>270</v>
       </c>
       <c r="Q35" s="7">
         <f>P35*N35</f>
@@ -3450,20 +3447,20 @@
         <v>94</v>
       </c>
       <c r="F36" s="12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G36" s="12" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="H36" s="12" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="I36" s="12"/>
       <c r="J36" s="12" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="K36" s="12" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="L36" s="12">
         <v>1</v>
@@ -3472,15 +3469,15 @@
         <f t="shared" ref="M36" si="34">L36*5</f>
         <v>5</v>
       </c>
-      <c r="N36" s="20" t="s">
-        <v>246</v>
-      </c>
-      <c r="O36" s="25" t="str">
+      <c r="N36" s="17" t="s">
+        <v>241</v>
+      </c>
+      <c r="O36" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P36" s="22" t="s">
-        <v>278</v>
+      <c r="P36" s="19" t="s">
+        <v>273</v>
       </c>
       <c r="Q36" s="13">
         <f t="shared" ref="Q36" si="35">P36*N36</f>
@@ -3504,20 +3501,20 @@
         <v>95</v>
       </c>
       <c r="F37" s="12" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="I37" s="6"/>
       <c r="J37" s="6" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="K37" s="6" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="L37" s="6">
         <v>2</v>
@@ -3526,15 +3523,15 @@
         <f>L37*5</f>
         <v>10</v>
       </c>
-      <c r="N37" s="21" t="s">
-        <v>247</v>
-      </c>
-      <c r="O37" s="25" t="str">
+      <c r="N37" s="18" t="s">
+        <v>242</v>
+      </c>
+      <c r="O37" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P37" s="23" t="s">
-        <v>279</v>
+      <c r="P37" s="20" t="s">
+        <v>274</v>
       </c>
       <c r="Q37" s="7">
         <f>P37*N37</f>
@@ -3558,20 +3555,20 @@
         <v>96</v>
       </c>
       <c r="F38" s="12" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="G38" s="12" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H38" s="12" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="I38" s="12"/>
       <c r="J38" s="6" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="K38" s="6" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="L38" s="12">
         <v>1</v>
@@ -3580,15 +3577,15 @@
         <f t="shared" ref="M38" si="36">L38*5</f>
         <v>5</v>
       </c>
-      <c r="N38" s="20" t="s">
-        <v>248</v>
-      </c>
-      <c r="O38" s="25" t="str">
+      <c r="N38" s="17" t="s">
+        <v>243</v>
+      </c>
+      <c r="O38" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P38" s="22" t="s">
-        <v>280</v>
+      <c r="P38" s="19" t="s">
+        <v>275</v>
       </c>
       <c r="Q38" s="13">
         <f t="shared" ref="Q38" si="37">P38*N38</f>
@@ -3612,20 +3609,20 @@
         <v>95</v>
       </c>
       <c r="F39" s="12" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="I39" s="6"/>
       <c r="J39" s="6" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="K39" s="6" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="L39" s="6">
         <v>3</v>
@@ -3634,15 +3631,15 @@
         <f>L39*5</f>
         <v>15</v>
       </c>
-      <c r="N39" s="21" t="s">
-        <v>251</v>
-      </c>
-      <c r="O39" s="25" t="str">
+      <c r="N39" s="18" t="s">
+        <v>246</v>
+      </c>
+      <c r="O39" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P39" s="23" t="s">
-        <v>281</v>
+      <c r="P39" s="20" t="s">
+        <v>276</v>
       </c>
       <c r="Q39" s="7">
         <f>P39*N39</f>
@@ -3666,20 +3663,20 @@
         <v>97</v>
       </c>
       <c r="F40" s="12" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G40" s="12" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="H40" s="12" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="I40" s="12"/>
       <c r="J40" s="12" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="K40" s="6" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="L40" s="12">
         <v>1</v>
@@ -3688,15 +3685,15 @@
         <f t="shared" ref="M40" si="38">L40*5</f>
         <v>5</v>
       </c>
-      <c r="N40" s="20" t="s">
-        <v>248</v>
-      </c>
-      <c r="O40" s="25" t="str">
+      <c r="N40" s="17" t="s">
+        <v>243</v>
+      </c>
+      <c r="O40" s="21" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P40" s="22" t="s">
-        <v>282</v>
+      <c r="P40" s="19" t="s">
+        <v>277</v>
       </c>
       <c r="Q40" s="13">
         <f t="shared" ref="Q40" si="39">P40*N40</f>
@@ -3704,7 +3701,7 @@
       </c>
       <c r="R40" s="12"/>
     </row>
-    <row r="41" spans="1:18" ht="24.75" thickBot="1">
+    <row r="41" spans="1:18" ht="48.75" thickBot="1">
       <c r="A41" s="1"/>
       <c r="B41" s="8">
         <f>ROW(B41) - ROW($B$2)</f>
@@ -3717,23 +3714,23 @@
         <v>59</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>98</v>
+        <v>281</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>118</v>
+        <v>282</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>152</v>
+        <v>283</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>175</v>
+        <v>284</v>
       </c>
       <c r="I41" s="6"/>
       <c r="J41" s="6" t="s">
-        <v>213</v>
+        <v>285</v>
       </c>
       <c r="K41" s="6" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="L41" s="6">
         <v>1</v>
@@ -3742,19 +3739,18 @@
         <f>L41*5</f>
         <v>5</v>
       </c>
-      <c r="N41" s="21" t="s">
-        <v>245</v>
-      </c>
-      <c r="O41" s="26" t="str">
-        <f t="shared" si="3"/>
-        <v>LCSC</v>
-      </c>
-      <c r="P41" s="23" t="s">
-        <v>283</v>
+      <c r="N41" s="18">
+        <v>6</v>
+      </c>
+      <c r="O41" s="27" t="s">
+        <v>279</v>
+      </c>
+      <c r="P41" s="20">
+        <v>1.5250999999999999</v>
       </c>
       <c r="Q41" s="7">
         <f>P41*N41</f>
-        <v>0.69599999999999995</v>
+        <v>9.150599999999999</v>
       </c>
       <c r="R41" s="6"/>
     </row>
@@ -3772,14 +3768,14 @@
       <c r="K42" s="1"/>
       <c r="L42" s="1"/>
       <c r="M42" s="1"/>
-      <c r="N42" s="18" t="s">
+      <c r="N42" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="O42" s="24"/>
-      <c r="P42" s="19"/>
+      <c r="O42" s="25"/>
+      <c r="P42" s="26"/>
       <c r="Q42" s="10">
         <f>SUM(Q3:Q41)</f>
-        <v>75.220100000000002</v>
+        <v>83.674700000000001</v>
       </c>
       <c r="R42" s="1"/>
     </row>
@@ -3797,14 +3793,14 @@
       <c r="K43" s="1"/>
       <c r="L43" s="1"/>
       <c r="M43" s="1"/>
-      <c r="N43" s="18" t="s">
+      <c r="N43" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="O43" s="19"/>
-      <c r="P43" s="19"/>
+      <c r="O43" s="26"/>
+      <c r="P43" s="26"/>
       <c r="Q43" s="11">
         <f>Q42/5</f>
-        <v>15.04402</v>
+        <v>16.734940000000002</v>
       </c>
       <c r="R43" s="1"/>
     </row>
@@ -3820,8 +3816,10 @@
   <hyperlinks>
     <hyperlink ref="O8" r:id="rId1"/>
     <hyperlink ref="O3" r:id="rId2"/>
+    <hyperlink ref="E41" r:id="rId3"/>
+    <hyperlink ref="O41" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
WIFI Board BOM added With Price
</commit_message>
<xml_diff>
--- a/Design-Files/WIFI_BoardV4.0/BOM/BOM-With Price-WIFI_BoardV4.00.xlsx
+++ b/Design-Files/WIFI_BoardV4.0/BOM/BOM-With Price-WIFI_BoardV4.00.xlsx
@@ -5,21 +5,21 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\OliverStanton-WaterMonitor\Design-Files\WIFI_BoardV4.0\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iftikhar Ahmed\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="338">
   <si>
     <t>#</t>
   </si>
@@ -36,15 +36,12 @@
     <t>Capacitor</t>
   </si>
   <si>
-    <t>Capacitors</t>
+    <t>Diode</t>
   </si>
   <si>
     <t>Protection Device</t>
   </si>
   <si>
-    <t>Diode</t>
-  </si>
-  <si>
     <t>Connector</t>
   </si>
   <si>
@@ -57,9 +54,21 @@
     <t>Wire To Board Connector</t>
   </si>
   <si>
+    <t>Photo Sensor</t>
+  </si>
+  <si>
+    <t>Buzzer</t>
+  </si>
+  <si>
+    <t>Test Point</t>
+  </si>
+  <si>
     <t>Mosfet</t>
   </si>
   <si>
+    <t>Transister</t>
+  </si>
+  <si>
     <t>Resistor</t>
   </si>
   <si>
@@ -78,9 +87,15 @@
     <t>Module</t>
   </si>
   <si>
+    <t>Sensor</t>
+  </si>
+  <si>
     <t>IC</t>
   </si>
   <si>
+    <t>(TVS/ESD)</t>
+  </si>
+  <si>
     <t>Designator</t>
   </si>
   <si>
@@ -90,13 +105,13 @@
     <t>C2</t>
   </si>
   <si>
-    <t>C3</t>
+    <t>C3, C12, C13, C14</t>
   </si>
   <si>
     <t>C4</t>
   </si>
   <si>
-    <t>C5, C12, C13, C14</t>
+    <t>C5</t>
   </si>
   <si>
     <t>C7</t>
@@ -114,7 +129,16 @@
     <t>C15</t>
   </si>
   <si>
-    <t>D1, D2, D3</t>
+    <t>C16</t>
+  </si>
+  <si>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>D2</t>
+  </si>
+  <si>
+    <t>D3</t>
   </si>
   <si>
     <t>D4, D5, D6, D7, D8, D9</t>
@@ -135,19 +159,25 @@
     <t>J4</t>
   </si>
   <si>
+    <t>LED1</t>
+  </si>
+  <si>
+    <t>LS1</t>
+  </si>
+  <si>
+    <t>P1, P2, P3, P4, P5</t>
+  </si>
+  <si>
     <t>Q1</t>
   </si>
   <si>
-    <t>Q2</t>
-  </si>
-  <si>
-    <t>Q3</t>
-  </si>
-  <si>
-    <t>Q4</t>
-  </si>
-  <si>
-    <t>R1, R19, R20, R21, R22</t>
+    <t>Q2, Q3</t>
+  </si>
+  <si>
+    <t>Q5</t>
+  </si>
+  <si>
+    <t>R1, R19, R20, R21</t>
   </si>
   <si>
     <t>R2, R3, R12</t>
@@ -171,21 +201,27 @@
     <t>R14</t>
   </si>
   <si>
-    <t>R15</t>
-  </si>
-  <si>
-    <t>R16</t>
+    <t>R15, R16</t>
   </si>
   <si>
     <t>R17, R18</t>
   </si>
   <si>
+    <t>R22, R29</t>
+  </si>
+  <si>
     <t>R23</t>
   </si>
   <si>
     <t>R24</t>
   </si>
   <si>
+    <t>R26, R28</t>
+  </si>
+  <si>
+    <t>R27</t>
+  </si>
+  <si>
     <t>SW1, SW2</t>
   </si>
   <si>
@@ -201,13 +237,19 @@
     <t>U2</t>
   </si>
   <si>
+    <t>U3</t>
+  </si>
+  <si>
+    <t>U4</t>
+  </si>
+  <si>
     <t>Description</t>
   </si>
   <si>
     <t>CAP CER 10000PF 25V X5R 0402</t>
   </si>
   <si>
-    <t>47uF 50V 66mA@120Hz ±20% SMD,D6.3xL7.7mm Aluminum Electrolytic Capacitors - SMD ROHS</t>
+    <t>CAP TANT 47UF 10% 25V 2917</t>
   </si>
   <si>
     <t>CAP CER 0.1UF 25V X5R 0402</t>
@@ -225,7 +267,7 @@
     <t>CAP CER 0.1UF 16V X7R 0402</t>
   </si>
   <si>
-    <t>CAP TANT 10UF 20% 10V 0603</t>
+    <t>CAP TANT 10UF 10% 16V 1206</t>
   </si>
   <si>
     <t>CAP CER 0.1UF 50V X5R 0603</t>
@@ -234,9 +276,18 @@
     <t>CAP CER 0.1UF 50V X5R 0402</t>
   </si>
   <si>
+    <t>CAP CER 0.1UF 50V Y5V 0603</t>
+  </si>
+  <si>
     <t>40V 500mV@2A 2A SMA(DO-214AC) Schottky Barrier Diodes (SBD) ROHS</t>
   </si>
   <si>
+    <t>DIODE ZENER 6.2V 500MW SOD123</t>
+  </si>
+  <si>
+    <t>DIODE GEN PURP 100V 300MA SOD123</t>
+  </si>
+  <si>
     <t>5V 10V 3.3V Bi-Directional SOD-882 ESD Protection Devices ROHS</t>
   </si>
   <si>
@@ -255,16 +306,22 @@
     <t>1x12P 12P PicoBlade(MX 1.25) Tin 12 -25℃~+85℃ 2A 1 1.25mm Brass Surface Mount,Vertical SMD,P=1.25mm Wire To Board Connector ROHS</t>
   </si>
   <si>
+    <t>SENSOR PHOTO 630NM 2SMD</t>
+  </si>
+  <si>
+    <t>Externally Driven 85dB@3V,10cm 3V 2700Hz SMD,D=9mm Buzzers ROHS</t>
+  </si>
+  <si>
+    <t>Test Point ON</t>
+  </si>
+  <si>
     <t>30V 5.8A 32mΩ@10V,5.8A 1.4W 1.4V@250uA N Channel SOT-23 MOSFETs ROHS</t>
   </si>
   <si>
-    <t>30V 4.1A 60mΩ@10V,4.1A 350mW 3V@250uA P Channel SOT-23 MOSFETs ROHS</t>
-  </si>
-  <si>
     <t>50V 220mA 3.5Ω@10V,220mA 225mW 1.6V@1mA N Channel SOT-23 MOSFETs ROHS</t>
   </si>
   <si>
-    <t>TRANS NPN 40V 0.6A SMD SOT23-3</t>
+    <t>TRANS NPN 160V 0.6A SOT-23</t>
   </si>
   <si>
     <t>RES 10K OHM 1% 1/16W 0402</t>
@@ -294,18 +351,24 @@
     <t>RES 1K OHM 5% 1/16W 0402</t>
   </si>
   <si>
-    <t>RES 4.7K OHM 1% 1/16W 0402</t>
-  </si>
-  <si>
     <t>RES 47K OHM 1% 1/16W 0402</t>
   </si>
   <si>
+    <t>RES 100K OHM 1% 1/10W 0603</t>
+  </si>
+  <si>
     <t>RES 15K OHM 1% 1/10W 0603</t>
   </si>
   <si>
     <t>RES 3.3K OHM 0.5% 1/10W 0603</t>
   </si>
   <si>
+    <t>RES SMD 4.7K OHM 1% 1/10W 0603</t>
+  </si>
+  <si>
+    <t>RES 20K OHM 1% 1/10W 0603</t>
+  </si>
+  <si>
     <t>SWITCH TACTILE SPST-NO 0.05A 12V</t>
   </si>
   <si>
@@ -315,13 +378,22 @@
     <t>SMD,18x25.5mm WiFi Modules ROHS</t>
   </si>
   <si>
+    <t>Plugin Human Body Sensing Sensor ROHS</t>
+  </si>
+  <si>
+    <t>IC REG LINEAR 3.3V 1A 8DFN</t>
+  </si>
+  <si>
+    <t>6A 12V 150W 6V Unidirectional 5V SOT-23-6 ESD and Surge Protection (TVS/ESD) ROHS</t>
+  </si>
+  <si>
     <t>Footprint</t>
   </si>
   <si>
     <t>Cap-0402</t>
   </si>
   <si>
-    <t>RVT1H470M0607</t>
+    <t>Case-D</t>
   </si>
   <si>
     <t>Cap-0603</t>
@@ -330,33 +402,51 @@
     <t>Tant-0805</t>
   </si>
   <si>
-    <t>Tant-0603</t>
+    <t>Case-A</t>
   </si>
   <si>
     <t>SMA</t>
   </si>
   <si>
+    <t>SOD-123</t>
+  </si>
+  <si>
     <t>SOD-882 Bi Directional</t>
   </si>
   <si>
     <t>SOD323F</t>
   </si>
   <si>
+    <t>Voltlink Target</t>
+  </si>
+  <si>
+    <t>TYPE-C-31-M-12_</t>
+  </si>
+  <si>
     <t>F0502-B-18-15T-R</t>
   </si>
   <si>
     <t>HC-1.25-12PLT</t>
   </si>
   <si>
+    <t>ALS-PT19-315C/L177/TR_</t>
+  </si>
+  <si>
+    <t>YS-SBZ9032C03R16_</t>
+  </si>
+  <si>
+    <t>Test-point - 0.5mm</t>
+  </si>
+  <si>
     <t>sot-23</t>
   </si>
   <si>
+    <t>Sot-23</t>
+  </si>
+  <si>
     <t>SOT-23</t>
   </si>
   <si>
-    <t>Sot-23</t>
-  </si>
-  <si>
     <t>Res-0402</t>
   </si>
   <si>
@@ -369,15 +459,30 @@
     <t>PEC11R-4215F-N0024</t>
   </si>
   <si>
+    <t>TL3300CF160Q.</t>
+  </si>
+  <si>
     <t>41-SMD Module</t>
   </si>
   <si>
+    <t>AS312</t>
+  </si>
+  <si>
+    <t>DFN-8(1.2x1.6)</t>
+  </si>
+  <si>
+    <t>SOT-23-6</t>
+  </si>
+  <si>
     <t>Manufacturer Part Number</t>
   </si>
   <si>
     <t>CC0402KRX5R8BB103</t>
   </si>
   <si>
+    <t>T495D476K025ATE250</t>
+  </si>
+  <si>
     <t>CC0402KRX5R8BB104</t>
   </si>
   <si>
@@ -393,7 +498,7 @@
     <t>CC0402JRX7R7BB104</t>
   </si>
   <si>
-    <t>TR8M106M010C2000</t>
+    <t>T491A106K016AT</t>
   </si>
   <si>
     <t>CC0603KRX5R9BB104</t>
@@ -402,9 +507,18 @@
     <t>C1005X5R1H104K050BB</t>
   </si>
   <si>
+    <t>CC0603ZRY5V9BB104</t>
+  </si>
+  <si>
     <t>SS24A</t>
   </si>
   <si>
+    <t>MMSZ5234B-7-F</t>
+  </si>
+  <si>
+    <t>1N4148W-7-F</t>
+  </si>
+  <si>
     <t>LESD8D3.3CAT5G</t>
   </si>
   <si>
@@ -417,16 +531,19 @@
     <t>TYPE-C-31-M-12</t>
   </si>
   <si>
+    <t>ALS-PT19-315C/L177/TR8</t>
+  </si>
+  <si>
+    <t>YS-SBZ9032C03R16</t>
+  </si>
+  <si>
     <t>AO3400A</t>
   </si>
   <si>
-    <t>AO3407</t>
-  </si>
-  <si>
     <t>BSS138</t>
   </si>
   <si>
-    <t>MMBT2222A-7-F</t>
+    <t>MMBT5551LT1G</t>
   </si>
   <si>
     <t>RC0402FR-0710KL</t>
@@ -453,31 +570,43 @@
     <t>RC0402JR-071KL</t>
   </si>
   <si>
-    <t>RC0402FR-074K7L</t>
-  </si>
-  <si>
     <t>RC0402FR-0747KL</t>
   </si>
   <si>
+    <t>RC0603FR-07100KL</t>
+  </si>
+  <si>
     <t>RC0603FR-0715KL</t>
   </si>
   <si>
     <t>RC0603DR-073K3L</t>
   </si>
   <si>
+    <t>RC0603FR-074K7L</t>
+  </si>
+  <si>
+    <t>RC0603FR-0720KL</t>
+  </si>
+  <si>
     <t>TL3300CF160Q</t>
   </si>
   <si>
     <t>ESP32-S3-WROOM-1-N8R2</t>
   </si>
   <si>
+    <t>LD56100DPU33R</t>
+  </si>
+  <si>
+    <t>USBLC6-2SC6</t>
+  </si>
+  <si>
     <t>Manufacturer</t>
   </si>
   <si>
     <t>Yageo</t>
   </si>
   <si>
-    <t>ROQANG</t>
+    <t>KEMET</t>
   </si>
   <si>
     <t>Murata</t>
@@ -486,15 +615,15 @@
     <t>Rohm</t>
   </si>
   <si>
-    <t>Vishay Sprague</t>
-  </si>
-  <si>
     <t>TDK</t>
   </si>
   <si>
     <t>Guangdong Hottech</t>
   </si>
   <si>
+    <t>Diodes</t>
+  </si>
+  <si>
     <t>LRC</t>
   </si>
   <si>
@@ -513,13 +642,19 @@
     <t>HCTL</t>
   </si>
   <si>
+    <t>Everlight</t>
+  </si>
+  <si>
+    <t>Fengming</t>
+  </si>
+  <si>
     <t>BORN</t>
   </si>
   <si>
     <t>Slkor(SLKORMICRO Elec.)</t>
   </si>
   <si>
-    <t>Diodes</t>
+    <t>ON Semiconductor</t>
   </si>
   <si>
     <t>Vishay Dale</t>
@@ -537,13 +672,22 @@
     <t>Espressif Systems</t>
   </si>
   <si>
+    <t>Senba Sensing Tech</t>
+  </si>
+  <si>
+    <t>STMicroelectronics</t>
+  </si>
+  <si>
+    <t>TECH PUBLIC</t>
+  </si>
+  <si>
     <t>LCSC Part Number</t>
   </si>
   <si>
     <t>C576726</t>
   </si>
   <si>
-    <t>C72523</t>
+    <t>C1952924</t>
   </si>
   <si>
     <t>C106256</t>
@@ -561,7 +705,7 @@
     <t>C541464</t>
   </si>
   <si>
-    <t>C1952781</t>
+    <t>C110055</t>
   </si>
   <si>
     <t>C110022</t>
@@ -570,9 +714,15 @@
     <t>C2181865</t>
   </si>
   <si>
+    <t>C106221</t>
+  </si>
+  <si>
     <t>C2886579</t>
   </si>
   <si>
+    <t>C83528</t>
+  </si>
+  <si>
     <t>C172409</t>
   </si>
   <si>
@@ -588,16 +738,19 @@
     <t>C2937190</t>
   </si>
   <si>
+    <t>C146233</t>
+  </si>
+  <si>
+    <t>C409828</t>
+  </si>
+  <si>
     <t>C344010</t>
   </si>
   <si>
-    <t>C181093</t>
-  </si>
-  <si>
     <t>C426569</t>
   </si>
   <si>
-    <t>C94515</t>
+    <t>C909756</t>
   </si>
   <si>
     <t>C60490</t>
@@ -627,18 +780,24 @@
     <t>C105637</t>
   </si>
   <si>
-    <t>C105871</t>
-  </si>
-  <si>
     <t>C93943</t>
   </si>
   <si>
+    <t>C14675</t>
+  </si>
+  <si>
     <t>C114661</t>
   </si>
   <si>
     <t>C723574</t>
   </si>
   <si>
+    <t>C99782</t>
+  </si>
+  <si>
+    <t>C105575</t>
+  </si>
+  <si>
     <t>C231329</t>
   </si>
   <si>
@@ -648,6 +807,15 @@
     <t>C2913204</t>
   </si>
   <si>
+    <t>C90465</t>
+  </si>
+  <si>
+    <t>C2969937</t>
+  </si>
+  <si>
+    <t>C2827654</t>
+  </si>
+  <si>
     <t>0.01uF</t>
   </si>
   <si>
@@ -690,16 +858,22 @@
     <t>1K</t>
   </si>
   <si>
+    <t>47K</t>
+  </si>
+  <si>
+    <t>100K</t>
+  </si>
+  <si>
+    <t>15K</t>
+  </si>
+  <si>
+    <t>3.3K</t>
+  </si>
+  <si>
     <t>4.7K</t>
   </si>
   <si>
-    <t>47K</t>
-  </si>
-  <si>
-    <t>15K</t>
-  </si>
-  <si>
-    <t>3.3K</t>
+    <t>20K</t>
   </si>
   <si>
     <t>Quantity</t>
@@ -729,154 +903,136 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>Custom</t>
+    <t>LCSC</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t>0.0020</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>0.0393</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>0.0332</t>
+  </si>
+  <si>
+    <t>Digikey</t>
+  </si>
+  <si>
+    <t>0.1317</t>
+  </si>
+  <si>
+    <t>0.0018</t>
+  </si>
+  <si>
+    <t>0.0034</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>0.0985</t>
+  </si>
+  <si>
+    <t>0.1738</t>
+  </si>
+  <si>
+    <t>0.0391</t>
+  </si>
+  <si>
+    <t>0.1706</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>0.0088</t>
+  </si>
+  <si>
+    <t>0.0448</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>0.0717</t>
+  </si>
+  <si>
+    <t>0.0210</t>
+  </si>
+  <si>
+    <t>0.1555</t>
+  </si>
+  <si>
+    <t>1.3376</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>0.6953</t>
+  </si>
+  <si>
+    <t>5.4071</t>
+  </si>
+  <si>
+    <t>0.0006</t>
+  </si>
+  <si>
+    <t>0.0287</t>
+  </si>
+  <si>
+    <t>0.0011</t>
+  </si>
+  <si>
+    <t>0.0012</t>
+  </si>
+  <si>
+    <t>0.0185</t>
+  </si>
+  <si>
+    <t>0.0007</t>
+  </si>
+  <si>
+    <t>0.0053</t>
+  </si>
+  <si>
+    <t>0.0517</t>
+  </si>
+  <si>
+    <t>DO NOT PLACE</t>
   </si>
   <si>
     <t>-</t>
   </si>
   <si>
-    <t>RK73G1JTTD1002F</t>
-  </si>
-  <si>
-    <t>KOA Speer Elec</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>100</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>50</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>0.0265</t>
-  </si>
-  <si>
-    <t>0.0020</t>
-  </si>
-  <si>
-    <t>0.0393</t>
-  </si>
-  <si>
-    <t>0.0332</t>
-  </si>
-  <si>
-    <t>0.1317</t>
-  </si>
-  <si>
-    <t>0.0018</t>
-  </si>
-  <si>
-    <t>3.2443</t>
-  </si>
-  <si>
-    <t>0.0034</t>
-  </si>
-  <si>
-    <t>0.0985</t>
-  </si>
-  <si>
-    <t>0.0210</t>
-  </si>
-  <si>
-    <t>0.0088</t>
-  </si>
-  <si>
-    <t>0.0448</t>
-  </si>
-  <si>
-    <t>0.0717</t>
-  </si>
-  <si>
-    <t>0.1738</t>
-  </si>
-  <si>
-    <t>0.0391</t>
-  </si>
-  <si>
-    <t>0.1706</t>
-  </si>
-  <si>
-    <t>0.0517</t>
-  </si>
-  <si>
-    <t>0.0274</t>
-  </si>
-  <si>
-    <t>0.0170</t>
-  </si>
-  <si>
-    <t>0.0275</t>
-  </si>
-  <si>
-    <t>0.0006</t>
-  </si>
-  <si>
-    <t>0.0287</t>
-  </si>
-  <si>
-    <t>0.0011</t>
-  </si>
-  <si>
-    <t>0.0012</t>
-  </si>
-  <si>
-    <t>0.0185</t>
-  </si>
-  <si>
-    <t>0.0007</t>
-  </si>
-  <si>
-    <t>0.0053</t>
-  </si>
-  <si>
-    <t>0.1555</t>
-  </si>
-  <si>
-    <t>1.3376</t>
-  </si>
-  <si>
-    <t>0.6953</t>
-  </si>
-  <si>
-    <t>5.4071</t>
-  </si>
-  <si>
-    <t>Digikey</t>
-  </si>
-  <si>
-    <t>LCSC</t>
+    <t>C151818</t>
   </si>
   <si>
     <t>C143791</t>
   </si>
   <si>
-    <t>55dB@(120Hz) 1A Fixed 3.3V Positive 10V SOT-223-5 Voltage Regulators - Linear, Low Drop Out (LDO) Regulators ROHS</t>
-  </si>
-  <si>
-    <t>SOT-223-5</t>
-  </si>
-  <si>
-    <t>LP38692MPX-3.3/NOPB</t>
-  </si>
-  <si>
-    <t>TI</t>
-  </si>
-  <si>
-    <t>C2866079</t>
+    <t>HT240S030</t>
+  </si>
+  <si>
+    <t>Peripheral</t>
+  </si>
+  <si>
+    <t>LCD</t>
+  </si>
+  <si>
+    <t>Quotation Required From Custom Supplier</t>
+  </si>
+  <si>
+    <t>Eya Display</t>
   </si>
 </sst>
 </file>
@@ -887,7 +1043,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -968,6 +1124,31 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <strike/>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <strike/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -995,7 +1176,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -1097,54 +1278,8 @@
         <color indexed="64"/>
       </left>
       <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
       <top/>
       <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -1165,16 +1300,38 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="medium">
         <color indexed="64"/>
       </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -1186,7 +1343,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1233,19 +1390,34 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1255,16 +1427,12 @@
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1554,15 +1722,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:R55"/>
+  <dimension ref="A1:R65"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
     <col min="3" max="3" width="18" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="27.42578125" customWidth="1"/>
     <col min="5" max="5" width="30.85546875" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17" bestFit="1" customWidth="1"/>
@@ -1570,11 +1738,10 @@
     <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.140625" customWidth="1"/>
     <col min="16" max="16" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="27" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="15.75" thickBot="1">
@@ -1588,14 +1755,14 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
-      <c r="N1" s="23"/>
-      <c r="O1" s="23"/>
-      <c r="P1" s="23"/>
-      <c r="Q1" s="23"/>
-      <c r="R1" s="23"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
+      <c r="N1" s="28"/>
+      <c r="O1" s="28"/>
+      <c r="P1" s="28"/>
+      <c r="Q1" s="28"/>
+      <c r="R1" s="28"/>
     </row>
     <row r="2" spans="1:18" ht="15.75" thickBot="1">
       <c r="A2" s="1"/>
@@ -1606,52 +1773,52 @@
         <v>3</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>98</v>
+        <v>122</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>117</v>
+        <v>151</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>150</v>
+        <v>193</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>228</v>
+        <v>286</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>172</v>
+        <v>220</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>229</v>
+        <v>287</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>227</v>
+        <v>285</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>230</v>
+        <v>288</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>231</v>
+        <v>289</v>
       </c>
       <c r="O2" s="5" t="s">
-        <v>232</v>
+        <v>290</v>
       </c>
       <c r="P2" s="5" t="s">
-        <v>233</v>
+        <v>291</v>
       </c>
       <c r="Q2" s="5" t="s">
-        <v>234</v>
+        <v>292</v>
       </c>
       <c r="R2" s="5" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" ht="15.75" thickBot="1">
       <c r="A3" s="1"/>
       <c r="B3" s="8">
         <f>ROW(B3) - ROW($B$2)</f>
@@ -1661,26 +1828,28 @@
         <v>4</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>118</v>
+        <v>152</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="I3" s="6"/>
+        <v>194</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>330</v>
+      </c>
       <c r="J3" s="6" t="s">
-        <v>173</v>
+        <v>221</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>209</v>
+        <v>265</v>
       </c>
       <c r="L3" s="6">
         <v>2</v>
@@ -1689,13 +1858,13 @@
         <f>L3*5</f>
         <v>10</v>
       </c>
-      <c r="N3" s="18">
+      <c r="N3" s="17">
         <v>100</v>
       </c>
-      <c r="O3" s="22" t="s">
-        <v>279</v>
-      </c>
-      <c r="P3" s="20">
+      <c r="O3" s="18" t="s">
+        <v>294</v>
+      </c>
+      <c r="P3" s="19">
         <v>1.1999999999999999E-3</v>
       </c>
       <c r="Q3" s="7">
@@ -1704,36 +1873,38 @@
       </c>
       <c r="R3" s="6"/>
     </row>
-    <row r="4" spans="1:18" ht="36">
+    <row r="4" spans="1:18">
       <c r="A4" s="1"/>
       <c r="B4" s="9">
-        <f t="shared" ref="B4:B40" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B51" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="15" t="s">
         <v>4</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>236</v>
+        <v>124</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>100</v>
+        <v>153</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>152</v>
-      </c>
-      <c r="I4" s="12"/>
+        <v>195</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>330</v>
+      </c>
       <c r="J4" s="12" t="s">
-        <v>174</v>
+        <v>222</v>
       </c>
       <c r="K4" s="12" t="s">
-        <v>210</v>
+        <v>266</v>
       </c>
       <c r="L4" s="12">
         <v>1</v>
@@ -1742,19 +1913,18 @@
         <f t="shared" ref="M4" si="1">L4*5</f>
         <v>5</v>
       </c>
-      <c r="N4" s="17" t="s">
-        <v>240</v>
-      </c>
-      <c r="O4" s="21" t="str">
-        <f>HYPERLINK(M4, "LCSC")</f>
-        <v>LCSC</v>
-      </c>
-      <c r="P4" s="19" t="s">
-        <v>247</v>
+      <c r="N4" s="12">
+        <v>5</v>
+      </c>
+      <c r="O4" s="18" t="s">
+        <v>294</v>
+      </c>
+      <c r="P4" s="13">
+        <v>0.87160000000000004</v>
       </c>
       <c r="Q4" s="13">
         <f t="shared" ref="Q4" si="2">P4*N4</f>
-        <v>0.53</v>
+        <v>4.3580000000000005</v>
       </c>
       <c r="R4" s="12"/>
     </row>
@@ -1768,43 +1938,45 @@
         <v>4</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>63</v>
+        <v>77</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>119</v>
+        <v>154</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="I5" s="6"/>
+        <v>194</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>330</v>
+      </c>
       <c r="J5" s="6" t="s">
-        <v>175</v>
+        <v>223</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>211</v>
+        <v>267</v>
       </c>
       <c r="L5" s="6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M5" s="6">
         <f>L5*5</f>
-        <v>5</v>
-      </c>
-      <c r="N5" s="18" t="s">
-        <v>241</v>
-      </c>
-      <c r="O5" s="21" t="str">
-        <f t="shared" ref="O5:O41" si="3">HYPERLINK(M5, "LCSC")</f>
+        <v>20</v>
+      </c>
+      <c r="N5" s="17" t="s">
+        <v>295</v>
+      </c>
+      <c r="O5" s="20" t="str">
+        <f t="shared" ref="O5:O9" si="3">HYPERLINK(M5, "LCSC")</f>
         <v>LCSC</v>
       </c>
-      <c r="P5" s="20" t="s">
-        <v>248</v>
+      <c r="P5" s="19" t="s">
+        <v>296</v>
       </c>
       <c r="Q5" s="7">
         <f>P5*N5</f>
@@ -1822,26 +1994,28 @@
         <v>4</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>101</v>
+        <v>125</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>120</v>
+        <v>155</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>151</v>
-      </c>
-      <c r="I6" s="12"/>
+        <v>194</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>330</v>
+      </c>
       <c r="J6" s="12" t="s">
-        <v>176</v>
+        <v>224</v>
       </c>
       <c r="K6" s="12" t="s">
-        <v>212</v>
+        <v>268</v>
       </c>
       <c r="L6" s="12">
         <v>1</v>
@@ -1850,15 +2024,15 @@
         <f t="shared" ref="M6" si="4">L6*5</f>
         <v>5</v>
       </c>
-      <c r="N6" s="17" t="s">
-        <v>242</v>
-      </c>
-      <c r="O6" s="21" t="str">
+      <c r="N6" s="21" t="s">
+        <v>297</v>
+      </c>
+      <c r="O6" s="20" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P6" s="19" t="s">
-        <v>249</v>
+      <c r="P6" s="22" t="s">
+        <v>298</v>
       </c>
       <c r="Q6" s="13">
         <f t="shared" ref="Q6" si="5">P6*N6</f>
@@ -1872,47 +2046,49 @@
         <f>ROW(B7) - ROW($B$2)</f>
         <v>5</v>
       </c>
-      <c r="C7" s="14" t="s">
-        <v>5</v>
+      <c r="C7" s="15" t="s">
+        <v>4</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>65</v>
+        <v>79</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>121</v>
+        <v>156</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="I7" s="6"/>
+        <v>196</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>330</v>
+      </c>
       <c r="J7" s="6" t="s">
-        <v>177</v>
+        <v>225</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>213</v>
+        <v>269</v>
       </c>
       <c r="L7" s="6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M7" s="6">
         <f>L7*5</f>
-        <v>20</v>
-      </c>
-      <c r="N7" s="18" t="s">
-        <v>240</v>
-      </c>
-      <c r="O7" s="21" t="str">
+        <v>5</v>
+      </c>
+      <c r="N7" s="17" t="s">
+        <v>299</v>
+      </c>
+      <c r="O7" s="20" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P7" s="20" t="s">
-        <v>250</v>
+      <c r="P7" s="19" t="s">
+        <v>300</v>
       </c>
       <c r="Q7" s="7">
         <f>P7*N7</f>
@@ -1930,26 +2106,28 @@
         <v>4</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>102</v>
+        <v>126</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>122</v>
+        <v>157</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>154</v>
-      </c>
-      <c r="I8" s="12"/>
+        <v>197</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>330</v>
+      </c>
       <c r="J8" s="12" t="s">
-        <v>178</v>
+        <v>226</v>
       </c>
       <c r="K8" s="12" t="s">
-        <v>212</v>
+        <v>268</v>
       </c>
       <c r="L8" s="12">
         <v>1</v>
@@ -1958,14 +2136,14 @@
         <f t="shared" ref="M8" si="6">L8*5</f>
         <v>5</v>
       </c>
-      <c r="N8" s="17">
+      <c r="N8" s="21">
         <v>6</v>
       </c>
-      <c r="O8" s="21" t="s">
-        <v>278</v>
-      </c>
-      <c r="P8" s="19" t="s">
-        <v>251</v>
+      <c r="O8" s="20" t="s">
+        <v>301</v>
+      </c>
+      <c r="P8" s="22" t="s">
+        <v>302</v>
       </c>
       <c r="Q8" s="13">
         <f t="shared" ref="Q8" si="7">P8*N8</f>
@@ -1979,30 +2157,32 @@
         <f>ROW(B9) - ROW($B$2)</f>
         <v>7</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="15" t="s">
         <v>4</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>67</v>
+        <v>81</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>123</v>
+        <v>158</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="I9" s="6"/>
+        <v>194</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>330</v>
+      </c>
       <c r="J9" s="6" t="s">
-        <v>179</v>
+        <v>227</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>214</v>
+        <v>270</v>
       </c>
       <c r="L9" s="6">
         <v>2</v>
@@ -2011,15 +2191,15 @@
         <f>L9*5</f>
         <v>10</v>
       </c>
-      <c r="N9" s="18" t="s">
-        <v>241</v>
-      </c>
-      <c r="O9" s="21" t="str">
+      <c r="N9" s="17" t="s">
+        <v>295</v>
+      </c>
+      <c r="O9" s="20" t="str">
         <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P9" s="20" t="s">
-        <v>252</v>
+      <c r="P9" s="19" t="s">
+        <v>303</v>
       </c>
       <c r="Q9" s="7">
         <f>P9*N9</f>
@@ -2037,26 +2217,28 @@
         <v>4</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>103</v>
+        <v>127</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>124</v>
+        <v>159</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>155</v>
-      </c>
-      <c r="I10" s="12"/>
+        <v>195</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>330</v>
+      </c>
       <c r="J10" s="12" t="s">
-        <v>180</v>
+        <v>228</v>
       </c>
       <c r="K10" s="12" t="s">
-        <v>215</v>
+        <v>271</v>
       </c>
       <c r="L10" s="12">
         <v>1</v>
@@ -2065,19 +2247,18 @@
         <f t="shared" ref="M10" si="8">L10*5</f>
         <v>5</v>
       </c>
-      <c r="N10" s="17" t="s">
-        <v>243</v>
-      </c>
-      <c r="O10" s="21" t="str">
-        <f t="shared" si="3"/>
-        <v>LCSC</v>
-      </c>
-      <c r="P10" s="19" t="s">
-        <v>253</v>
+      <c r="N10" s="12">
+        <v>6</v>
+      </c>
+      <c r="O10" s="20" t="s">
+        <v>294</v>
+      </c>
+      <c r="P10" s="13">
+        <v>0.13420000000000001</v>
       </c>
       <c r="Q10" s="13">
         <f t="shared" ref="Q10" si="9">P10*N10</f>
-        <v>16.221499999999999</v>
+        <v>0.80520000000000014</v>
       </c>
       <c r="R10" s="12"/>
     </row>
@@ -2087,30 +2268,32 @@
         <f>ROW(B11) - ROW($B$2)</f>
         <v>9</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="15" t="s">
         <v>4</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>101</v>
+        <v>125</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>125</v>
+        <v>160</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="I11" s="6"/>
+        <v>194</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>330</v>
+      </c>
       <c r="J11" s="6" t="s">
-        <v>181</v>
+        <v>229</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>211</v>
+        <v>267</v>
       </c>
       <c r="L11" s="6">
         <v>1</v>
@@ -2119,15 +2302,15 @@
         <f>L11*5</f>
         <v>5</v>
       </c>
-      <c r="N11" s="18" t="s">
-        <v>241</v>
-      </c>
-      <c r="O11" s="21" t="str">
-        <f t="shared" si="3"/>
+      <c r="N11" s="17" t="s">
+        <v>295</v>
+      </c>
+      <c r="O11" s="20" t="str">
+        <f t="shared" ref="O11:O12" si="10">HYPERLINK(M11, "LCSC")</f>
         <v>LCSC</v>
       </c>
-      <c r="P11" s="20" t="s">
-        <v>254</v>
+      <c r="P11" s="19" t="s">
+        <v>304</v>
       </c>
       <c r="Q11" s="7">
         <f>P11*N11</f>
@@ -2145,101 +2328,104 @@
         <v>4</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="G12" s="12" t="s">
-        <v>126</v>
+        <v>161</v>
       </c>
       <c r="H12" s="12" t="s">
-        <v>156</v>
-      </c>
-      <c r="I12" s="12"/>
+        <v>198</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>330</v>
+      </c>
       <c r="J12" s="12" t="s">
-        <v>182</v>
+        <v>230</v>
       </c>
       <c r="K12" s="12" t="s">
-        <v>214</v>
+        <v>270</v>
       </c>
       <c r="L12" s="12">
         <v>1</v>
       </c>
       <c r="M12" s="12">
-        <f t="shared" ref="M12" si="10">L12*5</f>
+        <f t="shared" ref="M12" si="11">L12*5</f>
         <v>5</v>
       </c>
-      <c r="N12" s="17" t="s">
-        <v>243</v>
-      </c>
-      <c r="O12" s="21" t="str">
-        <f t="shared" si="3"/>
+      <c r="N12" s="21" t="s">
+        <v>305</v>
+      </c>
+      <c r="O12" s="20" t="str">
+        <f t="shared" si="10"/>
         <v>LCSC</v>
       </c>
-      <c r="P12" s="19" t="s">
-        <v>255</v>
+      <c r="P12" s="22" t="s">
+        <v>306</v>
       </c>
       <c r="Q12" s="13">
-        <f t="shared" ref="Q12" si="11">P12*N12</f>
+        <f t="shared" ref="Q12" si="12">P12*N12</f>
         <v>0.49250000000000005</v>
       </c>
       <c r="R12" s="12"/>
     </row>
-    <row r="13" spans="1:18" ht="24">
+    <row r="13" spans="1:18">
       <c r="A13" s="1"/>
       <c r="B13" s="8">
         <f>ROW(B13) - ROW($B$2)</f>
         <v>11</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>104</v>
+        <v>125</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>127</v>
+        <v>162</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="I13" s="6"/>
+        <v>194</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>330</v>
+      </c>
       <c r="J13" s="6" t="s">
-        <v>183</v>
+        <v>231</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>237</v>
+        <v>270</v>
       </c>
       <c r="L13" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M13" s="6">
         <f>L13*5</f>
-        <v>15</v>
-      </c>
-      <c r="N13" s="18" t="s">
-        <v>240</v>
-      </c>
-      <c r="O13" s="21" t="str">
-        <f t="shared" si="3"/>
-        <v>LCSC</v>
-      </c>
-      <c r="P13" s="20" t="s">
-        <v>256</v>
+        <v>5</v>
+      </c>
+      <c r="N13" s="6">
+        <v>100</v>
+      </c>
+      <c r="O13" s="26" t="s">
+        <v>294</v>
+      </c>
+      <c r="P13" s="7">
+        <v>3.0999999999999999E-3</v>
       </c>
       <c r="Q13" s="7">
         <f>P13*N13</f>
-        <v>0.42000000000000004</v>
+        <v>0.31</v>
       </c>
       <c r="R13" s="6"/>
     </row>
@@ -2250,83 +2436,87 @@
         <v>12</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>105</v>
+        <v>128</v>
       </c>
       <c r="G14" s="12" t="s">
-        <v>128</v>
+        <v>163</v>
       </c>
       <c r="H14" s="12" t="s">
-        <v>158</v>
-      </c>
-      <c r="I14" s="12"/>
+        <v>199</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>330</v>
+      </c>
       <c r="J14" s="12" t="s">
-        <v>184</v>
-      </c>
-      <c r="K14" s="6" t="s">
-        <v>237</v>
+        <v>232</v>
+      </c>
+      <c r="K14" s="12" t="s">
+        <v>330</v>
       </c>
       <c r="L14" s="12">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M14" s="12">
-        <f t="shared" ref="M14" si="12">L14*5</f>
-        <v>30</v>
+        <f t="shared" ref="M14" si="13">L14*5</f>
+        <v>5</v>
       </c>
       <c r="N14" s="17" t="s">
-        <v>244</v>
-      </c>
-      <c r="O14" s="21" t="str">
-        <f t="shared" si="3"/>
+        <v>299</v>
+      </c>
+      <c r="O14" s="20" t="str">
+        <f t="shared" ref="O14" si="14">HYPERLINK(M14, "LCSC")</f>
         <v>LCSC</v>
       </c>
       <c r="P14" s="19" t="s">
-        <v>257</v>
+        <v>315</v>
       </c>
       <c r="Q14" s="13">
-        <f t="shared" ref="Q14" si="13">P14*N14</f>
-        <v>0.44</v>
+        <f t="shared" ref="Q14" si="15">P14*N14</f>
+        <v>0.42000000000000004</v>
       </c>
       <c r="R14" s="12"/>
     </row>
-    <row r="15" spans="1:18" ht="24">
+    <row r="15" spans="1:18">
       <c r="A15" s="1"/>
       <c r="B15" s="8">
         <f>ROW(B15) - ROW($B$2)</f>
         <v>13</v>
       </c>
-      <c r="C15" s="14" t="s">
-        <v>7</v>
+      <c r="C15" s="15" t="s">
+        <v>5</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>106</v>
+        <v>129</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>129</v>
+        <v>164</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="I15" s="6"/>
+        <v>200</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>330</v>
+      </c>
       <c r="J15" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="K15" s="6" t="s">
-        <v>237</v>
+        <v>331</v>
+      </c>
+      <c r="K15" s="12" t="s">
+        <v>330</v>
       </c>
       <c r="L15" s="6">
         <v>1</v>
@@ -2335,73 +2525,73 @@
         <f>L15*5</f>
         <v>5</v>
       </c>
-      <c r="N15" s="18" t="s">
-        <v>242</v>
-      </c>
-      <c r="O15" s="21" t="str">
-        <f t="shared" si="3"/>
-        <v>LCSC</v>
-      </c>
-      <c r="P15" s="20" t="s">
-        <v>258</v>
+      <c r="N15" s="6">
+        <v>20</v>
+      </c>
+      <c r="O15" s="26" t="s">
+        <v>294</v>
+      </c>
+      <c r="P15" s="7">
+        <v>2.8500000000000001E-2</v>
       </c>
       <c r="Q15" s="7">
         <f>P15*N15</f>
-        <v>0.44800000000000001</v>
+        <v>0.57000000000000006</v>
       </c>
       <c r="R15" s="6"/>
     </row>
-    <row r="16" spans="1:18" ht="24">
+    <row r="16" spans="1:18">
       <c r="A16" s="1"/>
       <c r="B16" s="9">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>236</v>
+        <v>129</v>
       </c>
       <c r="G16" s="12" t="s">
-        <v>130</v>
+        <v>165</v>
       </c>
       <c r="H16" s="12" t="s">
-        <v>160</v>
-      </c>
-      <c r="I16" s="12"/>
+        <v>200</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>330</v>
+      </c>
       <c r="J16" s="12" t="s">
-        <v>130</v>
-      </c>
-      <c r="K16" s="6" t="s">
-        <v>237</v>
+        <v>233</v>
+      </c>
+      <c r="K16" s="12" t="s">
+        <v>330</v>
       </c>
       <c r="L16" s="12">
         <v>1</v>
       </c>
       <c r="M16" s="12">
-        <f t="shared" ref="M16" si="14">L16*5</f>
+        <f t="shared" ref="M16" si="16">L16*5</f>
         <v>5</v>
       </c>
-      <c r="N16" s="17" t="s">
-        <v>245</v>
-      </c>
-      <c r="O16" s="21" t="str">
-        <f t="shared" si="3"/>
-        <v>LCSC</v>
-      </c>
-      <c r="P16" s="19" t="s">
-        <v>259</v>
+      <c r="N16" s="12">
+        <v>50</v>
+      </c>
+      <c r="O16" s="27" t="s">
+        <v>294</v>
+      </c>
+      <c r="P16" s="13">
+        <v>1.61E-2</v>
       </c>
       <c r="Q16" s="13">
-        <f t="shared" ref="Q16" si="15">P16*N16</f>
-        <v>0.86040000000000005</v>
+        <f t="shared" ref="Q16" si="17">P16*N16</f>
+        <v>0.80499999999999994</v>
       </c>
       <c r="R16" s="12"/>
     </row>
@@ -2412,137 +2602,143 @@
         <v>15</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="F17" s="12" t="s">
-        <v>236</v>
+        <v>89</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>130</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>131</v>
+        <v>166</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="I17" s="6"/>
+        <v>201</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>330</v>
+      </c>
       <c r="J17" s="6" t="s">
-        <v>186</v>
-      </c>
-      <c r="K17" s="6" t="s">
-        <v>237</v>
+        <v>234</v>
+      </c>
+      <c r="K17" s="12" t="s">
+        <v>330</v>
       </c>
       <c r="L17" s="6">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="M17" s="6">
         <f>L17*5</f>
-        <v>5</v>
-      </c>
-      <c r="N17" s="18" t="s">
-        <v>243</v>
-      </c>
-      <c r="O17" s="21" t="str">
-        <f t="shared" si="3"/>
+        <v>30</v>
+      </c>
+      <c r="N17" s="21" t="s">
+        <v>310</v>
+      </c>
+      <c r="O17" s="20" t="str">
+        <f t="shared" ref="O17:O19" si="18">HYPERLINK(M17, "LCSC")</f>
         <v>LCSC</v>
       </c>
-      <c r="P17" s="20" t="s">
-        <v>260</v>
+      <c r="P17" s="22" t="s">
+        <v>311</v>
       </c>
       <c r="Q17" s="7">
         <f>P17*N17</f>
-        <v>0.86899999999999999</v>
+        <v>0.44</v>
       </c>
       <c r="R17" s="6"/>
     </row>
-    <row r="18" spans="1:18" ht="48">
+    <row r="18" spans="1:18" ht="24">
       <c r="A18" s="1"/>
       <c r="B18" s="9">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>76</v>
+        <v>90</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>236</v>
+        <v>131</v>
       </c>
       <c r="G18" s="12" t="s">
-        <v>107</v>
+        <v>167</v>
       </c>
       <c r="H18" s="12" t="s">
-        <v>162</v>
-      </c>
-      <c r="I18" s="12"/>
+        <v>202</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>330</v>
+      </c>
       <c r="J18" s="12" t="s">
-        <v>187</v>
-      </c>
-      <c r="K18" s="6" t="s">
-        <v>237</v>
+        <v>235</v>
+      </c>
+      <c r="K18" s="12" t="s">
+        <v>330</v>
       </c>
       <c r="L18" s="12">
         <v>1</v>
       </c>
       <c r="M18" s="12">
-        <f t="shared" ref="M18" si="16">L18*5</f>
+        <f t="shared" ref="M18" si="19">L18*5</f>
         <v>5</v>
       </c>
       <c r="N18" s="17" t="s">
-        <v>243</v>
-      </c>
-      <c r="O18" s="21" t="str">
-        <f t="shared" si="3"/>
+        <v>297</v>
+      </c>
+      <c r="O18" s="20" t="str">
+        <f t="shared" si="18"/>
         <v>LCSC</v>
       </c>
       <c r="P18" s="19" t="s">
-        <v>261</v>
+        <v>312</v>
       </c>
       <c r="Q18" s="13">
-        <f t="shared" ref="Q18" si="17">P18*N18</f>
-        <v>0.19550000000000001</v>
+        <f t="shared" ref="Q18" si="20">P18*N18</f>
+        <v>0.44800000000000001</v>
       </c>
       <c r="R18" s="12"/>
     </row>
-    <row r="19" spans="1:18" ht="48">
+    <row r="19" spans="1:18" ht="24">
       <c r="A19" s="1"/>
       <c r="B19" s="8">
         <f>ROW(B19) - ROW($B$2)</f>
         <v>17</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="F19" s="12" t="s">
-        <v>236</v>
+        <v>91</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>132</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>108</v>
+        <v>168</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="I19" s="6"/>
+        <v>203</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>330</v>
+      </c>
       <c r="J19" s="6" t="s">
-        <v>188</v>
-      </c>
-      <c r="K19" s="6" t="s">
-        <v>237</v>
+        <v>168</v>
+      </c>
+      <c r="K19" s="12" t="s">
+        <v>330</v>
       </c>
       <c r="L19" s="6">
         <v>1</v>
@@ -2551,106 +2747,110 @@
         <f>L19*5</f>
         <v>5</v>
       </c>
-      <c r="N19" s="18" t="s">
-        <v>243</v>
-      </c>
-      <c r="O19" s="21" t="str">
-        <f t="shared" si="3"/>
+      <c r="N19" s="21" t="s">
+        <v>313</v>
+      </c>
+      <c r="O19" s="20" t="str">
+        <f t="shared" si="18"/>
         <v>LCSC</v>
       </c>
-      <c r="P19" s="20" t="s">
-        <v>262</v>
+      <c r="P19" s="22" t="s">
+        <v>314</v>
       </c>
       <c r="Q19" s="7">
         <f>P19*N19</f>
-        <v>0.85299999999999998</v>
+        <v>0.86040000000000005</v>
       </c>
       <c r="R19" s="6"/>
     </row>
-    <row r="20" spans="1:18" ht="36">
+    <row r="20" spans="1:18" ht="24">
       <c r="A20" s="1"/>
       <c r="B20" s="9">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>109</v>
+        <v>133</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>132</v>
+        <v>169</v>
       </c>
       <c r="H20" s="12" t="s">
-        <v>164</v>
-      </c>
-      <c r="I20" s="12"/>
+        <v>204</v>
+      </c>
+      <c r="I20" s="6" t="s">
+        <v>330</v>
+      </c>
       <c r="J20" s="12" t="s">
-        <v>189</v>
-      </c>
-      <c r="K20" s="6" t="s">
-        <v>237</v>
+        <v>236</v>
+      </c>
+      <c r="K20" s="12" t="s">
+        <v>330</v>
       </c>
       <c r="L20" s="12">
         <v>1</v>
       </c>
       <c r="M20" s="12">
-        <f t="shared" ref="M20" si="18">L20*5</f>
+        <f t="shared" ref="M20" si="21">L20*5</f>
         <v>5</v>
       </c>
       <c r="N20" s="17" t="s">
-        <v>242</v>
-      </c>
-      <c r="O20" s="21" t="str">
-        <f t="shared" si="3"/>
+        <v>305</v>
+      </c>
+      <c r="O20" s="20" t="str">
+        <f t="shared" ref="O20:O22" si="22">HYPERLINK(M20, "LCSC")</f>
         <v>LCSC</v>
       </c>
       <c r="P20" s="19" t="s">
-        <v>263</v>
+        <v>307</v>
       </c>
       <c r="Q20" s="13">
-        <f t="shared" ref="Q20" si="19">P20*N20</f>
-        <v>0.51700000000000002</v>
+        <f t="shared" ref="Q20" si="23">P20*N20</f>
+        <v>0.86899999999999999</v>
       </c>
       <c r="R20" s="12"/>
     </row>
-    <row r="21" spans="1:18" ht="36">
+    <row r="21" spans="1:18" ht="48">
       <c r="A21" s="1"/>
       <c r="B21" s="8">
         <f>ROW(B21) - ROW($B$2)</f>
         <v>19</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>110</v>
+        <v>134</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="I21" s="6"/>
+        <v>205</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>330</v>
+      </c>
       <c r="J21" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="K21" s="6" t="s">
         <v>237</v>
+      </c>
+      <c r="K21" s="12" t="s">
+        <v>330</v>
       </c>
       <c r="L21" s="6">
         <v>1</v>
@@ -2659,73 +2859,75 @@
         <f>L21*5</f>
         <v>5</v>
       </c>
-      <c r="N21" s="18" t="s">
-        <v>240</v>
-      </c>
-      <c r="O21" s="21" t="str">
-        <f t="shared" si="3"/>
+      <c r="N21" s="21" t="s">
+        <v>305</v>
+      </c>
+      <c r="O21" s="20" t="str">
+        <f t="shared" si="22"/>
         <v>LCSC</v>
       </c>
-      <c r="P21" s="20" t="s">
-        <v>264</v>
+      <c r="P21" s="22" t="s">
+        <v>308</v>
       </c>
       <c r="Q21" s="7">
         <f>P21*N21</f>
-        <v>0.54800000000000004</v>
+        <v>0.19550000000000001</v>
       </c>
       <c r="R21" s="6"/>
     </row>
-    <row r="22" spans="1:18" ht="36">
+    <row r="22" spans="1:18" ht="48">
       <c r="A22" s="1"/>
       <c r="B22" s="9">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="E22" s="12" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>111</v>
+        <v>135</v>
       </c>
       <c r="G22" s="12" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H22" s="12" t="s">
-        <v>165</v>
-      </c>
-      <c r="I22" s="12"/>
+        <v>206</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>330</v>
+      </c>
       <c r="J22" s="12" t="s">
-        <v>191</v>
-      </c>
-      <c r="K22" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
+      </c>
+      <c r="K22" s="12" t="s">
+        <v>330</v>
       </c>
       <c r="L22" s="12">
         <v>1</v>
       </c>
       <c r="M22" s="12">
-        <f t="shared" ref="M22" si="20">L22*5</f>
+        <f t="shared" ref="M22" si="24">L22*5</f>
         <v>5</v>
       </c>
       <c r="N22" s="17" t="s">
-        <v>244</v>
-      </c>
-      <c r="O22" s="21" t="str">
-        <f t="shared" si="3"/>
+        <v>305</v>
+      </c>
+      <c r="O22" s="20" t="str">
+        <f t="shared" si="22"/>
         <v>LCSC</v>
       </c>
       <c r="P22" s="19" t="s">
-        <v>265</v>
+        <v>309</v>
       </c>
       <c r="Q22" s="13">
-        <f t="shared" ref="Q22" si="21">P22*N22</f>
-        <v>0.85000000000000009</v>
+        <f t="shared" ref="Q22" si="25">P22*N22</f>
+        <v>0.85299999999999998</v>
       </c>
       <c r="R22" s="12"/>
     </row>
@@ -2736,29 +2938,31 @@
         <v>21</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>110</v>
+        <v>136</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>135</v>
+        <v>170</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="I23" s="6"/>
+        <v>207</v>
+      </c>
+      <c r="I23" s="6" t="s">
+        <v>330</v>
+      </c>
       <c r="J23" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="K23" s="6" t="s">
-        <v>237</v>
+        <v>239</v>
+      </c>
+      <c r="K23" s="12" t="s">
+        <v>330</v>
       </c>
       <c r="L23" s="6">
         <v>1</v>
@@ -2767,73 +2971,73 @@
         <f>L23*5</f>
         <v>5</v>
       </c>
-      <c r="N23" s="18" t="s">
-        <v>240</v>
-      </c>
-      <c r="O23" s="21" t="str">
-        <f t="shared" si="3"/>
-        <v>LCSC</v>
-      </c>
-      <c r="P23" s="20" t="s">
-        <v>266</v>
+      <c r="N23" s="6">
+        <v>5</v>
+      </c>
+      <c r="O23" s="26" t="s">
+        <v>294</v>
+      </c>
+      <c r="P23" s="7">
+        <v>9.9699999999999997E-2</v>
       </c>
       <c r="Q23" s="7">
         <f>P23*N23</f>
-        <v>0.55000000000000004</v>
+        <v>0.4985</v>
       </c>
       <c r="R23" s="6"/>
     </row>
-    <row r="24" spans="1:18">
+    <row r="24" spans="1:18" ht="24">
       <c r="A24" s="1"/>
       <c r="B24" s="9">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="E24" s="12" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>112</v>
+        <v>137</v>
       </c>
       <c r="G24" s="12" t="s">
-        <v>136</v>
+        <v>171</v>
       </c>
       <c r="H24" s="12" t="s">
-        <v>151</v>
-      </c>
-      <c r="I24" s="12"/>
+        <v>208</v>
+      </c>
+      <c r="I24" s="6" t="s">
+        <v>330</v>
+      </c>
       <c r="J24" s="12" t="s">
-        <v>193</v>
+        <v>240</v>
       </c>
       <c r="K24" s="12" t="s">
-        <v>216</v>
+        <v>330</v>
       </c>
       <c r="L24" s="12">
+        <v>1</v>
+      </c>
+      <c r="M24" s="12">
+        <f t="shared" ref="M24" si="26">L24*5</f>
         <v>5</v>
       </c>
-      <c r="M24" s="12">
-        <f t="shared" ref="M24" si="22">L24*5</f>
-        <v>25</v>
-      </c>
-      <c r="N24" s="17" t="s">
-        <v>241</v>
-      </c>
-      <c r="O24" s="21" t="str">
-        <f t="shared" si="3"/>
-        <v>LCSC</v>
-      </c>
-      <c r="P24" s="19" t="s">
-        <v>267</v>
+      <c r="N24" s="12">
+        <v>5</v>
+      </c>
+      <c r="O24" s="27" t="s">
+        <v>294</v>
+      </c>
+      <c r="P24" s="13">
+        <v>0.3271</v>
       </c>
       <c r="Q24" s="13">
-        <f t="shared" ref="Q24" si="23">P24*N24</f>
-        <v>0.06</v>
+        <f t="shared" ref="Q24" si="27">P24*N24</f>
+        <v>1.6355</v>
       </c>
       <c r="R24" s="12"/>
     </row>
@@ -2846,135 +3050,141 @@
       <c r="C25" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="D25" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="F25" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="G25" s="12" t="s">
-        <v>238</v>
-      </c>
-      <c r="H25" s="12" t="s">
-        <v>239</v>
-      </c>
-      <c r="I25" s="6"/>
-      <c r="J25" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="K25" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="L25" s="6">
-        <v>3</v>
-      </c>
-      <c r="M25" s="6">
+      <c r="D25" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="E25" s="23" t="s">
+        <v>97</v>
+      </c>
+      <c r="F25" s="23" t="s">
+        <v>138</v>
+      </c>
+      <c r="G25" s="23" t="s">
+        <v>138</v>
+      </c>
+      <c r="H25" s="23" t="s">
+        <v>330</v>
+      </c>
+      <c r="I25" s="23" t="s">
+        <v>330</v>
+      </c>
+      <c r="J25" s="23" t="s">
+        <v>330</v>
+      </c>
+      <c r="K25" s="23" t="s">
+        <v>330</v>
+      </c>
+      <c r="L25" s="23">
+        <v>5</v>
+      </c>
+      <c r="M25" s="23">
         <f>L25*5</f>
-        <v>15</v>
-      </c>
-      <c r="N25" s="18" t="s">
-        <v>240</v>
-      </c>
-      <c r="O25" s="21" t="str">
-        <f t="shared" si="3"/>
-        <v>LCSC</v>
-      </c>
-      <c r="P25" s="20" t="s">
-        <v>268</v>
-      </c>
-      <c r="Q25" s="7">
-        <f>P25*N25</f>
-        <v>0.57399999999999995</v>
-      </c>
-      <c r="R25" s="6"/>
-    </row>
-    <row r="26" spans="1:18">
+        <v>25</v>
+      </c>
+      <c r="N25" s="23" t="s">
+        <v>330</v>
+      </c>
+      <c r="O25" s="23" t="s">
+        <v>330</v>
+      </c>
+      <c r="P25" s="24" t="s">
+        <v>330</v>
+      </c>
+      <c r="Q25" s="24" t="s">
+        <v>330</v>
+      </c>
+      <c r="R25" s="25" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" ht="36">
       <c r="A26" s="1"/>
       <c r="B26" s="9">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="F26" s="12" t="s">
-        <v>113</v>
+        <v>139</v>
       </c>
       <c r="G26" s="12" t="s">
-        <v>137</v>
+        <v>172</v>
       </c>
       <c r="H26" s="12" t="s">
-        <v>151</v>
-      </c>
-      <c r="I26" s="12"/>
+        <v>209</v>
+      </c>
+      <c r="I26" s="12" t="s">
+        <v>330</v>
+      </c>
       <c r="J26" s="12" t="s">
-        <v>195</v>
+        <v>241</v>
       </c>
       <c r="K26" s="12" t="s">
-        <v>217</v>
+        <v>330</v>
       </c>
       <c r="L26" s="12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M26" s="12">
-        <f t="shared" ref="M26" si="24">L26*5</f>
-        <v>10</v>
-      </c>
-      <c r="N26" s="17" t="s">
-        <v>241</v>
-      </c>
-      <c r="O26" s="21" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="M26" si="28">L26*5</f>
+        <v>5</v>
+      </c>
+      <c r="N26" s="21" t="s">
+        <v>297</v>
+      </c>
+      <c r="O26" s="20" t="str">
+        <f t="shared" ref="O26" si="29">HYPERLINK(M26, "LCSC")</f>
         <v>LCSC</v>
       </c>
-      <c r="P26" s="19" t="s">
-        <v>269</v>
+      <c r="P26" s="22" t="s">
+        <v>328</v>
       </c>
       <c r="Q26" s="13">
-        <f t="shared" ref="Q26" si="25">P26*N26</f>
-        <v>0.11</v>
+        <f t="shared" ref="Q26" si="30">P26*N26</f>
+        <v>0.51700000000000002</v>
       </c>
       <c r="R26" s="12"/>
     </row>
-    <row r="27" spans="1:18">
+    <row r="27" spans="1:18" ht="36">
       <c r="A27" s="1"/>
       <c r="B27" s="8">
         <f>ROW(B27) - ROW($B$2)</f>
         <v>25</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>113</v>
+        <v>140</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>138</v>
+        <v>173</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="I27" s="6"/>
+        <v>210</v>
+      </c>
+      <c r="I27" s="12" t="s">
+        <v>330</v>
+      </c>
       <c r="J27" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="K27" s="6" t="s">
-        <v>218</v>
+        <v>242</v>
+      </c>
+      <c r="K27" s="12" t="s">
+        <v>330</v>
       </c>
       <c r="L27" s="6">
         <v>2</v>
@@ -2983,19 +3193,18 @@
         <f>L27*5</f>
         <v>10</v>
       </c>
-      <c r="N27" s="18" t="s">
-        <v>241</v>
-      </c>
-      <c r="O27" s="21" t="str">
-        <f t="shared" si="3"/>
-        <v>LCSC</v>
-      </c>
-      <c r="P27" s="20" t="s">
-        <v>270</v>
+      <c r="N27" s="6">
+        <v>50</v>
+      </c>
+      <c r="O27" s="26" t="s">
+        <v>294</v>
+      </c>
+      <c r="P27" s="7">
+        <v>1.66E-2</v>
       </c>
       <c r="Q27" s="7">
         <f>P27*N27</f>
-        <v>0.12</v>
+        <v>0.83</v>
       </c>
       <c r="R27" s="6"/>
     </row>
@@ -3005,51 +3214,52 @@
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C28" s="14" t="s">
-        <v>13</v>
+      <c r="C28" s="15" t="s">
+        <v>15</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="F28" s="12" t="s">
-        <v>112</v>
+        <v>141</v>
       </c>
       <c r="G28" s="12" t="s">
-        <v>139</v>
+        <v>174</v>
       </c>
       <c r="H28" s="12" t="s">
-        <v>167</v>
-      </c>
-      <c r="I28" s="12"/>
+        <v>211</v>
+      </c>
+      <c r="I28" s="12" t="s">
+        <v>330</v>
+      </c>
       <c r="J28" s="12" t="s">
-        <v>197</v>
+        <v>243</v>
       </c>
       <c r="K28" s="12" t="s">
-        <v>219</v>
+        <v>330</v>
       </c>
       <c r="L28" s="12">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M28" s="12">
-        <f t="shared" ref="M28" si="26">L28*5</f>
-        <v>20</v>
-      </c>
-      <c r="N28" s="17" t="s">
-        <v>240</v>
-      </c>
-      <c r="O28" s="21" t="str">
-        <f t="shared" si="3"/>
-        <v>LCSC</v>
-      </c>
-      <c r="P28" s="19" t="s">
-        <v>271</v>
+        <f t="shared" ref="M28" si="31">L28*5</f>
+        <v>5</v>
+      </c>
+      <c r="N28" s="12">
+        <v>50</v>
+      </c>
+      <c r="O28" s="26" t="s">
+        <v>294</v>
+      </c>
+      <c r="P28" s="13">
+        <v>9.5999999999999992E-3</v>
       </c>
       <c r="Q28" s="13">
-        <f t="shared" ref="Q28" si="27">P28*N28</f>
-        <v>0.37</v>
+        <f t="shared" ref="Q28" si="32">P28*N28</f>
+        <v>0.48</v>
       </c>
       <c r="R28" s="12"/>
     </row>
@@ -3060,50 +3270,52 @@
         <v>27</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>113</v>
+        <v>142</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>140</v>
+        <v>175</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="I29" s="6"/>
+        <v>194</v>
+      </c>
+      <c r="I29" s="12" t="s">
+        <v>330</v>
+      </c>
       <c r="J29" s="6" t="s">
-        <v>198</v>
+        <v>244</v>
       </c>
       <c r="K29" s="6" t="s">
-        <v>220</v>
+        <v>272</v>
       </c>
       <c r="L29" s="6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M29" s="6">
         <f>L29*5</f>
-        <v>5</v>
-      </c>
-      <c r="N29" s="18" t="s">
-        <v>241</v>
-      </c>
-      <c r="O29" s="21" t="str">
-        <f t="shared" si="3"/>
+        <v>20</v>
+      </c>
+      <c r="N29" s="21" t="s">
+        <v>295</v>
+      </c>
+      <c r="O29" s="20" t="str">
+        <f t="shared" ref="O29:O38" si="33">HYPERLINK(M29, "LCSC")</f>
         <v>LCSC</v>
       </c>
-      <c r="P29" s="20" t="s">
-        <v>270</v>
+      <c r="P29" s="22" t="s">
+        <v>321</v>
       </c>
       <c r="Q29" s="7">
         <f>P29*N29</f>
-        <v>0.12</v>
+        <v>0.06</v>
       </c>
       <c r="R29" s="6"/>
     </row>
@@ -3114,50 +3326,48 @@
         <v>28</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="E30" s="12" t="s">
-        <v>88</v>
+        <v>102</v>
       </c>
       <c r="F30" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="G30" s="12" t="s">
-        <v>141</v>
-      </c>
-      <c r="H30" s="12" t="s">
-        <v>151</v>
-      </c>
-      <c r="I30" s="12"/>
+        <v>143</v>
+      </c>
+      <c r="G30" s="12"/>
+      <c r="H30" s="12"/>
+      <c r="I30" s="12" t="s">
+        <v>330</v>
+      </c>
       <c r="J30" s="12" t="s">
-        <v>199</v>
+        <v>245</v>
       </c>
       <c r="K30" s="12" t="s">
-        <v>221</v>
+        <v>272</v>
       </c>
       <c r="L30" s="12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M30" s="12">
-        <f t="shared" ref="M30" si="28">L30*5</f>
-        <v>5</v>
+        <f t="shared" ref="M30" si="34">L30*5</f>
+        <v>15</v>
       </c>
       <c r="N30" s="17" t="s">
-        <v>241</v>
-      </c>
-      <c r="O30" s="21" t="str">
-        <f t="shared" si="3"/>
+        <v>299</v>
+      </c>
+      <c r="O30" s="20" t="str">
+        <f t="shared" si="33"/>
         <v>LCSC</v>
       </c>
       <c r="P30" s="19" t="s">
-        <v>272</v>
+        <v>322</v>
       </c>
       <c r="Q30" s="13">
-        <f t="shared" ref="Q30" si="29">P30*N30</f>
-        <v>6.9999999999999993E-2</v>
+        <f t="shared" ref="Q30" si="35">P30*N30</f>
+        <v>0.57399999999999995</v>
       </c>
       <c r="R30" s="12"/>
     </row>
@@ -3168,50 +3378,52 @@
         <v>29</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>112</v>
+        <v>143</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>142</v>
+        <v>176</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="I31" s="6"/>
+        <v>194</v>
+      </c>
+      <c r="I31" s="12" t="s">
+        <v>330</v>
+      </c>
       <c r="J31" s="6" t="s">
-        <v>200</v>
+        <v>246</v>
       </c>
       <c r="K31" s="6" t="s">
-        <v>217</v>
+        <v>273</v>
       </c>
       <c r="L31" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M31" s="6">
         <f>L31*5</f>
-        <v>5</v>
-      </c>
-      <c r="N31" s="18" t="s">
-        <v>241</v>
-      </c>
-      <c r="O31" s="21" t="str">
-        <f t="shared" si="3"/>
+        <v>10</v>
+      </c>
+      <c r="N31" s="21" t="s">
+        <v>295</v>
+      </c>
+      <c r="O31" s="20" t="str">
+        <f t="shared" si="33"/>
         <v>LCSC</v>
       </c>
-      <c r="P31" s="20" t="s">
-        <v>267</v>
+      <c r="P31" s="22" t="s">
+        <v>323</v>
       </c>
       <c r="Q31" s="7">
         <f>P31*N31</f>
-        <v>0.06</v>
+        <v>0.11</v>
       </c>
       <c r="R31" s="6"/>
     </row>
@@ -3222,50 +3434,52 @@
         <v>30</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="E32" s="12" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="F32" s="12" t="s">
-        <v>112</v>
+        <v>143</v>
       </c>
       <c r="G32" s="12" t="s">
-        <v>143</v>
+        <v>177</v>
       </c>
       <c r="H32" s="12" t="s">
-        <v>151</v>
-      </c>
-      <c r="I32" s="12"/>
+        <v>194</v>
+      </c>
+      <c r="I32" s="12" t="s">
+        <v>330</v>
+      </c>
       <c r="J32" s="12" t="s">
-        <v>201</v>
+        <v>247</v>
       </c>
       <c r="K32" s="12" t="s">
-        <v>222</v>
+        <v>274</v>
       </c>
       <c r="L32" s="12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M32" s="12">
-        <f t="shared" ref="M32" si="30">L32*5</f>
-        <v>5</v>
+        <f t="shared" ref="M32" si="36">L32*5</f>
+        <v>10</v>
       </c>
       <c r="N32" s="17" t="s">
-        <v>241</v>
-      </c>
-      <c r="O32" s="21" t="str">
-        <f t="shared" si="3"/>
+        <v>295</v>
+      </c>
+      <c r="O32" s="20" t="str">
+        <f t="shared" si="33"/>
         <v>LCSC</v>
       </c>
       <c r="P32" s="19" t="s">
-        <v>267</v>
+        <v>324</v>
       </c>
       <c r="Q32" s="13">
-        <f t="shared" ref="Q32" si="31">P32*N32</f>
-        <v>0.06</v>
+        <f t="shared" ref="Q32" si="37">P32*N32</f>
+        <v>0.12</v>
       </c>
       <c r="R32" s="12"/>
     </row>
@@ -3275,51 +3489,53 @@
         <f>ROW(B33) - ROW($B$2)</f>
         <v>31</v>
       </c>
-      <c r="C33" s="14" t="s">
-        <v>13</v>
+      <c r="C33" s="15" t="s">
+        <v>16</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>112</v>
+        <v>142</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>144</v>
+        <v>178</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="I33" s="6"/>
+        <v>212</v>
+      </c>
+      <c r="I33" s="12" t="s">
+        <v>330</v>
+      </c>
       <c r="J33" s="6" t="s">
-        <v>202</v>
+        <v>248</v>
       </c>
       <c r="K33" s="6" t="s">
-        <v>223</v>
+        <v>275</v>
       </c>
       <c r="L33" s="6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M33" s="6">
         <f>L33*5</f>
-        <v>5</v>
-      </c>
-      <c r="N33" s="18" t="s">
-        <v>241</v>
-      </c>
-      <c r="O33" s="21" t="str">
-        <f t="shared" si="3"/>
+        <v>20</v>
+      </c>
+      <c r="N33" s="21" t="s">
+        <v>299</v>
+      </c>
+      <c r="O33" s="20" t="str">
+        <f t="shared" si="33"/>
         <v>LCSC</v>
       </c>
-      <c r="P33" s="20" t="s">
-        <v>272</v>
+      <c r="P33" s="22" t="s">
+        <v>325</v>
       </c>
       <c r="Q33" s="7">
         <f>P33*N33</f>
-        <v>6.9999999999999993E-2</v>
+        <v>0.37</v>
       </c>
       <c r="R33" s="6"/>
     </row>
@@ -3330,50 +3546,52 @@
         <v>32</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="F34" s="12" t="s">
-        <v>112</v>
+        <v>143</v>
       </c>
       <c r="G34" s="12" t="s">
-        <v>145</v>
+        <v>179</v>
       </c>
       <c r="H34" s="12" t="s">
-        <v>151</v>
-      </c>
-      <c r="I34" s="12"/>
+        <v>194</v>
+      </c>
+      <c r="I34" s="12" t="s">
+        <v>330</v>
+      </c>
       <c r="J34" s="12" t="s">
-        <v>203</v>
+        <v>249</v>
       </c>
       <c r="K34" s="12" t="s">
-        <v>224</v>
+        <v>276</v>
       </c>
       <c r="L34" s="12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M34" s="12">
-        <f t="shared" ref="M34" si="32">L34*5</f>
-        <v>10</v>
+        <f t="shared" ref="M34" si="38">L34*5</f>
+        <v>5</v>
       </c>
       <c r="N34" s="17" t="s">
-        <v>241</v>
-      </c>
-      <c r="O34" s="21" t="str">
-        <f t="shared" si="3"/>
+        <v>295</v>
+      </c>
+      <c r="O34" s="20" t="str">
+        <f t="shared" si="33"/>
         <v>LCSC</v>
       </c>
       <c r="P34" s="19" t="s">
-        <v>272</v>
+        <v>324</v>
       </c>
       <c r="Q34" s="13">
-        <f t="shared" ref="Q34" si="33">P34*N34</f>
-        <v>6.9999999999999993E-2</v>
+        <f t="shared" ref="Q34" si="39">P34*N34</f>
+        <v>0.12</v>
       </c>
       <c r="R34" s="12"/>
     </row>
@@ -3384,29 +3602,31 @@
         <v>33</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>113</v>
+        <v>142</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>146</v>
+        <v>180</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="I35" s="6"/>
+        <v>194</v>
+      </c>
+      <c r="I35" s="12" t="s">
+        <v>330</v>
+      </c>
       <c r="J35" s="6" t="s">
-        <v>204</v>
+        <v>250</v>
       </c>
       <c r="K35" s="6" t="s">
-        <v>225</v>
+        <v>277</v>
       </c>
       <c r="L35" s="6">
         <v>1</v>
@@ -3415,19 +3635,19 @@
         <f>L35*5</f>
         <v>5</v>
       </c>
-      <c r="N35" s="18" t="s">
-        <v>241</v>
-      </c>
-      <c r="O35" s="21" t="str">
-        <f t="shared" si="3"/>
+      <c r="N35" s="21" t="s">
+        <v>295</v>
+      </c>
+      <c r="O35" s="20" t="str">
+        <f t="shared" si="33"/>
         <v>LCSC</v>
       </c>
-      <c r="P35" s="20" t="s">
-        <v>270</v>
+      <c r="P35" s="22" t="s">
+        <v>326</v>
       </c>
       <c r="Q35" s="7">
         <f>P35*N35</f>
-        <v>0.12</v>
+        <v>6.9999999999999993E-2</v>
       </c>
       <c r="R35" s="6"/>
     </row>
@@ -3438,50 +3658,52 @@
         <v>34</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D36" s="12" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="E36" s="12" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="F36" s="12" t="s">
-        <v>113</v>
+        <v>142</v>
       </c>
       <c r="G36" s="12" t="s">
-        <v>147</v>
+        <v>181</v>
       </c>
       <c r="H36" s="12" t="s">
-        <v>151</v>
-      </c>
-      <c r="I36" s="12"/>
+        <v>194</v>
+      </c>
+      <c r="I36" s="12" t="s">
+        <v>330</v>
+      </c>
       <c r="J36" s="12" t="s">
-        <v>205</v>
+        <v>251</v>
       </c>
       <c r="K36" s="12" t="s">
-        <v>226</v>
+        <v>273</v>
       </c>
       <c r="L36" s="12">
         <v>1</v>
       </c>
       <c r="M36" s="12">
-        <f t="shared" ref="M36" si="34">L36*5</f>
+        <f t="shared" ref="M36" si="40">L36*5</f>
         <v>5</v>
       </c>
       <c r="N36" s="17" t="s">
-        <v>241</v>
-      </c>
-      <c r="O36" s="21" t="str">
-        <f t="shared" si="3"/>
+        <v>295</v>
+      </c>
+      <c r="O36" s="20" t="str">
+        <f t="shared" si="33"/>
         <v>LCSC</v>
       </c>
       <c r="P36" s="19" t="s">
-        <v>273</v>
+        <v>321</v>
       </c>
       <c r="Q36" s="13">
-        <f t="shared" ref="Q36" si="35">P36*N36</f>
-        <v>0.53</v>
+        <f t="shared" ref="Q36" si="41">P36*N36</f>
+        <v>0.06</v>
       </c>
       <c r="R36" s="12"/>
     </row>
@@ -3492,29 +3714,31 @@
         <v>35</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="F37" s="12" t="s">
-        <v>236</v>
+        <v>109</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>142</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>114</v>
+        <v>182</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="I37" s="6"/>
+        <v>194</v>
+      </c>
+      <c r="I37" s="12" t="s">
+        <v>330</v>
+      </c>
       <c r="J37" s="6" t="s">
-        <v>206</v>
+        <v>252</v>
       </c>
       <c r="K37" s="6" t="s">
-        <v>237</v>
+        <v>278</v>
       </c>
       <c r="L37" s="6">
         <v>2</v>
@@ -3523,19 +3747,19 @@
         <f>L37*5</f>
         <v>10</v>
       </c>
-      <c r="N37" s="18" t="s">
-        <v>242</v>
-      </c>
-      <c r="O37" s="21" t="str">
-        <f t="shared" si="3"/>
+      <c r="N37" s="21" t="s">
+        <v>295</v>
+      </c>
+      <c r="O37" s="20" t="str">
+        <f t="shared" si="33"/>
         <v>LCSC</v>
       </c>
-      <c r="P37" s="20" t="s">
-        <v>274</v>
+      <c r="P37" s="22" t="s">
+        <v>321</v>
       </c>
       <c r="Q37" s="7">
         <f>P37*N37</f>
-        <v>1.5549999999999999</v>
+        <v>0.06</v>
       </c>
       <c r="R37" s="6"/>
     </row>
@@ -3549,47 +3773,49 @@
         <v>16</v>
       </c>
       <c r="D38" s="12" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E38" s="12" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="F38" s="12" t="s">
-        <v>236</v>
+        <v>142</v>
       </c>
       <c r="G38" s="12" t="s">
-        <v>115</v>
+        <v>183</v>
       </c>
       <c r="H38" s="12" t="s">
-        <v>169</v>
-      </c>
-      <c r="I38" s="12"/>
-      <c r="J38" s="6" t="s">
-        <v>280</v>
-      </c>
-      <c r="K38" s="6" t="s">
-        <v>237</v>
+        <v>194</v>
+      </c>
+      <c r="I38" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="J38" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="K38" s="12" t="s">
+        <v>279</v>
       </c>
       <c r="L38" s="12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M38" s="12">
-        <f t="shared" ref="M38" si="36">L38*5</f>
-        <v>5</v>
-      </c>
-      <c r="N38" s="17" t="s">
-        <v>243</v>
-      </c>
-      <c r="O38" s="21" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="M38" si="42">L38*5</f>
+        <v>10</v>
+      </c>
+      <c r="N38" s="21" t="s">
+        <v>295</v>
+      </c>
+      <c r="O38" s="20" t="str">
+        <f t="shared" si="33"/>
         <v>LCSC</v>
       </c>
-      <c r="P38" s="19" t="s">
-        <v>275</v>
+      <c r="P38" s="22" t="s">
+        <v>326</v>
       </c>
       <c r="Q38" s="13">
-        <f t="shared" ref="Q38" si="37">P38*N38</f>
-        <v>6.6879999999999997</v>
+        <f t="shared" ref="Q38" si="43">P38*N38</f>
+        <v>6.9999999999999993E-2</v>
       </c>
       <c r="R38" s="12"/>
     </row>
@@ -3603,47 +3829,48 @@
         <v>17</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="F39" s="12" t="s">
-        <v>236</v>
+        <v>111</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>143</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>148</v>
+        <v>184</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="I39" s="6"/>
+        <v>194</v>
+      </c>
+      <c r="I39" s="12" t="s">
+        <v>330</v>
+      </c>
       <c r="J39" s="6" t="s">
-        <v>207</v>
+        <v>254</v>
       </c>
       <c r="K39" s="6" t="s">
-        <v>237</v>
+        <v>280</v>
       </c>
       <c r="L39" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M39" s="6">
         <f>L39*5</f>
-        <v>15</v>
-      </c>
-      <c r="N39" s="18" t="s">
-        <v>246</v>
-      </c>
-      <c r="O39" s="21" t="str">
-        <f t="shared" si="3"/>
-        <v>LCSC</v>
-      </c>
-      <c r="P39" s="20" t="s">
-        <v>276</v>
+        <v>10</v>
+      </c>
+      <c r="N39" s="6">
+        <v>100</v>
+      </c>
+      <c r="O39" s="20" t="s">
+        <v>294</v>
+      </c>
+      <c r="P39" s="7">
+        <v>1E-3</v>
       </c>
       <c r="Q39" s="7">
         <f>P39*N39</f>
-        <v>10.429500000000001</v>
+        <v>0.1</v>
       </c>
       <c r="R39" s="6"/>
     </row>
@@ -3654,83 +3881,87 @@
         <v>38</v>
       </c>
       <c r="C40" s="15" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D40" s="12" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="E40" s="12" t="s">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="F40" s="12" t="s">
-        <v>116</v>
+        <v>143</v>
       </c>
       <c r="G40" s="12" t="s">
-        <v>149</v>
+        <v>185</v>
       </c>
       <c r="H40" s="12" t="s">
-        <v>171</v>
-      </c>
-      <c r="I40" s="12"/>
+        <v>194</v>
+      </c>
+      <c r="I40" s="12" t="s">
+        <v>330</v>
+      </c>
       <c r="J40" s="12" t="s">
-        <v>208</v>
-      </c>
-      <c r="K40" s="6" t="s">
-        <v>237</v>
+        <v>255</v>
+      </c>
+      <c r="K40" s="12" t="s">
+        <v>281</v>
       </c>
       <c r="L40" s="12">
         <v>1</v>
       </c>
       <c r="M40" s="12">
-        <f t="shared" ref="M40" si="38">L40*5</f>
+        <f t="shared" ref="M40" si="44">L40*5</f>
         <v>5</v>
       </c>
       <c r="N40" s="17" t="s">
-        <v>243</v>
-      </c>
-      <c r="O40" s="21" t="str">
-        <f t="shared" si="3"/>
+        <v>295</v>
+      </c>
+      <c r="O40" s="20" t="str">
+        <f t="shared" ref="O40:O41" si="45">HYPERLINK(M40, "LCSC")</f>
         <v>LCSC</v>
       </c>
       <c r="P40" s="19" t="s">
-        <v>277</v>
+        <v>324</v>
       </c>
       <c r="Q40" s="13">
-        <f t="shared" ref="Q40" si="39">P40*N40</f>
-        <v>27.035499999999999</v>
+        <f t="shared" ref="Q40" si="46">P40*N40</f>
+        <v>0.12</v>
       </c>
       <c r="R40" s="12"/>
     </row>
-    <row r="41" spans="1:18" ht="48.75" thickBot="1">
+    <row r="41" spans="1:18">
       <c r="A41" s="1"/>
       <c r="B41" s="8">
         <f>ROW(B41) - ROW($B$2)</f>
         <v>39</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>281</v>
+        <v>113</v>
       </c>
       <c r="F41" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="G41" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="H41" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="I41" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="J41" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="K41" s="6" t="s">
         <v>282</v>
-      </c>
-      <c r="G41" s="6" t="s">
-        <v>283</v>
-      </c>
-      <c r="H41" s="6" t="s">
-        <v>284</v>
-      </c>
-      <c r="I41" s="6"/>
-      <c r="J41" s="6" t="s">
-        <v>285</v>
-      </c>
-      <c r="K41" s="6" t="s">
-        <v>237</v>
       </c>
       <c r="L41" s="6">
         <v>1</v>
@@ -3739,87 +3970,653 @@
         <f>L41*5</f>
         <v>5</v>
       </c>
-      <c r="N41" s="18">
-        <v>6</v>
-      </c>
-      <c r="O41" s="27" t="s">
-        <v>279</v>
-      </c>
-      <c r="P41" s="20">
-        <v>1.5250999999999999</v>
+      <c r="N41" s="21" t="s">
+        <v>295</v>
+      </c>
+      <c r="O41" s="20" t="str">
+        <f t="shared" si="45"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P41" s="22" t="s">
+        <v>327</v>
       </c>
       <c r="Q41" s="7">
         <f>P41*N41</f>
-        <v>9.150599999999999</v>
+        <v>0.53</v>
       </c>
       <c r="R41" s="6"/>
     </row>
-    <row r="42" spans="1:18" ht="19.5" thickBot="1">
+    <row r="42" spans="1:18">
       <c r="A42" s="1"/>
-      <c r="B42" s="1"/>
-      <c r="C42" s="1"/>
-      <c r="D42" s="1"/>
-      <c r="E42" s="1"/>
-      <c r="F42" s="1"/>
-      <c r="G42" s="1"/>
-      <c r="H42" s="1"/>
-      <c r="I42" s="1"/>
-      <c r="J42" s="1"/>
-      <c r="K42" s="1"/>
-      <c r="L42" s="1"/>
-      <c r="M42" s="1"/>
-      <c r="N42" s="24" t="s">
+      <c r="B42" s="9">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+      <c r="C42" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D42" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="E42" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="F42" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="G42" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="H42" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="I42" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="J42" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="K42" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="L42" s="12">
+        <v>2</v>
+      </c>
+      <c r="M42" s="12">
+        <f t="shared" ref="M42" si="47">L42*5</f>
+        <v>10</v>
+      </c>
+      <c r="N42" s="12">
+        <v>100</v>
+      </c>
+      <c r="O42" s="20" t="s">
+        <v>294</v>
+      </c>
+      <c r="P42" s="13">
+        <v>1.1000000000000001E-3</v>
+      </c>
+      <c r="Q42" s="13">
+        <f t="shared" ref="Q42" si="48">P42*N42</f>
+        <v>0.11</v>
+      </c>
+      <c r="R42" s="12"/>
+    </row>
+    <row r="43" spans="1:18">
+      <c r="A43" s="1"/>
+      <c r="B43" s="8">
+        <f>ROW(B43) - ROW($B$2)</f>
+        <v>41</v>
+      </c>
+      <c r="C43" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="F43" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="G43" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="H43" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="I43" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="J43" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="K43" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L43" s="6">
         <v>1</v>
       </c>
-      <c r="O42" s="25"/>
-      <c r="P42" s="26"/>
-      <c r="Q42" s="10">
-        <f>SUM(Q3:Q41)</f>
-        <v>83.674700000000001</v>
-      </c>
-      <c r="R42" s="1"/>
-    </row>
-    <row r="43" spans="1:18" ht="19.5" thickBot="1">
-      <c r="A43" s="1"/>
-      <c r="B43" s="1"/>
-      <c r="C43" s="1"/>
-      <c r="D43" s="1"/>
-      <c r="E43" s="1"/>
-      <c r="F43" s="1"/>
-      <c r="G43" s="1"/>
-      <c r="H43" s="1"/>
-      <c r="I43" s="1"/>
-      <c r="J43" s="1"/>
-      <c r="K43" s="1"/>
-      <c r="L43" s="1"/>
-      <c r="M43" s="1"/>
-      <c r="N43" s="24" t="s">
+      <c r="M43" s="6">
+        <f>L43*5</f>
+        <v>5</v>
+      </c>
+      <c r="N43" s="6">
+        <v>100</v>
+      </c>
+      <c r="O43" s="20" t="s">
+        <v>294</v>
+      </c>
+      <c r="P43" s="7">
+        <v>1.1999999999999999E-3</v>
+      </c>
+      <c r="Q43" s="7">
+        <f>P43*N43</f>
+        <v>0.12</v>
+      </c>
+      <c r="R43" s="6"/>
+    </row>
+    <row r="44" spans="1:18">
+      <c r="A44" s="1"/>
+      <c r="B44" s="9">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="C44" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="D44" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="E44" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="F44" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="G44" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="H44" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="I44" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="J44" s="12" t="s">
+        <v>259</v>
+      </c>
+      <c r="K44" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="L44" s="12">
         <v>2</v>
       </c>
-      <c r="O43" s="26"/>
-      <c r="P43" s="26"/>
-      <c r="Q43" s="11">
-        <f>Q42/5</f>
-        <v>16.734940000000002</v>
-      </c>
-      <c r="R43" s="1"/>
-    </row>
-    <row r="55" spans="13:13">
-      <c r="M55" s="16"/>
+      <c r="M44" s="12">
+        <f t="shared" ref="M44" si="49">L44*5</f>
+        <v>10</v>
+      </c>
+      <c r="N44" s="17" t="s">
+        <v>297</v>
+      </c>
+      <c r="O44" s="20" t="str">
+        <f t="shared" ref="O44:O47" si="50">HYPERLINK(M44, "LCSC")</f>
+        <v>LCSC</v>
+      </c>
+      <c r="P44" s="19" t="s">
+        <v>316</v>
+      </c>
+      <c r="Q44" s="13">
+        <f t="shared" ref="Q44" si="51">P44*N44</f>
+        <v>1.5549999999999999</v>
+      </c>
+      <c r="R44" s="12"/>
+    </row>
+    <row r="45" spans="1:18">
+      <c r="A45" s="1"/>
+      <c r="B45" s="8">
+        <f>ROW(B45) - ROW($B$2)</f>
+        <v>43</v>
+      </c>
+      <c r="C45" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="E45" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="F45" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="G45" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="H45" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="I45" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="J45" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="K45" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="L45" s="6">
+        <v>1</v>
+      </c>
+      <c r="M45" s="6">
+        <f>L45*5</f>
+        <v>5</v>
+      </c>
+      <c r="N45" s="21" t="s">
+        <v>305</v>
+      </c>
+      <c r="O45" s="20" t="str">
+        <f t="shared" si="50"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P45" s="22" t="s">
+        <v>317</v>
+      </c>
+      <c r="Q45" s="7">
+        <f>P45*N45</f>
+        <v>6.6879999999999997</v>
+      </c>
+      <c r="R45" s="6"/>
+    </row>
+    <row r="46" spans="1:18">
+      <c r="A46" s="1"/>
+      <c r="B46" s="9">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+      <c r="C46" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D46" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="E46" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="F46" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="G46" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="H46" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="I46" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="J46" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="K46" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="L46" s="12">
+        <v>3</v>
+      </c>
+      <c r="M46" s="12">
+        <f t="shared" ref="M46" si="52">L46*5</f>
+        <v>15</v>
+      </c>
+      <c r="N46" s="17" t="s">
+        <v>318</v>
+      </c>
+      <c r="O46" s="20" t="str">
+        <f t="shared" si="50"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P46" s="19" t="s">
+        <v>319</v>
+      </c>
+      <c r="Q46" s="13">
+        <f t="shared" ref="Q46" si="53">P46*N46</f>
+        <v>10.429500000000001</v>
+      </c>
+      <c r="R46" s="12"/>
+    </row>
+    <row r="47" spans="1:18">
+      <c r="A47" s="1"/>
+      <c r="B47" s="8">
+        <f>ROW(B47) - ROW($B$2)</f>
+        <v>45</v>
+      </c>
+      <c r="C47" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E47" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="F47" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="G47" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="H47" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="I47" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="J47" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="K47" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="L47" s="6">
+        <v>1</v>
+      </c>
+      <c r="M47" s="6">
+        <f>L47*5</f>
+        <v>5</v>
+      </c>
+      <c r="N47" s="21" t="s">
+        <v>305</v>
+      </c>
+      <c r="O47" s="20" t="str">
+        <f t="shared" si="50"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P47" s="22" t="s">
+        <v>320</v>
+      </c>
+      <c r="Q47" s="7">
+        <f>P47*N47</f>
+        <v>27.035499999999999</v>
+      </c>
+      <c r="R47" s="6"/>
+    </row>
+    <row r="48" spans="1:18" ht="24">
+      <c r="A48" s="1"/>
+      <c r="B48" s="9">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+      <c r="C48" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D48" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="E48" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="F48" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="G48" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H48" s="12" t="s">
+        <v>217</v>
+      </c>
+      <c r="I48" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="J48" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="K48" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="L48" s="12">
+        <v>1</v>
+      </c>
+      <c r="M48" s="12">
+        <f t="shared" ref="M48" si="54">L48*5</f>
+        <v>5</v>
+      </c>
+      <c r="N48" s="12">
+        <v>5</v>
+      </c>
+      <c r="O48" s="27" t="s">
+        <v>294</v>
+      </c>
+      <c r="P48" s="13">
+        <v>0.93330000000000002</v>
+      </c>
+      <c r="Q48" s="13">
+        <f t="shared" ref="Q48" si="55">P48*N48</f>
+        <v>4.6665000000000001</v>
+      </c>
+      <c r="R48" s="12"/>
+    </row>
+    <row r="49" spans="1:18">
+      <c r="A49" s="1"/>
+      <c r="B49" s="8">
+        <f>ROW(B49) - ROW($B$2)</f>
+        <v>47</v>
+      </c>
+      <c r="C49" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="E49" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="F49" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="G49" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="H49" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="I49" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="J49" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="K49" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="L49" s="6">
+        <v>1</v>
+      </c>
+      <c r="M49" s="6">
+        <f>L49*5</f>
+        <v>5</v>
+      </c>
+      <c r="N49" s="6">
+        <v>5</v>
+      </c>
+      <c r="O49" s="27" t="s">
+        <v>294</v>
+      </c>
+      <c r="P49" s="7">
+        <v>0.71709999999999996</v>
+      </c>
+      <c r="Q49" s="7">
+        <f>P49*N49</f>
+        <v>3.5854999999999997</v>
+      </c>
+      <c r="R49" s="6"/>
+    </row>
+    <row r="50" spans="1:18" ht="36">
+      <c r="A50" s="1"/>
+      <c r="B50" s="9">
+        <f t="shared" si="0"/>
+        <v>48</v>
+      </c>
+      <c r="C50" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="D50" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="E50" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="F50" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="G50" s="12" t="s">
+        <v>192</v>
+      </c>
+      <c r="H50" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="I50" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="J50" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="K50" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="L50" s="12">
+        <v>1</v>
+      </c>
+      <c r="M50" s="12">
+        <f t="shared" ref="M50:M51" si="56">L50*5</f>
+        <v>5</v>
+      </c>
+      <c r="N50" s="12">
+        <v>10</v>
+      </c>
+      <c r="O50" s="27" t="s">
+        <v>294</v>
+      </c>
+      <c r="P50" s="13">
+        <v>3.8100000000000002E-2</v>
+      </c>
+      <c r="Q50" s="13">
+        <f t="shared" ref="Q50" si="57">P50*N50</f>
+        <v>0.38100000000000001</v>
+      </c>
+      <c r="R50" s="12"/>
+    </row>
+    <row r="51" spans="1:18" ht="45.75" thickBot="1">
+      <c r="A51" s="1"/>
+      <c r="B51" s="9">
+        <f t="shared" si="0"/>
+        <v>49</v>
+      </c>
+      <c r="C51" s="15" t="s">
+        <v>334</v>
+      </c>
+      <c r="D51" s="12" t="s">
+        <v>335</v>
+      </c>
+      <c r="E51" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="F51" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="G51" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="H51" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="I51" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="J51" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="K51" s="12" t="s">
+        <v>330</v>
+      </c>
+      <c r="L51" s="12">
+        <v>1</v>
+      </c>
+      <c r="M51" s="12">
+        <f t="shared" si="56"/>
+        <v>5</v>
+      </c>
+      <c r="N51" s="12">
+        <v>5</v>
+      </c>
+      <c r="O51" s="27" t="s">
+        <v>337</v>
+      </c>
+      <c r="P51" s="13"/>
+      <c r="Q51" s="13"/>
+      <c r="R51" s="31" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="52" spans="1:18" ht="19.5" thickBot="1">
+      <c r="A52" s="1"/>
+      <c r="B52" s="1"/>
+      <c r="C52" s="1"/>
+      <c r="D52" s="1"/>
+      <c r="E52" s="1"/>
+      <c r="F52" s="1"/>
+      <c r="G52" s="1"/>
+      <c r="H52" s="1"/>
+      <c r="I52" s="1"/>
+      <c r="J52" s="1"/>
+      <c r="K52" s="1"/>
+      <c r="L52" s="1"/>
+      <c r="M52" s="1"/>
+      <c r="N52" s="29" t="s">
+        <v>1</v>
+      </c>
+      <c r="O52" s="30"/>
+      <c r="P52" s="30"/>
+      <c r="Q52" s="10">
+        <f>SUM(Q3:Q50)</f>
+        <v>75.009799999999998</v>
+      </c>
+      <c r="R52" s="1"/>
+    </row>
+    <row r="53" spans="1:18" ht="19.5" thickBot="1">
+      <c r="A53" s="1"/>
+      <c r="B53" s="1"/>
+      <c r="C53" s="1"/>
+      <c r="D53" s="1"/>
+      <c r="E53" s="1"/>
+      <c r="F53" s="1"/>
+      <c r="G53" s="1"/>
+      <c r="H53" s="1"/>
+      <c r="I53" s="1"/>
+      <c r="J53" s="1"/>
+      <c r="K53" s="1"/>
+      <c r="L53" s="1"/>
+      <c r="M53" s="1"/>
+      <c r="N53" s="29" t="s">
+        <v>2</v>
+      </c>
+      <c r="O53" s="30"/>
+      <c r="P53" s="30"/>
+      <c r="Q53" s="11">
+        <f>Q52/5</f>
+        <v>15.00196</v>
+      </c>
+      <c r="R53" s="1"/>
+    </row>
+    <row r="65" spans="13:13">
+      <c r="M65" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="K1:R1"/>
-    <mergeCell ref="N42:P42"/>
-    <mergeCell ref="N43:P43"/>
+    <mergeCell ref="N52:P52"/>
+    <mergeCell ref="N53:P53"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="O8" r:id="rId1"/>
-    <hyperlink ref="O3" r:id="rId2"/>
-    <hyperlink ref="E41" r:id="rId3"/>
-    <hyperlink ref="O41" r:id="rId4"/>
+    <hyperlink ref="O3" r:id="rId1"/>
+    <hyperlink ref="O8" r:id="rId2"/>
+    <hyperlink ref="O4" r:id="rId3"/>
+    <hyperlink ref="O10" r:id="rId4"/>
+    <hyperlink ref="O13" r:id="rId5"/>
+    <hyperlink ref="O15" r:id="rId6"/>
+    <hyperlink ref="O16" r:id="rId7"/>
+    <hyperlink ref="O23" r:id="rId8"/>
+    <hyperlink ref="O24" r:id="rId9"/>
+    <hyperlink ref="O27" r:id="rId10"/>
+    <hyperlink ref="O28" r:id="rId11"/>
+    <hyperlink ref="O39" r:id="rId12"/>
+    <hyperlink ref="O42" r:id="rId13"/>
+    <hyperlink ref="O43" r:id="rId14"/>
+    <hyperlink ref="O48" r:id="rId15"/>
+    <hyperlink ref="O49" r:id="rId16"/>
+    <hyperlink ref="O50" r:id="rId17"/>
+    <hyperlink ref="O51" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId19"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
100 Pcs BOM Updated.
</commit_message>
<xml_diff>
--- a/Design-Files/WIFI_BoardV4.0/BOM/BOM-With Price-WIFI_BoardV4.00.xlsx
+++ b/Design-Files/WIFI_BoardV4.0/BOM/BOM-With Price-WIFI_BoardV4.00.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iftikhar Ahmed\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\OliverStanton-WaterMonitor\Design-Files\WIFI_BoardV4.0\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -13,13 +13,14 @@
   </bookViews>
   <sheets>
     <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
+    <sheet name="100 Boards" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1115" uniqueCount="378">
   <si>
     <t>#</t>
   </si>
@@ -927,9 +928,6 @@
     <t>Digikey</t>
   </si>
   <si>
-    <t>0.1317</t>
-  </si>
-  <si>
     <t>0.0018</t>
   </si>
   <si>
@@ -1033,6 +1031,129 @@
   </si>
   <si>
     <t>Eya Display</t>
+  </si>
+  <si>
+    <t>Quantity (100 Boards)</t>
+  </si>
+  <si>
+    <t>MOQ (100 Boards)</t>
+  </si>
+  <si>
+    <t>Unit Cost (100 Boards)</t>
+  </si>
+  <si>
+    <t>Total Cost (100 Boards)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Remarks</t>
+  </si>
+  <si>
+    <t>400</t>
+  </si>
+  <si>
+    <t>0.5718</t>
+  </si>
+  <si>
+    <t>0.0315</t>
+  </si>
+  <si>
+    <t>0.0333</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  </t>
+  </si>
+  <si>
+    <t>200</t>
+  </si>
+  <si>
+    <t>600</t>
+  </si>
+  <si>
+    <t>108</t>
+  </si>
+  <si>
+    <t>0.0017</t>
+  </si>
+  <si>
+    <t>0.0917</t>
+  </si>
+  <si>
+    <t>0.0795</t>
+  </si>
+  <si>
+    <t>0.0031</t>
+  </si>
+  <si>
+    <t>0.0285</t>
+  </si>
+  <si>
+    <t>0.0161</t>
+  </si>
+  <si>
+    <t>0.0069</t>
+  </si>
+  <si>
+    <t>0.0354</t>
+  </si>
+  <si>
+    <t>0.0722</t>
+  </si>
+  <si>
+    <t>0.1368</t>
+  </si>
+  <si>
+    <t>0.0313</t>
+  </si>
+  <si>
+    <t>0.1319</t>
+  </si>
+  <si>
+    <t>0.0799</t>
+  </si>
+  <si>
+    <t>0.2548</t>
+  </si>
+  <si>
+    <t>300</t>
+  </si>
+  <si>
+    <t>0.0430</t>
+  </si>
+  <si>
+    <t>0.0166</t>
+  </si>
+  <si>
+    <t>0.0096</t>
+  </si>
+  <si>
+    <t>0.0220</t>
+  </si>
+  <si>
+    <t>0.0181</t>
+  </si>
+  <si>
+    <t>0.0010</t>
+  </si>
+  <si>
+    <t>0.1034</t>
+  </si>
+  <si>
+    <t>1.1080</t>
+  </si>
+  <si>
+    <t>0.5196</t>
+  </si>
+  <si>
+    <t>3.7058</t>
+  </si>
+  <si>
+    <t>0.5588</t>
+  </si>
+  <si>
+    <t>0.5240</t>
+  </si>
+  <si>
+    <t>0.0297</t>
   </si>
 </sst>
 </file>
@@ -1176,7 +1297,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -1336,6 +1457,19 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1343,7 +1477,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1420,6 +1554,9 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1431,8 +1568,20 @@
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1755,14 +1904,14 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
-      <c r="O1" s="28"/>
-      <c r="P1" s="28"/>
-      <c r="Q1" s="28"/>
-      <c r="R1" s="28"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+      <c r="O1" s="29"/>
+      <c r="P1" s="29"/>
+      <c r="Q1" s="29"/>
+      <c r="R1" s="29"/>
     </row>
     <row r="2" spans="1:18" ht="15.75" thickBot="1">
       <c r="A2" s="1"/>
@@ -1843,7 +1992,7 @@
         <v>194</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J3" s="6" t="s">
         <v>221</v>
@@ -1898,7 +2047,7 @@
         <v>195</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J4" s="12" t="s">
         <v>222</v>
@@ -1953,7 +2102,7 @@
         <v>194</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J5" s="6" t="s">
         <v>223</v>
@@ -2009,7 +2158,7 @@
         <v>194</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J6" s="12" t="s">
         <v>224</v>
@@ -2065,7 +2214,7 @@
         <v>196</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J7" s="6" t="s">
         <v>225</v>
@@ -2121,7 +2270,7 @@
         <v>197</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J8" s="12" t="s">
         <v>226</v>
@@ -2142,12 +2291,12 @@
       <c r="O8" s="20" t="s">
         <v>301</v>
       </c>
-      <c r="P8" s="22" t="s">
-        <v>302</v>
+      <c r="P8" s="22">
+        <v>0.77</v>
       </c>
       <c r="Q8" s="13">
         <f t="shared" ref="Q8" si="7">P8*N8</f>
-        <v>0.79020000000000001</v>
+        <v>4.62</v>
       </c>
       <c r="R8" s="12"/>
     </row>
@@ -2176,7 +2325,7 @@
         <v>194</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J9" s="6" t="s">
         <v>227</v>
@@ -2199,7 +2348,7 @@
         <v>LCSC</v>
       </c>
       <c r="P9" s="19" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="Q9" s="7">
         <f>P9*N9</f>
@@ -2232,7 +2381,7 @@
         <v>195</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J10" s="12" t="s">
         <v>228</v>
@@ -2287,7 +2436,7 @@
         <v>194</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J11" s="6" t="s">
         <v>229</v>
@@ -2310,7 +2459,7 @@
         <v>LCSC</v>
       </c>
       <c r="P11" s="19" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="Q11" s="7">
         <f>P11*N11</f>
@@ -2343,7 +2492,7 @@
         <v>198</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J12" s="12" t="s">
         <v>230</v>
@@ -2359,14 +2508,14 @@
         <v>5</v>
       </c>
       <c r="N12" s="21" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="O12" s="20" t="str">
         <f t="shared" si="10"/>
         <v>LCSC</v>
       </c>
       <c r="P12" s="22" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="Q12" s="13">
         <f t="shared" ref="Q12" si="12">P12*N12</f>
@@ -2399,7 +2548,7 @@
         <v>194</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J13" s="6" t="s">
         <v>231</v>
@@ -2454,13 +2603,13 @@
         <v>199</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J14" s="12" t="s">
         <v>232</v>
       </c>
       <c r="K14" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L14" s="12">
         <v>1</v>
@@ -2477,7 +2626,7 @@
         <v>LCSC</v>
       </c>
       <c r="P14" s="19" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="Q14" s="13">
         <f t="shared" ref="Q14" si="15">P14*N14</f>
@@ -2510,13 +2659,13 @@
         <v>200</v>
       </c>
       <c r="I15" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J15" s="6" t="s">
         <v>330</v>
       </c>
-      <c r="J15" s="6" t="s">
-        <v>331</v>
-      </c>
       <c r="K15" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L15" s="6">
         <v>1</v>
@@ -2565,13 +2714,13 @@
         <v>200</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J16" s="12" t="s">
         <v>233</v>
       </c>
       <c r="K16" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L16" s="12">
         <v>1</v>
@@ -2620,13 +2769,13 @@
         <v>201</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J17" s="6" t="s">
         <v>234</v>
       </c>
       <c r="K17" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L17" s="6">
         <v>6</v>
@@ -2636,14 +2785,14 @@
         <v>30</v>
       </c>
       <c r="N17" s="21" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="O17" s="20" t="str">
         <f t="shared" ref="O17:O19" si="18">HYPERLINK(M17, "LCSC")</f>
         <v>LCSC</v>
       </c>
       <c r="P17" s="22" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="Q17" s="7">
         <f>P17*N17</f>
@@ -2676,13 +2825,13 @@
         <v>202</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J18" s="12" t="s">
         <v>235</v>
       </c>
       <c r="K18" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L18" s="12">
         <v>1</v>
@@ -2699,7 +2848,7 @@
         <v>LCSC</v>
       </c>
       <c r="P18" s="19" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="Q18" s="13">
         <f t="shared" ref="Q18" si="20">P18*N18</f>
@@ -2732,13 +2881,13 @@
         <v>203</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J19" s="6" t="s">
         <v>168</v>
       </c>
       <c r="K19" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L19" s="6">
         <v>1</v>
@@ -2748,14 +2897,14 @@
         <v>5</v>
       </c>
       <c r="N19" s="21" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="O19" s="20" t="str">
         <f t="shared" si="18"/>
         <v>LCSC</v>
       </c>
       <c r="P19" s="22" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="Q19" s="7">
         <f>P19*N19</f>
@@ -2788,13 +2937,13 @@
         <v>204</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J20" s="12" t="s">
         <v>236</v>
       </c>
       <c r="K20" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L20" s="12">
         <v>1</v>
@@ -2804,14 +2953,14 @@
         <v>5</v>
       </c>
       <c r="N20" s="17" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="O20" s="20" t="str">
         <f t="shared" ref="O20:O22" si="22">HYPERLINK(M20, "LCSC")</f>
         <v>LCSC</v>
       </c>
       <c r="P20" s="19" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="Q20" s="13">
         <f t="shared" ref="Q20" si="23">P20*N20</f>
@@ -2844,13 +2993,13 @@
         <v>205</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J21" s="6" t="s">
         <v>237</v>
       </c>
       <c r="K21" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L21" s="6">
         <v>1</v>
@@ -2860,14 +3009,14 @@
         <v>5</v>
       </c>
       <c r="N21" s="21" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="O21" s="20" t="str">
         <f t="shared" si="22"/>
         <v>LCSC</v>
       </c>
       <c r="P21" s="22" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="Q21" s="7">
         <f>P21*N21</f>
@@ -2900,13 +3049,13 @@
         <v>206</v>
       </c>
       <c r="I22" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J22" s="12" t="s">
         <v>238</v>
       </c>
       <c r="K22" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L22" s="12">
         <v>1</v>
@@ -2916,18 +3065,17 @@
         <v>5</v>
       </c>
       <c r="N22" s="17" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="O22" s="20" t="str">
         <f t="shared" si="22"/>
         <v>LCSC</v>
       </c>
       <c r="P22" s="19" t="s">
-        <v>309</v>
-      </c>
-      <c r="Q22" s="13">
-        <f t="shared" ref="Q22" si="25">P22*N22</f>
-        <v>0.85299999999999998</v>
+        <v>308</v>
+      </c>
+      <c r="Q22" s="13" t="s">
+        <v>346</v>
       </c>
       <c r="R22" s="12"/>
     </row>
@@ -2956,13 +3104,13 @@
         <v>207</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J23" s="6" t="s">
         <v>239</v>
       </c>
       <c r="K23" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L23" s="6">
         <v>1</v>
@@ -3011,19 +3159,19 @@
         <v>208</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J24" s="12" t="s">
         <v>240</v>
       </c>
       <c r="K24" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L24" s="12">
         <v>1</v>
       </c>
       <c r="M24" s="12">
-        <f t="shared" ref="M24" si="26">L24*5</f>
+        <f t="shared" ref="M24" si="25">L24*5</f>
         <v>5</v>
       </c>
       <c r="N24" s="12">
@@ -3036,7 +3184,7 @@
         <v>0.3271</v>
       </c>
       <c r="Q24" s="13">
-        <f t="shared" ref="Q24" si="27">P24*N24</f>
+        <f t="shared" ref="Q24" si="26">P24*N24</f>
         <v>1.6355</v>
       </c>
       <c r="R24" s="12"/>
@@ -3063,16 +3211,16 @@
         <v>138</v>
       </c>
       <c r="H25" s="23" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="I25" s="23" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J25" s="23" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="K25" s="23" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L25" s="23">
         <v>5</v>
@@ -3082,19 +3230,19 @@
         <v>25</v>
       </c>
       <c r="N25" s="23" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="O25" s="23" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="P25" s="24" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="Q25" s="24" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="R25" s="25" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="26" spans="1:18" ht="36">
@@ -3122,33 +3270,33 @@
         <v>209</v>
       </c>
       <c r="I26" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J26" s="12" t="s">
         <v>241</v>
       </c>
       <c r="K26" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L26" s="12">
         <v>1</v>
       </c>
       <c r="M26" s="12">
-        <f t="shared" ref="M26" si="28">L26*5</f>
+        <f t="shared" ref="M26" si="27">L26*5</f>
         <v>5</v>
       </c>
       <c r="N26" s="21" t="s">
         <v>297</v>
       </c>
       <c r="O26" s="20" t="str">
-        <f t="shared" ref="O26" si="29">HYPERLINK(M26, "LCSC")</f>
+        <f t="shared" ref="O26" si="28">HYPERLINK(M26, "LCSC")</f>
         <v>LCSC</v>
       </c>
       <c r="P26" s="22" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="Q26" s="13">
-        <f t="shared" ref="Q26" si="30">P26*N26</f>
+        <f t="shared" ref="Q26" si="29">P26*N26</f>
         <v>0.51700000000000002</v>
       </c>
       <c r="R26" s="12"/>
@@ -3178,13 +3326,13 @@
         <v>210</v>
       </c>
       <c r="I27" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J27" s="6" t="s">
         <v>242</v>
       </c>
       <c r="K27" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L27" s="6">
         <v>2</v>
@@ -3233,19 +3381,19 @@
         <v>211</v>
       </c>
       <c r="I28" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J28" s="12" t="s">
         <v>243</v>
       </c>
       <c r="K28" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L28" s="12">
         <v>1</v>
       </c>
       <c r="M28" s="12">
-        <f t="shared" ref="M28" si="31">L28*5</f>
+        <f t="shared" ref="M28" si="30">L28*5</f>
         <v>5</v>
       </c>
       <c r="N28" s="12">
@@ -3258,7 +3406,7 @@
         <v>9.5999999999999992E-3</v>
       </c>
       <c r="Q28" s="13">
-        <f t="shared" ref="Q28" si="32">P28*N28</f>
+        <f t="shared" ref="Q28" si="31">P28*N28</f>
         <v>0.48</v>
       </c>
       <c r="R28" s="12"/>
@@ -3288,7 +3436,7 @@
         <v>194</v>
       </c>
       <c r="I29" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J29" s="6" t="s">
         <v>244</v>
@@ -3307,11 +3455,11 @@
         <v>295</v>
       </c>
       <c r="O29" s="20" t="str">
-        <f t="shared" ref="O29:O38" si="33">HYPERLINK(M29, "LCSC")</f>
+        <f t="shared" ref="O29:O38" si="32">HYPERLINK(M29, "LCSC")</f>
         <v>LCSC</v>
       </c>
       <c r="P29" s="22" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="Q29" s="7">
         <f>P29*N29</f>
@@ -3340,7 +3488,7 @@
       <c r="G30" s="12"/>
       <c r="H30" s="12"/>
       <c r="I30" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J30" s="12" t="s">
         <v>245</v>
@@ -3352,21 +3500,21 @@
         <v>3</v>
       </c>
       <c r="M30" s="12">
-        <f t="shared" ref="M30" si="34">L30*5</f>
+        <f t="shared" ref="M30" si="33">L30*5</f>
         <v>15</v>
       </c>
       <c r="N30" s="17" t="s">
         <v>299</v>
       </c>
       <c r="O30" s="20" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="32"/>
         <v>LCSC</v>
       </c>
       <c r="P30" s="19" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="Q30" s="13">
-        <f t="shared" ref="Q30" si="35">P30*N30</f>
+        <f t="shared" ref="Q30" si="34">P30*N30</f>
         <v>0.57399999999999995</v>
       </c>
       <c r="R30" s="12"/>
@@ -3396,7 +3544,7 @@
         <v>194</v>
       </c>
       <c r="I31" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J31" s="6" t="s">
         <v>246</v>
@@ -3415,11 +3563,11 @@
         <v>295</v>
       </c>
       <c r="O31" s="20" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="32"/>
         <v>LCSC</v>
       </c>
       <c r="P31" s="22" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="Q31" s="7">
         <f>P31*N31</f>
@@ -3452,7 +3600,7 @@
         <v>194</v>
       </c>
       <c r="I32" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J32" s="12" t="s">
         <v>247</v>
@@ -3464,21 +3612,21 @@
         <v>2</v>
       </c>
       <c r="M32" s="12">
-        <f t="shared" ref="M32" si="36">L32*5</f>
+        <f t="shared" ref="M32" si="35">L32*5</f>
         <v>10</v>
       </c>
       <c r="N32" s="17" t="s">
         <v>295</v>
       </c>
       <c r="O32" s="20" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="32"/>
         <v>LCSC</v>
       </c>
       <c r="P32" s="19" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="Q32" s="13">
-        <f t="shared" ref="Q32" si="37">P32*N32</f>
+        <f t="shared" ref="Q32" si="36">P32*N32</f>
         <v>0.12</v>
       </c>
       <c r="R32" s="12"/>
@@ -3508,7 +3656,7 @@
         <v>212</v>
       </c>
       <c r="I33" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J33" s="6" t="s">
         <v>248</v>
@@ -3527,11 +3675,11 @@
         <v>299</v>
       </c>
       <c r="O33" s="20" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="32"/>
         <v>LCSC</v>
       </c>
       <c r="P33" s="22" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="Q33" s="7">
         <f>P33*N33</f>
@@ -3564,7 +3712,7 @@
         <v>194</v>
       </c>
       <c r="I34" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J34" s="12" t="s">
         <v>249</v>
@@ -3576,21 +3724,21 @@
         <v>1</v>
       </c>
       <c r="M34" s="12">
-        <f t="shared" ref="M34" si="38">L34*5</f>
+        <f t="shared" ref="M34" si="37">L34*5</f>
         <v>5</v>
       </c>
       <c r="N34" s="17" t="s">
         <v>295</v>
       </c>
       <c r="O34" s="20" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="32"/>
         <v>LCSC</v>
       </c>
       <c r="P34" s="19" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="Q34" s="13">
-        <f t="shared" ref="Q34" si="39">P34*N34</f>
+        <f t="shared" ref="Q34" si="38">P34*N34</f>
         <v>0.12</v>
       </c>
       <c r="R34" s="12"/>
@@ -3620,7 +3768,7 @@
         <v>194</v>
       </c>
       <c r="I35" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J35" s="6" t="s">
         <v>250</v>
@@ -3639,11 +3787,11 @@
         <v>295</v>
       </c>
       <c r="O35" s="20" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="32"/>
         <v>LCSC</v>
       </c>
       <c r="P35" s="22" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="Q35" s="7">
         <f>P35*N35</f>
@@ -3676,7 +3824,7 @@
         <v>194</v>
       </c>
       <c r="I36" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J36" s="12" t="s">
         <v>251</v>
@@ -3688,21 +3836,21 @@
         <v>1</v>
       </c>
       <c r="M36" s="12">
-        <f t="shared" ref="M36" si="40">L36*5</f>
+        <f t="shared" ref="M36" si="39">L36*5</f>
         <v>5</v>
       </c>
       <c r="N36" s="17" t="s">
         <v>295</v>
       </c>
       <c r="O36" s="20" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="32"/>
         <v>LCSC</v>
       </c>
       <c r="P36" s="19" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="Q36" s="13">
-        <f t="shared" ref="Q36" si="41">P36*N36</f>
+        <f t="shared" ref="Q36" si="40">P36*N36</f>
         <v>0.06</v>
       </c>
       <c r="R36" s="12"/>
@@ -3732,7 +3880,7 @@
         <v>194</v>
       </c>
       <c r="I37" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J37" s="6" t="s">
         <v>252</v>
@@ -3751,11 +3899,11 @@
         <v>295</v>
       </c>
       <c r="O37" s="20" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="32"/>
         <v>LCSC</v>
       </c>
       <c r="P37" s="22" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="Q37" s="7">
         <f>P37*N37</f>
@@ -3788,7 +3936,7 @@
         <v>194</v>
       </c>
       <c r="I38" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J38" s="12" t="s">
         <v>253</v>
@@ -3800,21 +3948,21 @@
         <v>2</v>
       </c>
       <c r="M38" s="12">
-        <f t="shared" ref="M38" si="42">L38*5</f>
+        <f t="shared" ref="M38" si="41">L38*5</f>
         <v>10</v>
       </c>
       <c r="N38" s="21" t="s">
         <v>295</v>
       </c>
       <c r="O38" s="20" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="32"/>
         <v>LCSC</v>
       </c>
       <c r="P38" s="22" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="Q38" s="13">
-        <f t="shared" ref="Q38" si="43">P38*N38</f>
+        <f t="shared" ref="Q38" si="42">P38*N38</f>
         <v>6.9999999999999993E-2</v>
       </c>
       <c r="R38" s="12"/>
@@ -3844,7 +3992,7 @@
         <v>194</v>
       </c>
       <c r="I39" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J39" s="6" t="s">
         <v>254</v>
@@ -3899,7 +4047,7 @@
         <v>194</v>
       </c>
       <c r="I40" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J40" s="12" t="s">
         <v>255</v>
@@ -3911,21 +4059,21 @@
         <v>1</v>
       </c>
       <c r="M40" s="12">
-        <f t="shared" ref="M40" si="44">L40*5</f>
+        <f t="shared" ref="M40" si="43">L40*5</f>
         <v>5</v>
       </c>
       <c r="N40" s="17" t="s">
         <v>295</v>
       </c>
       <c r="O40" s="20" t="str">
-        <f t="shared" ref="O40:O41" si="45">HYPERLINK(M40, "LCSC")</f>
+        <f t="shared" ref="O40:O41" si="44">HYPERLINK(M40, "LCSC")</f>
         <v>LCSC</v>
       </c>
       <c r="P40" s="19" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="Q40" s="13">
-        <f t="shared" ref="Q40" si="46">P40*N40</f>
+        <f t="shared" ref="Q40" si="45">P40*N40</f>
         <v>0.12</v>
       </c>
       <c r="R40" s="12"/>
@@ -3955,7 +4103,7 @@
         <v>194</v>
       </c>
       <c r="I41" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J41" s="6" t="s">
         <v>256</v>
@@ -3974,11 +4122,11 @@
         <v>295</v>
       </c>
       <c r="O41" s="20" t="str">
-        <f t="shared" si="45"/>
+        <f t="shared" si="44"/>
         <v>LCSC</v>
       </c>
       <c r="P41" s="22" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="Q41" s="7">
         <f>P41*N41</f>
@@ -4011,7 +4159,7 @@
         <v>194</v>
       </c>
       <c r="I42" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J42" s="12" t="s">
         <v>257</v>
@@ -4023,7 +4171,7 @@
         <v>2</v>
       </c>
       <c r="M42" s="12">
-        <f t="shared" ref="M42" si="47">L42*5</f>
+        <f t="shared" ref="M42" si="46">L42*5</f>
         <v>10</v>
       </c>
       <c r="N42" s="12">
@@ -4036,7 +4184,7 @@
         <v>1.1000000000000001E-3</v>
       </c>
       <c r="Q42" s="13">
-        <f t="shared" ref="Q42" si="48">P42*N42</f>
+        <f t="shared" ref="Q42" si="47">P42*N42</f>
         <v>0.11</v>
       </c>
       <c r="R42" s="12"/>
@@ -4066,7 +4214,7 @@
         <v>194</v>
       </c>
       <c r="I43" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J43" s="6" t="s">
         <v>258</v>
@@ -4121,33 +4269,33 @@
         <v>213</v>
       </c>
       <c r="I44" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J44" s="12" t="s">
         <v>259</v>
       </c>
       <c r="K44" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L44" s="12">
         <v>2</v>
       </c>
       <c r="M44" s="12">
-        <f t="shared" ref="M44" si="49">L44*5</f>
+        <f t="shared" ref="M44" si="48">L44*5</f>
         <v>10</v>
       </c>
       <c r="N44" s="17" t="s">
         <v>297</v>
       </c>
       <c r="O44" s="20" t="str">
-        <f t="shared" ref="O44:O47" si="50">HYPERLINK(M44, "LCSC")</f>
+        <f t="shared" ref="O44:O47" si="49">HYPERLINK(M44, "LCSC")</f>
         <v>LCSC</v>
       </c>
       <c r="P44" s="19" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="Q44" s="13">
-        <f t="shared" ref="Q44" si="51">P44*N44</f>
+        <f t="shared" ref="Q44" si="50">P44*N44</f>
         <v>1.5549999999999999</v>
       </c>
       <c r="R44" s="12"/>
@@ -4177,13 +4325,13 @@
         <v>214</v>
       </c>
       <c r="I45" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J45" s="6" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="K45" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L45" s="6">
         <v>1</v>
@@ -4193,14 +4341,14 @@
         <v>5</v>
       </c>
       <c r="N45" s="21" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="O45" s="20" t="str">
-        <f t="shared" si="50"/>
+        <f t="shared" si="49"/>
         <v>LCSC</v>
       </c>
       <c r="P45" s="22" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="Q45" s="7">
         <f>P45*N45</f>
@@ -4233,33 +4381,33 @@
         <v>215</v>
       </c>
       <c r="I46" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J46" s="12" t="s">
         <v>260</v>
       </c>
       <c r="K46" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L46" s="12">
         <v>3</v>
       </c>
       <c r="M46" s="12">
-        <f t="shared" ref="M46" si="52">L46*5</f>
+        <f t="shared" ref="M46" si="51">L46*5</f>
         <v>15</v>
       </c>
       <c r="N46" s="17" t="s">
+        <v>317</v>
+      </c>
+      <c r="O46" s="20" t="str">
+        <f t="shared" si="49"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P46" s="19" t="s">
         <v>318</v>
       </c>
-      <c r="O46" s="20" t="str">
-        <f t="shared" si="50"/>
-        <v>LCSC</v>
-      </c>
-      <c r="P46" s="19" t="s">
-        <v>319</v>
-      </c>
       <c r="Q46" s="13">
-        <f t="shared" ref="Q46" si="53">P46*N46</f>
+        <f t="shared" ref="Q46" si="52">P46*N46</f>
         <v>10.429500000000001</v>
       </c>
       <c r="R46" s="12"/>
@@ -4289,13 +4437,13 @@
         <v>216</v>
       </c>
       <c r="I47" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J47" s="6" t="s">
         <v>261</v>
       </c>
       <c r="K47" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L47" s="6">
         <v>1</v>
@@ -4305,14 +4453,14 @@
         <v>5</v>
       </c>
       <c r="N47" s="21" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="O47" s="20" t="str">
-        <f t="shared" si="50"/>
+        <f t="shared" si="49"/>
         <v>LCSC</v>
       </c>
       <c r="P47" s="22" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="Q47" s="7">
         <f>P47*N47</f>
@@ -4345,19 +4493,19 @@
         <v>217</v>
       </c>
       <c r="I48" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J48" s="12" t="s">
         <v>262</v>
       </c>
       <c r="K48" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L48" s="12">
         <v>1</v>
       </c>
       <c r="M48" s="12">
-        <f t="shared" ref="M48" si="54">L48*5</f>
+        <f t="shared" ref="M48" si="53">L48*5</f>
         <v>5</v>
       </c>
       <c r="N48" s="12">
@@ -4370,7 +4518,7 @@
         <v>0.93330000000000002</v>
       </c>
       <c r="Q48" s="13">
-        <f t="shared" ref="Q48" si="55">P48*N48</f>
+        <f t="shared" ref="Q48" si="54">P48*N48</f>
         <v>4.6665000000000001</v>
       </c>
       <c r="R48" s="12"/>
@@ -4400,13 +4548,13 @@
         <v>218</v>
       </c>
       <c r="I49" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J49" s="6" t="s">
         <v>263</v>
       </c>
       <c r="K49" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L49" s="6">
         <v>1</v>
@@ -4455,19 +4603,19 @@
         <v>219</v>
       </c>
       <c r="I50" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J50" s="12" t="s">
         <v>264</v>
       </c>
       <c r="K50" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L50" s="12">
         <v>1</v>
       </c>
       <c r="M50" s="12">
-        <f t="shared" ref="M50:M51" si="56">L50*5</f>
+        <f t="shared" ref="M50:M51" si="55">L50*5</f>
         <v>5</v>
       </c>
       <c r="N50" s="12">
@@ -4480,7 +4628,7 @@
         <v>3.8100000000000002E-2</v>
       </c>
       <c r="Q50" s="13">
-        <f t="shared" ref="Q50" si="57">P50*N50</f>
+        <f t="shared" ref="Q50" si="56">P50*N50</f>
         <v>0.38100000000000001</v>
       </c>
       <c r="R50" s="12"/>
@@ -4492,49 +4640,49 @@
         <v>49</v>
       </c>
       <c r="C51" s="15" t="s">
+        <v>333</v>
+      </c>
+      <c r="D51" s="12" t="s">
         <v>334</v>
       </c>
-      <c r="D51" s="12" t="s">
-        <v>335</v>
-      </c>
       <c r="E51" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F51" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="G51" s="12" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="H51" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="I51" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J51" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="K51" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L51" s="12">
         <v>1</v>
       </c>
       <c r="M51" s="12">
-        <f t="shared" si="56"/>
+        <f t="shared" si="55"/>
         <v>5</v>
       </c>
       <c r="N51" s="12">
         <v>5</v>
       </c>
       <c r="O51" s="27" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="P51" s="13"/>
       <c r="Q51" s="13"/>
-      <c r="R51" s="31" t="s">
-        <v>336</v>
+      <c r="R51" s="28" t="s">
+        <v>335</v>
       </c>
     </row>
     <row r="52" spans="1:18" ht="19.5" thickBot="1">
@@ -4551,14 +4699,14 @@
       <c r="K52" s="1"/>
       <c r="L52" s="1"/>
       <c r="M52" s="1"/>
-      <c r="N52" s="29" t="s">
+      <c r="N52" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="O52" s="30"/>
-      <c r="P52" s="30"/>
+      <c r="O52" s="31"/>
+      <c r="P52" s="31"/>
       <c r="Q52" s="10">
         <f>SUM(Q3:Q50)</f>
-        <v>75.009799999999998</v>
+        <v>77.986599999999996</v>
       </c>
       <c r="R52" s="1"/>
     </row>
@@ -4576,14 +4724,14 @@
       <c r="K53" s="1"/>
       <c r="L53" s="1"/>
       <c r="M53" s="1"/>
-      <c r="N53" s="29" t="s">
+      <c r="N53" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="O53" s="30"/>
-      <c r="P53" s="30"/>
+      <c r="O53" s="31"/>
+      <c r="P53" s="31"/>
       <c r="Q53" s="11">
         <f>Q52/5</f>
-        <v>15.00196</v>
+        <v>15.59732</v>
       </c>
       <c r="R53" s="1"/>
     </row>
@@ -4619,4 +4767,2900 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId19"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:R53"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.85546875" customWidth="1"/>
+    <col min="4" max="4" width="21.42578125" customWidth="1"/>
+    <col min="5" max="5" width="27.85546875" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20" customWidth="1"/>
+    <col min="14" max="14" width="17.28515625" customWidth="1"/>
+    <col min="15" max="15" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="19.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" ht="15.75" thickBot="1">
+      <c r="A1" s="1"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+      <c r="O1" s="29"/>
+      <c r="P1" s="29"/>
+      <c r="Q1" s="29"/>
+      <c r="R1" s="29"/>
+    </row>
+    <row r="2" spans="1:18" ht="15.75" thickBot="1">
+      <c r="A2" s="1"/>
+      <c r="B2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>337</v>
+      </c>
+      <c r="N2" s="35" t="s">
+        <v>338</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>290</v>
+      </c>
+      <c r="P2" s="36" t="s">
+        <v>339</v>
+      </c>
+      <c r="Q2" s="5" t="s">
+        <v>340</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" s="33" customFormat="1" ht="15.75" thickBot="1">
+      <c r="A3" s="32"/>
+      <c r="B3" s="8">
+        <f>ROW(B3) - ROW($B$2)</f>
+        <v>1</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="L3" s="6">
+        <v>2</v>
+      </c>
+      <c r="M3" s="6">
+        <f>L3*100</f>
+        <v>200</v>
+      </c>
+      <c r="N3" s="17">
+        <v>100</v>
+      </c>
+      <c r="O3" s="18" t="s">
+        <v>294</v>
+      </c>
+      <c r="P3" s="19">
+        <v>1.1999999999999999E-3</v>
+      </c>
+      <c r="Q3" s="7">
+        <f>P3*N3</f>
+        <v>0.12</v>
+      </c>
+      <c r="R3" s="6"/>
+    </row>
+    <row r="4" spans="1:18" s="33" customFormat="1">
+      <c r="A4" s="32"/>
+      <c r="B4" s="9">
+        <f t="shared" ref="B4:B51" si="0">ROW(B4) - ROW($B$2)</f>
+        <v>2</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J4" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="K4" s="12" t="s">
+        <v>266</v>
+      </c>
+      <c r="L4" s="12">
+        <v>1</v>
+      </c>
+      <c r="M4" s="6">
+        <f t="shared" ref="M4:M51" si="1">L4*100</f>
+        <v>100</v>
+      </c>
+      <c r="N4" s="12" t="s">
+        <v>295</v>
+      </c>
+      <c r="O4" s="18" t="s">
+        <v>294</v>
+      </c>
+      <c r="P4" s="13" t="s">
+        <v>343</v>
+      </c>
+      <c r="Q4" s="13">
+        <f t="shared" ref="Q4" si="2">P4*N4</f>
+        <v>57.18</v>
+      </c>
+      <c r="R4" s="12"/>
+    </row>
+    <row r="5" spans="1:18" s="33" customFormat="1">
+      <c r="A5" s="32"/>
+      <c r="B5" s="8">
+        <f>ROW(B5) - ROW($B$2)</f>
+        <v>3</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="L5" s="6">
+        <v>4</v>
+      </c>
+      <c r="M5" s="6">
+        <f t="shared" si="1"/>
+        <v>400</v>
+      </c>
+      <c r="N5" s="17" t="s">
+        <v>342</v>
+      </c>
+      <c r="O5" s="34" t="str">
+        <f t="shared" ref="O5:O9" si="3">HYPERLINK(M5, "LCSC")</f>
+        <v>LCSC</v>
+      </c>
+      <c r="P5" s="19" t="s">
+        <v>296</v>
+      </c>
+      <c r="Q5" s="7">
+        <f>P5*N5</f>
+        <v>0.8</v>
+      </c>
+      <c r="R5" s="6"/>
+    </row>
+    <row r="6" spans="1:18" s="33" customFormat="1">
+      <c r="A6" s="32"/>
+      <c r="B6" s="9">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J6" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="K6" s="12" t="s">
+        <v>268</v>
+      </c>
+      <c r="L6" s="12">
+        <v>1</v>
+      </c>
+      <c r="M6" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N6" s="21" t="s">
+        <v>295</v>
+      </c>
+      <c r="O6" s="34" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P6" s="22" t="s">
+        <v>344</v>
+      </c>
+      <c r="Q6" s="13">
+        <f t="shared" ref="Q6" si="4">P6*N6</f>
+        <v>3.15</v>
+      </c>
+      <c r="R6" s="12"/>
+    </row>
+    <row r="7" spans="1:18" s="33" customFormat="1">
+      <c r="A7" s="32"/>
+      <c r="B7" s="8">
+        <f>ROW(B7) - ROW($B$2)</f>
+        <v>5</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="L7" s="6">
+        <v>1</v>
+      </c>
+      <c r="M7" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N7" s="17" t="s">
+        <v>295</v>
+      </c>
+      <c r="O7" s="34" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P7" s="19" t="s">
+        <v>345</v>
+      </c>
+      <c r="Q7" s="7">
+        <f>P7*N7</f>
+        <v>3.3300000000000005</v>
+      </c>
+      <c r="R7" s="6"/>
+    </row>
+    <row r="8" spans="1:18" s="33" customFormat="1" ht="24">
+      <c r="A8" s="32"/>
+      <c r="B8" s="9">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>157</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J8" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="K8" s="12" t="s">
+        <v>268</v>
+      </c>
+      <c r="L8" s="12">
+        <v>1</v>
+      </c>
+      <c r="M8" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N8" s="21">
+        <v>100</v>
+      </c>
+      <c r="O8" s="34" t="s">
+        <v>301</v>
+      </c>
+      <c r="P8" s="22">
+        <v>0.33639999999999998</v>
+      </c>
+      <c r="Q8" s="13">
+        <f t="shared" ref="Q8" si="5">P8*N8</f>
+        <v>33.64</v>
+      </c>
+      <c r="R8" s="12"/>
+    </row>
+    <row r="9" spans="1:18" s="33" customFormat="1">
+      <c r="A9" s="32"/>
+      <c r="B9" s="8">
+        <f>ROW(B9) - ROW($B$2)</f>
+        <v>7</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="L9" s="6">
+        <v>2</v>
+      </c>
+      <c r="M9" s="6">
+        <f t="shared" si="1"/>
+        <v>200</v>
+      </c>
+      <c r="N9" s="17" t="s">
+        <v>347</v>
+      </c>
+      <c r="O9" s="34" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P9" s="19" t="s">
+        <v>350</v>
+      </c>
+      <c r="Q9" s="7">
+        <f>P9*N9</f>
+        <v>0.33999999999999997</v>
+      </c>
+      <c r="R9" s="6"/>
+    </row>
+    <row r="10" spans="1:18" s="33" customFormat="1">
+      <c r="A10" s="32"/>
+      <c r="B10" s="9">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J10" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="K10" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="L10" s="12">
+        <v>1</v>
+      </c>
+      <c r="M10" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N10" s="12" t="s">
+        <v>295</v>
+      </c>
+      <c r="O10" s="34" t="s">
+        <v>294</v>
+      </c>
+      <c r="P10" s="13" t="s">
+        <v>351</v>
+      </c>
+      <c r="Q10" s="13">
+        <f t="shared" ref="Q10" si="6">P10*N10</f>
+        <v>9.17</v>
+      </c>
+      <c r="R10" s="12"/>
+    </row>
+    <row r="11" spans="1:18" s="33" customFormat="1">
+      <c r="A11" s="32"/>
+      <c r="B11" s="8">
+        <f>ROW(B11) - ROW($B$2)</f>
+        <v>9</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="L11" s="6">
+        <v>1</v>
+      </c>
+      <c r="M11" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N11" s="17" t="s">
+        <v>295</v>
+      </c>
+      <c r="O11" s="34" t="str">
+        <f t="shared" ref="O11:O12" si="7">HYPERLINK(M11, "LCSC")</f>
+        <v>LCSC</v>
+      </c>
+      <c r="P11" s="19" t="s">
+        <v>303</v>
+      </c>
+      <c r="Q11" s="7">
+        <f>P11*N11</f>
+        <v>0.33999999999999997</v>
+      </c>
+      <c r="R11" s="6"/>
+    </row>
+    <row r="12" spans="1:18" s="33" customFormat="1">
+      <c r="A12" s="32"/>
+      <c r="B12" s="9">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J12" s="12" t="s">
+        <v>230</v>
+      </c>
+      <c r="K12" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="L12" s="12">
+        <v>1</v>
+      </c>
+      <c r="M12" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N12" s="21" t="s">
+        <v>295</v>
+      </c>
+      <c r="O12" s="34" t="str">
+        <f t="shared" si="7"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P12" s="22" t="s">
+        <v>352</v>
+      </c>
+      <c r="Q12" s="13">
+        <f t="shared" ref="Q12" si="8">P12*N12</f>
+        <v>7.95</v>
+      </c>
+      <c r="R12" s="12"/>
+    </row>
+    <row r="13" spans="1:18" s="33" customFormat="1">
+      <c r="A13" s="32"/>
+      <c r="B13" s="8">
+        <f>ROW(B13) - ROW($B$2)</f>
+        <v>11</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="L13" s="6">
+        <v>1</v>
+      </c>
+      <c r="M13" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N13" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="O13" s="26" t="s">
+        <v>294</v>
+      </c>
+      <c r="P13" s="7" t="s">
+        <v>353</v>
+      </c>
+      <c r="Q13" s="7">
+        <f>P13*N13</f>
+        <v>0.31</v>
+      </c>
+      <c r="R13" s="6"/>
+    </row>
+    <row r="14" spans="1:18" s="33" customFormat="1" ht="36">
+      <c r="A14" s="32"/>
+      <c r="B14" s="9">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>128</v>
+      </c>
+      <c r="G14" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="H14" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J14" s="12" t="s">
+        <v>232</v>
+      </c>
+      <c r="K14" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="L14" s="12">
+        <v>1</v>
+      </c>
+      <c r="M14" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N14" s="17" t="s">
+        <v>295</v>
+      </c>
+      <c r="O14" s="34" t="str">
+        <f t="shared" ref="O14" si="9">HYPERLINK(M14, "LCSC")</f>
+        <v>LCSC</v>
+      </c>
+      <c r="P14" s="19" t="s">
+        <v>314</v>
+      </c>
+      <c r="Q14" s="13">
+        <f t="shared" ref="Q14" si="10">P14*N14</f>
+        <v>2.1</v>
+      </c>
+      <c r="R14" s="12"/>
+    </row>
+    <row r="15" spans="1:18" s="33" customFormat="1">
+      <c r="A15" s="32"/>
+      <c r="B15" s="8">
+        <f>ROW(B15) - ROW($B$2)</f>
+        <v>13</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="K15" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="L15" s="6">
+        <v>1</v>
+      </c>
+      <c r="M15" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N15" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="O15" s="26" t="s">
+        <v>294</v>
+      </c>
+      <c r="P15" s="7" t="s">
+        <v>354</v>
+      </c>
+      <c r="Q15" s="7">
+        <f>P15*N15</f>
+        <v>2.85</v>
+      </c>
+      <c r="R15" s="6"/>
+    </row>
+    <row r="16" spans="1:18" s="33" customFormat="1" ht="24">
+      <c r="A16" s="32"/>
+      <c r="B16" s="9">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="G16" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="H16" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J16" s="12" t="s">
+        <v>233</v>
+      </c>
+      <c r="K16" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="L16" s="12">
+        <v>1</v>
+      </c>
+      <c r="M16" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N16" s="12" t="s">
+        <v>295</v>
+      </c>
+      <c r="O16" s="27" t="s">
+        <v>294</v>
+      </c>
+      <c r="P16" s="13" t="s">
+        <v>355</v>
+      </c>
+      <c r="Q16" s="13">
+        <f t="shared" ref="Q16" si="11">P16*N16</f>
+        <v>1.6099999999999999</v>
+      </c>
+      <c r="R16" s="12"/>
+    </row>
+    <row r="17" spans="1:18" s="33" customFormat="1" ht="25.5">
+      <c r="A17" s="32"/>
+      <c r="B17" s="8">
+        <f>ROW(B17) - ROW($B$2)</f>
+        <v>15</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="K17" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="L17" s="6">
+        <v>6</v>
+      </c>
+      <c r="M17" s="6">
+        <f t="shared" si="1"/>
+        <v>600</v>
+      </c>
+      <c r="N17" s="21" t="s">
+        <v>348</v>
+      </c>
+      <c r="O17" s="34" t="str">
+        <f t="shared" ref="O17:O22" si="12">HYPERLINK(M17, "LCSC")</f>
+        <v>LCSC</v>
+      </c>
+      <c r="P17" s="22" t="s">
+        <v>356</v>
+      </c>
+      <c r="Q17" s="7">
+        <f>P17*N17</f>
+        <v>4.1399999999999997</v>
+      </c>
+      <c r="R17" s="6"/>
+    </row>
+    <row r="18" spans="1:18" s="33" customFormat="1" ht="36">
+      <c r="A18" s="32"/>
+      <c r="B18" s="9">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="G18" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="H18" s="12" t="s">
+        <v>202</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J18" s="12" t="s">
+        <v>235</v>
+      </c>
+      <c r="K18" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="L18" s="12">
+        <v>1</v>
+      </c>
+      <c r="M18" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N18" s="17" t="s">
+        <v>295</v>
+      </c>
+      <c r="O18" s="34" t="str">
+        <f t="shared" si="12"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P18" s="19" t="s">
+        <v>357</v>
+      </c>
+      <c r="Q18" s="13">
+        <f t="shared" ref="Q18" si="13">P18*N18</f>
+        <v>3.54</v>
+      </c>
+      <c r="R18" s="12"/>
+    </row>
+    <row r="19" spans="1:18" s="33" customFormat="1" ht="36">
+      <c r="A19" s="32"/>
+      <c r="B19" s="8">
+        <f>ROW(B19) - ROW($B$2)</f>
+        <v>17</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="K19" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="L19" s="6">
+        <v>1</v>
+      </c>
+      <c r="M19" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N19" s="21" t="s">
+        <v>349</v>
+      </c>
+      <c r="O19" s="34" t="str">
+        <f t="shared" si="12"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P19" s="22" t="s">
+        <v>358</v>
+      </c>
+      <c r="Q19" s="7">
+        <f>P19*N19</f>
+        <v>7.7976000000000001</v>
+      </c>
+      <c r="R19" s="6"/>
+    </row>
+    <row r="20" spans="1:18" s="33" customFormat="1" ht="24">
+      <c r="A20" s="32"/>
+      <c r="B20" s="9">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="G20" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="H20" s="12" t="s">
+        <v>204</v>
+      </c>
+      <c r="I20" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J20" s="12" t="s">
+        <v>236</v>
+      </c>
+      <c r="K20" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="L20" s="12">
+        <v>1</v>
+      </c>
+      <c r="M20" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N20" s="17" t="s">
+        <v>295</v>
+      </c>
+      <c r="O20" s="34" t="str">
+        <f t="shared" si="12"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P20" s="19" t="s">
+        <v>359</v>
+      </c>
+      <c r="Q20" s="13">
+        <f t="shared" ref="Q20" si="14">P20*N20</f>
+        <v>13.68</v>
+      </c>
+      <c r="R20" s="12"/>
+    </row>
+    <row r="21" spans="1:18" s="33" customFormat="1" ht="48">
+      <c r="A21" s="32"/>
+      <c r="B21" s="8">
+        <f>ROW(B21) - ROW($B$2)</f>
+        <v>19</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J21" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="K21" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="L21" s="6">
+        <v>1</v>
+      </c>
+      <c r="M21" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N21" s="21" t="s">
+        <v>295</v>
+      </c>
+      <c r="O21" s="34" t="str">
+        <f t="shared" si="12"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P21" s="22" t="s">
+        <v>360</v>
+      </c>
+      <c r="Q21" s="7">
+        <f>P21*N21</f>
+        <v>3.1300000000000003</v>
+      </c>
+      <c r="R21" s="6"/>
+    </row>
+    <row r="22" spans="1:18" s="33" customFormat="1" ht="60">
+      <c r="A22" s="32"/>
+      <c r="B22" s="9">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="G22" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="H22" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J22" s="12" t="s">
+        <v>238</v>
+      </c>
+      <c r="K22" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="L22" s="12">
+        <v>1</v>
+      </c>
+      <c r="M22" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N22" s="17" t="s">
+        <v>295</v>
+      </c>
+      <c r="O22" s="34" t="str">
+        <f t="shared" si="12"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P22" s="19" t="s">
+        <v>361</v>
+      </c>
+      <c r="Q22" s="13">
+        <f t="shared" ref="Q22" si="15">P22*N22</f>
+        <v>13.19</v>
+      </c>
+      <c r="R22" s="12"/>
+    </row>
+    <row r="23" spans="1:18" s="33" customFormat="1" ht="24">
+      <c r="A23" s="32"/>
+      <c r="B23" s="8">
+        <f>ROW(B23) - ROW($B$2)</f>
+        <v>21</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="I23" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J23" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="K23" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="L23" s="6">
+        <v>1</v>
+      </c>
+      <c r="M23" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N23" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="O23" s="26" t="s">
+        <v>294</v>
+      </c>
+      <c r="P23" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="Q23" s="7">
+        <f>P23*N23</f>
+        <v>7.99</v>
+      </c>
+      <c r="R23" s="6"/>
+    </row>
+    <row r="24" spans="1:18" s="33" customFormat="1" ht="36">
+      <c r="A24" s="32"/>
+      <c r="B24" s="9">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="C24" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="F24" s="12" t="s">
+        <v>137</v>
+      </c>
+      <c r="G24" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="H24" s="12" t="s">
+        <v>208</v>
+      </c>
+      <c r="I24" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="J24" s="12" t="s">
+        <v>240</v>
+      </c>
+      <c r="K24" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="L24" s="12">
+        <v>1</v>
+      </c>
+      <c r="M24" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N24" s="12" t="s">
+        <v>295</v>
+      </c>
+      <c r="O24" s="27" t="s">
+        <v>294</v>
+      </c>
+      <c r="P24" s="13" t="s">
+        <v>363</v>
+      </c>
+      <c r="Q24" s="13">
+        <f t="shared" ref="Q24" si="16">P24*N24</f>
+        <v>25.480000000000004</v>
+      </c>
+      <c r="R24" s="12"/>
+    </row>
+    <row r="25" spans="1:18" s="33" customFormat="1" ht="30">
+      <c r="A25" s="32"/>
+      <c r="B25" s="8">
+        <f>ROW(B25) - ROW($B$2)</f>
+        <v>23</v>
+      </c>
+      <c r="C25" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="E25" s="23" t="s">
+        <v>97</v>
+      </c>
+      <c r="F25" s="23" t="s">
+        <v>138</v>
+      </c>
+      <c r="G25" s="23" t="s">
+        <v>138</v>
+      </c>
+      <c r="H25" s="23" t="s">
+        <v>329</v>
+      </c>
+      <c r="I25" s="23" t="s">
+        <v>329</v>
+      </c>
+      <c r="J25" s="23" t="s">
+        <v>329</v>
+      </c>
+      <c r="K25" s="23" t="s">
+        <v>329</v>
+      </c>
+      <c r="L25" s="23">
+        <v>5</v>
+      </c>
+      <c r="M25" s="6">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N25" s="23" t="s">
+        <v>329</v>
+      </c>
+      <c r="O25" s="23" t="s">
+        <v>329</v>
+      </c>
+      <c r="P25" s="24" t="s">
+        <v>329</v>
+      </c>
+      <c r="Q25" s="24" t="s">
+        <v>329</v>
+      </c>
+      <c r="R25" s="25" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" s="33" customFormat="1" ht="36">
+      <c r="A26" s="32"/>
+      <c r="B26" s="9">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="E26" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="F26" s="12" t="s">
+        <v>139</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="H26" s="12" t="s">
+        <v>209</v>
+      </c>
+      <c r="I26" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J26" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="K26" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="L26" s="12">
+        <v>1</v>
+      </c>
+      <c r="M26" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N26" s="21" t="s">
+        <v>295</v>
+      </c>
+      <c r="O26" s="34" t="str">
+        <f t="shared" ref="O26" si="17">HYPERLINK(M26, "LCSC")</f>
+        <v>LCSC</v>
+      </c>
+      <c r="P26" s="22" t="s">
+        <v>365</v>
+      </c>
+      <c r="Q26" s="13">
+        <f t="shared" ref="Q26" si="18">P26*N26</f>
+        <v>4.3</v>
+      </c>
+      <c r="R26" s="12"/>
+    </row>
+    <row r="27" spans="1:18" s="33" customFormat="1" ht="36">
+      <c r="A27" s="32"/>
+      <c r="B27" s="8">
+        <f>ROW(B27) - ROW($B$2)</f>
+        <v>25</v>
+      </c>
+      <c r="C27" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="I27" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J27" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="K27" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="L27" s="6">
+        <v>2</v>
+      </c>
+      <c r="M27" s="6">
+        <f t="shared" si="1"/>
+        <v>200</v>
+      </c>
+      <c r="N27" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="O27" s="26" t="s">
+        <v>294</v>
+      </c>
+      <c r="P27" s="7" t="s">
+        <v>366</v>
+      </c>
+      <c r="Q27" s="7">
+        <f>P27*N27</f>
+        <v>3.32</v>
+      </c>
+      <c r="R27" s="6"/>
+    </row>
+    <row r="28" spans="1:18" s="33" customFormat="1" ht="24">
+      <c r="A28" s="32"/>
+      <c r="B28" s="9">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="E28" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="F28" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="G28" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="H28" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="I28" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J28" s="12" t="s">
+        <v>243</v>
+      </c>
+      <c r="K28" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="L28" s="12">
+        <v>1</v>
+      </c>
+      <c r="M28" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N28" s="12" t="s">
+        <v>295</v>
+      </c>
+      <c r="O28" s="26" t="s">
+        <v>294</v>
+      </c>
+      <c r="P28" s="13" t="s">
+        <v>367</v>
+      </c>
+      <c r="Q28" s="13">
+        <f t="shared" ref="Q28" si="19">P28*N28</f>
+        <v>0.96</v>
+      </c>
+      <c r="R28" s="12"/>
+    </row>
+    <row r="29" spans="1:18" s="33" customFormat="1">
+      <c r="A29" s="32"/>
+      <c r="B29" s="8">
+        <f>ROW(B29) - ROW($B$2)</f>
+        <v>27</v>
+      </c>
+      <c r="C29" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="I29" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J29" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="K29" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="L29" s="6">
+        <v>4</v>
+      </c>
+      <c r="M29" s="6">
+        <f t="shared" si="1"/>
+        <v>400</v>
+      </c>
+      <c r="N29" s="21" t="s">
+        <v>342</v>
+      </c>
+      <c r="O29" s="34" t="str">
+        <f t="shared" ref="O29:O38" si="20">HYPERLINK(M29, "LCSC")</f>
+        <v>LCSC</v>
+      </c>
+      <c r="P29" s="22" t="s">
+        <v>320</v>
+      </c>
+      <c r="Q29" s="7">
+        <f>P29*N29</f>
+        <v>0.24</v>
+      </c>
+      <c r="R29" s="6"/>
+    </row>
+    <row r="30" spans="1:18" s="33" customFormat="1">
+      <c r="A30" s="32"/>
+      <c r="B30" s="9">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="F30" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="G30" s="12"/>
+      <c r="H30" s="12"/>
+      <c r="I30" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J30" s="12" t="s">
+        <v>245</v>
+      </c>
+      <c r="K30" s="12" t="s">
+        <v>272</v>
+      </c>
+      <c r="L30" s="12">
+        <v>3</v>
+      </c>
+      <c r="M30" s="6">
+        <f t="shared" si="1"/>
+        <v>300</v>
+      </c>
+      <c r="N30" s="17" t="s">
+        <v>364</v>
+      </c>
+      <c r="O30" s="34" t="str">
+        <f t="shared" si="20"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P30" s="19" t="s">
+        <v>368</v>
+      </c>
+      <c r="Q30" s="13">
+        <f t="shared" ref="Q30" si="21">P30*N30</f>
+        <v>6.6</v>
+      </c>
+      <c r="R30" s="12"/>
+    </row>
+    <row r="31" spans="1:18" s="33" customFormat="1">
+      <c r="A31" s="32"/>
+      <c r="B31" s="8">
+        <f>ROW(B31) - ROW($B$2)</f>
+        <v>29</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="I31" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J31" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="K31" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="L31" s="6">
+        <v>2</v>
+      </c>
+      <c r="M31" s="6">
+        <f t="shared" si="1"/>
+        <v>200</v>
+      </c>
+      <c r="N31" s="21" t="s">
+        <v>347</v>
+      </c>
+      <c r="O31" s="34" t="str">
+        <f t="shared" si="20"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P31" s="22" t="s">
+        <v>322</v>
+      </c>
+      <c r="Q31" s="7">
+        <f>P31*N31</f>
+        <v>0.22</v>
+      </c>
+      <c r="R31" s="6"/>
+    </row>
+    <row r="32" spans="1:18" s="33" customFormat="1">
+      <c r="A32" s="32"/>
+      <c r="B32" s="9">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="C32" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D32" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="E32" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="F32" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="G32" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="H32" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="I32" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J32" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="K32" s="12" t="s">
+        <v>274</v>
+      </c>
+      <c r="L32" s="12">
+        <v>2</v>
+      </c>
+      <c r="M32" s="6">
+        <f t="shared" si="1"/>
+        <v>200</v>
+      </c>
+      <c r="N32" s="17" t="s">
+        <v>347</v>
+      </c>
+      <c r="O32" s="34" t="str">
+        <f t="shared" si="20"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P32" s="19" t="s">
+        <v>323</v>
+      </c>
+      <c r="Q32" s="13">
+        <f t="shared" ref="Q32" si="22">P32*N32</f>
+        <v>0.24</v>
+      </c>
+      <c r="R32" s="12"/>
+    </row>
+    <row r="33" spans="1:18" s="33" customFormat="1">
+      <c r="A33" s="32"/>
+      <c r="B33" s="8">
+        <f>ROW(B33) - ROW($B$2)</f>
+        <v>31</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="I33" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J33" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="K33" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L33" s="6">
+        <v>4</v>
+      </c>
+      <c r="M33" s="6">
+        <f t="shared" si="1"/>
+        <v>400</v>
+      </c>
+      <c r="N33" s="21" t="s">
+        <v>342</v>
+      </c>
+      <c r="O33" s="34" t="str">
+        <f t="shared" si="20"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P33" s="22" t="s">
+        <v>369</v>
+      </c>
+      <c r="Q33" s="7">
+        <f>P33*N33</f>
+        <v>7.24</v>
+      </c>
+      <c r="R33" s="6"/>
+    </row>
+    <row r="34" spans="1:18" s="33" customFormat="1">
+      <c r="A34" s="32"/>
+      <c r="B34" s="9">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+      <c r="C34" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D34" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="E34" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="F34" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="G34" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="H34" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="I34" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J34" s="12" t="s">
+        <v>249</v>
+      </c>
+      <c r="K34" s="12" t="s">
+        <v>276</v>
+      </c>
+      <c r="L34" s="12">
+        <v>1</v>
+      </c>
+      <c r="M34" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N34" s="17" t="s">
+        <v>295</v>
+      </c>
+      <c r="O34" s="34" t="str">
+        <f t="shared" si="20"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P34" s="19" t="s">
+        <v>323</v>
+      </c>
+      <c r="Q34" s="13">
+        <f t="shared" ref="Q34" si="23">P34*N34</f>
+        <v>0.12</v>
+      </c>
+      <c r="R34" s="12"/>
+    </row>
+    <row r="35" spans="1:18" s="33" customFormat="1">
+      <c r="A35" s="32"/>
+      <c r="B35" s="8">
+        <f>ROW(B35) - ROW($B$2)</f>
+        <v>33</v>
+      </c>
+      <c r="C35" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="G35" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="I35" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J35" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="K35" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="L35" s="6">
+        <v>1</v>
+      </c>
+      <c r="M35" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N35" s="21" t="s">
+        <v>295</v>
+      </c>
+      <c r="O35" s="34" t="str">
+        <f t="shared" si="20"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P35" s="22" t="s">
+        <v>325</v>
+      </c>
+      <c r="Q35" s="7">
+        <f>P35*N35</f>
+        <v>6.9999999999999993E-2</v>
+      </c>
+      <c r="R35" s="6"/>
+    </row>
+    <row r="36" spans="1:18" s="33" customFormat="1">
+      <c r="A36" s="32"/>
+      <c r="B36" s="9">
+        <f t="shared" si="0"/>
+        <v>34</v>
+      </c>
+      <c r="C36" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="D36" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="E36" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="F36" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="G36" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="H36" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="I36" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J36" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="K36" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="L36" s="12">
+        <v>1</v>
+      </c>
+      <c r="M36" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N36" s="17" t="s">
+        <v>295</v>
+      </c>
+      <c r="O36" s="34" t="str">
+        <f t="shared" si="20"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P36" s="19" t="s">
+        <v>320</v>
+      </c>
+      <c r="Q36" s="13">
+        <f t="shared" ref="Q36" si="24">P36*N36</f>
+        <v>0.06</v>
+      </c>
+      <c r="R36" s="12"/>
+    </row>
+    <row r="37" spans="1:18" s="33" customFormat="1">
+      <c r="A37" s="32"/>
+      <c r="B37" s="8">
+        <f>ROW(B37) - ROW($B$2)</f>
+        <v>35</v>
+      </c>
+      <c r="C37" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="I37" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J37" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="K37" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="L37" s="6">
+        <v>2</v>
+      </c>
+      <c r="M37" s="6">
+        <f t="shared" si="1"/>
+        <v>200</v>
+      </c>
+      <c r="N37" s="21" t="s">
+        <v>347</v>
+      </c>
+      <c r="O37" s="34" t="str">
+        <f t="shared" si="20"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P37" s="22" t="s">
+        <v>320</v>
+      </c>
+      <c r="Q37" s="7">
+        <f>P37*N37</f>
+        <v>0.12</v>
+      </c>
+      <c r="R37" s="6"/>
+    </row>
+    <row r="38" spans="1:18" s="33" customFormat="1">
+      <c r="A38" s="32"/>
+      <c r="B38" s="9">
+        <f t="shared" si="0"/>
+        <v>36</v>
+      </c>
+      <c r="C38" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D38" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="E38" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="F38" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="G38" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="H38" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="I38" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J38" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="K38" s="12" t="s">
+        <v>279</v>
+      </c>
+      <c r="L38" s="12">
+        <v>2</v>
+      </c>
+      <c r="M38" s="6">
+        <f t="shared" si="1"/>
+        <v>200</v>
+      </c>
+      <c r="N38" s="21" t="s">
+        <v>347</v>
+      </c>
+      <c r="O38" s="34" t="str">
+        <f t="shared" si="20"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P38" s="22" t="s">
+        <v>325</v>
+      </c>
+      <c r="Q38" s="13">
+        <f t="shared" ref="Q38" si="25">P38*N38</f>
+        <v>0.13999999999999999</v>
+      </c>
+      <c r="R38" s="12"/>
+    </row>
+    <row r="39" spans="1:18" s="33" customFormat="1">
+      <c r="A39" s="32"/>
+      <c r="B39" s="8">
+        <f>ROW(B39) - ROW($B$2)</f>
+        <v>37</v>
+      </c>
+      <c r="C39" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="G39" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="H39" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="I39" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J39" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="K39" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="L39" s="6">
+        <v>2</v>
+      </c>
+      <c r="M39" s="6">
+        <f t="shared" si="1"/>
+        <v>200</v>
+      </c>
+      <c r="N39" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="O39" s="34" t="s">
+        <v>294</v>
+      </c>
+      <c r="P39" s="7" t="s">
+        <v>370</v>
+      </c>
+      <c r="Q39" s="7">
+        <f>P39*N39</f>
+        <v>0.2</v>
+      </c>
+      <c r="R39" s="6"/>
+    </row>
+    <row r="40" spans="1:18" s="33" customFormat="1">
+      <c r="A40" s="32"/>
+      <c r="B40" s="9">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+      <c r="C40" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="E40" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="F40" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="G40" s="12" t="s">
+        <v>185</v>
+      </c>
+      <c r="H40" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="I40" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J40" s="12" t="s">
+        <v>255</v>
+      </c>
+      <c r="K40" s="12" t="s">
+        <v>281</v>
+      </c>
+      <c r="L40" s="12">
+        <v>1</v>
+      </c>
+      <c r="M40" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N40" s="17" t="s">
+        <v>295</v>
+      </c>
+      <c r="O40" s="34" t="str">
+        <f t="shared" ref="O40:O41" si="26">HYPERLINK(M40, "LCSC")</f>
+        <v>LCSC</v>
+      </c>
+      <c r="P40" s="19" t="s">
+        <v>323</v>
+      </c>
+      <c r="Q40" s="13">
+        <f t="shared" ref="Q40" si="27">P40*N40</f>
+        <v>0.12</v>
+      </c>
+      <c r="R40" s="12"/>
+    </row>
+    <row r="41" spans="1:18" s="33" customFormat="1">
+      <c r="A41" s="32"/>
+      <c r="B41" s="8">
+        <f>ROW(B41) - ROW($B$2)</f>
+        <v>39</v>
+      </c>
+      <c r="C41" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="G41" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="H41" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="I41" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J41" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="K41" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="L41" s="6">
+        <v>1</v>
+      </c>
+      <c r="M41" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N41" s="21" t="s">
+        <v>295</v>
+      </c>
+      <c r="O41" s="34" t="str">
+        <f t="shared" si="26"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P41" s="22" t="s">
+        <v>326</v>
+      </c>
+      <c r="Q41" s="7">
+        <f>P41*N41</f>
+        <v>0.53</v>
+      </c>
+      <c r="R41" s="6"/>
+    </row>
+    <row r="42" spans="1:18" s="33" customFormat="1">
+      <c r="A42" s="32"/>
+      <c r="B42" s="9">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+      <c r="C42" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D42" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="E42" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="F42" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="G42" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="H42" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="I42" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J42" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="K42" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="L42" s="12">
+        <v>2</v>
+      </c>
+      <c r="M42" s="6">
+        <f t="shared" si="1"/>
+        <v>200</v>
+      </c>
+      <c r="N42" s="12" t="s">
+        <v>347</v>
+      </c>
+      <c r="O42" s="34" t="s">
+        <v>294</v>
+      </c>
+      <c r="P42" s="13" t="s">
+        <v>322</v>
+      </c>
+      <c r="Q42" s="13">
+        <f t="shared" ref="Q42" si="28">P42*N42</f>
+        <v>0.22</v>
+      </c>
+      <c r="R42" s="12"/>
+    </row>
+    <row r="43" spans="1:18" s="33" customFormat="1">
+      <c r="A43" s="32"/>
+      <c r="B43" s="8">
+        <f>ROW(B43) - ROW($B$2)</f>
+        <v>41</v>
+      </c>
+      <c r="C43" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="F43" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="G43" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="H43" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="I43" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J43" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="K43" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="L43" s="6">
+        <v>1</v>
+      </c>
+      <c r="M43" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N43" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="O43" s="34" t="s">
+        <v>294</v>
+      </c>
+      <c r="P43" s="7" t="s">
+        <v>323</v>
+      </c>
+      <c r="Q43" s="7">
+        <f>P43*N43</f>
+        <v>0.12</v>
+      </c>
+      <c r="R43" s="6"/>
+    </row>
+    <row r="44" spans="1:18" s="33" customFormat="1">
+      <c r="A44" s="32"/>
+      <c r="B44" s="9">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="C44" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="D44" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="E44" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="F44" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="G44" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="H44" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="I44" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J44" s="12" t="s">
+        <v>259</v>
+      </c>
+      <c r="K44" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="L44" s="12">
+        <v>2</v>
+      </c>
+      <c r="M44" s="6">
+        <f t="shared" si="1"/>
+        <v>200</v>
+      </c>
+      <c r="N44" s="17" t="s">
+        <v>347</v>
+      </c>
+      <c r="O44" s="34" t="str">
+        <f t="shared" ref="O44:O47" si="29">HYPERLINK(M44, "LCSC")</f>
+        <v>LCSC</v>
+      </c>
+      <c r="P44" s="19" t="s">
+        <v>371</v>
+      </c>
+      <c r="Q44" s="13">
+        <f t="shared" ref="Q44" si="30">P44*N44</f>
+        <v>20.68</v>
+      </c>
+      <c r="R44" s="12"/>
+    </row>
+    <row r="45" spans="1:18" s="33" customFormat="1" ht="24">
+      <c r="A45" s="32"/>
+      <c r="B45" s="8">
+        <f>ROW(B45) - ROW($B$2)</f>
+        <v>43</v>
+      </c>
+      <c r="C45" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="E45" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="F45" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="G45" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="H45" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="I45" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J45" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="K45" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="L45" s="6">
+        <v>1</v>
+      </c>
+      <c r="M45" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N45" s="21" t="s">
+        <v>295</v>
+      </c>
+      <c r="O45" s="34" t="str">
+        <f t="shared" si="29"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P45" s="22" t="s">
+        <v>372</v>
+      </c>
+      <c r="Q45" s="7">
+        <f>P45*N45</f>
+        <v>110.80000000000001</v>
+      </c>
+      <c r="R45" s="6"/>
+    </row>
+    <row r="46" spans="1:18" s="33" customFormat="1">
+      <c r="A46" s="32"/>
+      <c r="B46" s="9">
+        <f t="shared" si="0"/>
+        <v>44</v>
+      </c>
+      <c r="C46" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D46" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="E46" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="F46" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="G46" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="H46" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="I46" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J46" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="K46" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="L46" s="12">
+        <v>3</v>
+      </c>
+      <c r="M46" s="6">
+        <f t="shared" si="1"/>
+        <v>300</v>
+      </c>
+      <c r="N46" s="17" t="s">
+        <v>364</v>
+      </c>
+      <c r="O46" s="34" t="str">
+        <f t="shared" si="29"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P46" s="19" t="s">
+        <v>373</v>
+      </c>
+      <c r="Q46" s="13">
+        <f t="shared" ref="Q46" si="31">P46*N46</f>
+        <v>155.88</v>
+      </c>
+      <c r="R46" s="12"/>
+    </row>
+    <row r="47" spans="1:18" s="33" customFormat="1" ht="24">
+      <c r="A47" s="32"/>
+      <c r="B47" s="8">
+        <f>ROW(B47) - ROW($B$2)</f>
+        <v>45</v>
+      </c>
+      <c r="C47" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E47" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="F47" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="G47" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="H47" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="I47" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J47" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="K47" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="L47" s="6">
+        <v>1</v>
+      </c>
+      <c r="M47" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N47" s="21" t="s">
+        <v>295</v>
+      </c>
+      <c r="O47" s="34" t="str">
+        <f t="shared" si="29"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P47" s="22" t="s">
+        <v>374</v>
+      </c>
+      <c r="Q47" s="7">
+        <f>P47*N47</f>
+        <v>370.58</v>
+      </c>
+      <c r="R47" s="6"/>
+    </row>
+    <row r="48" spans="1:18" s="33" customFormat="1" ht="24">
+      <c r="A48" s="32"/>
+      <c r="B48" s="9">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+      <c r="C48" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D48" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="E48" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="F48" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="G48" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H48" s="12" t="s">
+        <v>217</v>
+      </c>
+      <c r="I48" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J48" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="K48" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="L48" s="12">
+        <v>1</v>
+      </c>
+      <c r="M48" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N48" s="12" t="s">
+        <v>295</v>
+      </c>
+      <c r="O48" s="27" t="s">
+        <v>294</v>
+      </c>
+      <c r="P48" s="13" t="s">
+        <v>375</v>
+      </c>
+      <c r="Q48" s="13">
+        <f t="shared" ref="Q48" si="32">P48*N48</f>
+        <v>55.879999999999995</v>
+      </c>
+      <c r="R48" s="12"/>
+    </row>
+    <row r="49" spans="1:18" s="33" customFormat="1" ht="24">
+      <c r="A49" s="32"/>
+      <c r="B49" s="8">
+        <f>ROW(B49) - ROW($B$2)</f>
+        <v>47</v>
+      </c>
+      <c r="C49" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="E49" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="F49" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="G49" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="H49" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="I49" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J49" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="K49" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="L49" s="6">
+        <v>1</v>
+      </c>
+      <c r="M49" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N49" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="O49" s="27" t="s">
+        <v>294</v>
+      </c>
+      <c r="P49" s="7" t="s">
+        <v>376</v>
+      </c>
+      <c r="Q49" s="7">
+        <f>P49*N49</f>
+        <v>52.400000000000006</v>
+      </c>
+      <c r="R49" s="6"/>
+    </row>
+    <row r="50" spans="1:18" s="33" customFormat="1" ht="36">
+      <c r="A50" s="32"/>
+      <c r="B50" s="9">
+        <f t="shared" si="0"/>
+        <v>48</v>
+      </c>
+      <c r="C50" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="D50" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="E50" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="F50" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="G50" s="12" t="s">
+        <v>192</v>
+      </c>
+      <c r="H50" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="I50" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J50" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="K50" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="L50" s="12">
+        <v>1</v>
+      </c>
+      <c r="M50" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N50" s="12" t="s">
+        <v>295</v>
+      </c>
+      <c r="O50" s="27" t="s">
+        <v>294</v>
+      </c>
+      <c r="P50" s="13" t="s">
+        <v>377</v>
+      </c>
+      <c r="Q50" s="13">
+        <f t="shared" ref="Q50" si="33">P50*N50</f>
+        <v>2.97</v>
+      </c>
+      <c r="R50" s="12"/>
+    </row>
+    <row r="51" spans="1:18" s="33" customFormat="1" ht="90.75" thickBot="1">
+      <c r="A51" s="32"/>
+      <c r="B51" s="9">
+        <f t="shared" si="0"/>
+        <v>49</v>
+      </c>
+      <c r="C51" s="15" t="s">
+        <v>333</v>
+      </c>
+      <c r="D51" s="12" t="s">
+        <v>334</v>
+      </c>
+      <c r="E51" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="F51" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="G51" s="12" t="s">
+        <v>332</v>
+      </c>
+      <c r="H51" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="I51" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="J51" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="K51" s="12" t="s">
+        <v>329</v>
+      </c>
+      <c r="L51" s="12">
+        <v>1</v>
+      </c>
+      <c r="M51" s="6">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N51" s="12">
+        <v>5</v>
+      </c>
+      <c r="O51" s="27" t="s">
+        <v>336</v>
+      </c>
+      <c r="P51" s="13"/>
+      <c r="Q51" s="13"/>
+      <c r="R51" s="28" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="52" spans="1:18" ht="19.5" thickBot="1">
+      <c r="A52" s="1"/>
+      <c r="B52" s="1"/>
+      <c r="C52" s="1"/>
+      <c r="D52" s="1"/>
+      <c r="E52" s="1"/>
+      <c r="F52" s="1"/>
+      <c r="G52" s="1"/>
+      <c r="H52" s="1"/>
+      <c r="I52" s="1"/>
+      <c r="J52" s="1"/>
+      <c r="K52" s="1"/>
+      <c r="L52" s="1"/>
+      <c r="M52" s="1"/>
+      <c r="N52" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="O52" s="31"/>
+      <c r="P52" s="31"/>
+      <c r="Q52" s="10">
+        <f>SUM(Q3:Q50)</f>
+        <v>995.84760000000006</v>
+      </c>
+      <c r="R52" s="1"/>
+    </row>
+    <row r="53" spans="1:18" ht="19.5" thickBot="1">
+      <c r="A53" s="1"/>
+      <c r="B53" s="1"/>
+      <c r="C53" s="1"/>
+      <c r="D53" s="1"/>
+      <c r="E53" s="1"/>
+      <c r="F53" s="1"/>
+      <c r="G53" s="1"/>
+      <c r="H53" s="1"/>
+      <c r="I53" s="1"/>
+      <c r="J53" s="1"/>
+      <c r="K53" s="1"/>
+      <c r="L53" s="1"/>
+      <c r="M53" s="1"/>
+      <c r="N53" s="30" t="s">
+        <v>2</v>
+      </c>
+      <c r="O53" s="31"/>
+      <c r="P53" s="31"/>
+      <c r="Q53" s="11">
+        <f>Q52/100</f>
+        <v>9.958476000000001</v>
+      </c>
+      <c r="R53" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="K1:R1"/>
+    <mergeCell ref="N52:P52"/>
+    <mergeCell ref="N53:P53"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="O3" r:id="rId1"/>
+    <hyperlink ref="O8" r:id="rId2"/>
+    <hyperlink ref="O4" r:id="rId3"/>
+    <hyperlink ref="O10" r:id="rId4"/>
+    <hyperlink ref="O13" r:id="rId5"/>
+    <hyperlink ref="O15" r:id="rId6"/>
+    <hyperlink ref="O16" r:id="rId7"/>
+    <hyperlink ref="O23" r:id="rId8"/>
+    <hyperlink ref="O24" r:id="rId9"/>
+    <hyperlink ref="O27" r:id="rId10"/>
+    <hyperlink ref="O28" r:id="rId11"/>
+    <hyperlink ref="O39" r:id="rId12"/>
+    <hyperlink ref="O42" r:id="rId13"/>
+    <hyperlink ref="O43" r:id="rId14"/>
+    <hyperlink ref="O48" r:id="rId15"/>
+    <hyperlink ref="O49" r:id="rId16"/>
+    <hyperlink ref="O50" r:id="rId17"/>
+    <hyperlink ref="O51" r:id="rId18"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>